<commit_message>
Publish 0.28 intro tutorials and reviewed workbook dialogue
</commit_message>
<xml_diff>
--- a/data/source.xlsx
+++ b/data/source.xlsx
@@ -2108,7 +2108,7 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="T_DialogueGroup" displayName="T_DialogueGroup" ref="A1:K74" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="T_DialogueGroup" displayName="T_DialogueGroup" ref="A1:K89" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="GroupID"/>
     <x:tableColumn id="2" name="Name"/>
@@ -2268,7 +2268,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="T_Guide" displayName="T_Guide" ref="A1:C196" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="T_Guide" displayName="T_Guide" ref="A1:C207" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="3">
     <x:tableColumn id="1" name="Group"/>
     <x:tableColumn id="2" name="Topic"/>
@@ -2279,7 +2279,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="T_Dialogue" displayName="T_Dialogue" ref="A1:F114" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="T_Dialogue" displayName="T_Dialogue" ref="A1:F130" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="DialogueID"/>
     <x:tableColumn id="2" name="GroupID"/>
@@ -3423,6 +3423,54 @@
         <v>80073</v>
       </c>
     </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="9">
+        <v>10004</v>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cut</t>
+        </is>
+      </c>
+      <c r="C8" s="9">
+        <v>80074</v>
+      </c>
+      <c r="D8" s="4">
+        <v>80075</v>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="9">
+        <v>10004</v>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">draw</t>
+        </is>
+      </c>
+      <c r="C9" s="9">
+        <v>80076</v>
+      </c>
+      <c r="D9" s="4">
+        <v>80077</v>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="9">
+        <v>10004</v>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">attach</t>
+        </is>
+      </c>
+      <c r="C10" s="9">
+        <v>80078</v>
+      </c>
+      <c r="D10" s="4">
+        <v>80079</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D7"/>
   <dataValidations count="1">
@@ -5982,7 +6030,7 @@
         </x:is>
       </x:c>
       <x:c r="D38" s="5" t="b">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E38" s="4" t="inlineStr">
         <x:is>
@@ -6443,7 +6491,7 @@
       </x:c>
       <x:c r="B48" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">샌즈 · 세 번째 MISS 식은땀</x:t>
+          <x:t xml:space="preserve">샌즈 · 마지막 빈틈 경계</x:t>
         </x:is>
       </x:c>
       <x:c r="C48" s="4" t="inlineStr">
@@ -6460,17 +6508,17 @@
         </x:is>
       </x:c>
       <x:c r="F48" s="10">
-        <x:v>23</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="G48" s="9">
-        <x:v>1500</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="H48" s="9">
         <x:v>250</x:v>
       </x:c>
       <x:c r="I48" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">첫 MISS와 함께 재생. 말하는 중에도 빈틈 게이지와 연타 진행.</x:t>
+          <x:t xml:space="preserve">세 번째 페이즈 빈틈 시작, 공격과 함께 말한다.</x:t>
         </x:is>
       </x:c>
       <x:c r="J48" s="4" t="inlineStr">
@@ -7379,11 +7427,11 @@
     </x:row>
     <x:row r="68" ht="18" customHeight="1">
       <x:c r="A68" s="9">
-        <x:v>80067</x:v>
+        <x:v>80068</x:v>
       </x:c>
       <x:c r="B68" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">샌즈 · 야차가 끝난 미용실</x:t>
+          <x:t xml:space="preserve">취준좀비 · 색·무늬 꾸미기 · 자세한 부탁</x:t>
         </x:is>
       </x:c>
       <x:c r="C68" s="4" t="inlineStr">
@@ -7410,7 +7458,7 @@
       </x:c>
       <x:c r="I68" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">통합 프로토타입 미용실 대사</x:t>
+          <x:t xml:space="preserve">미용 대사 연결에서 선택하는 부탁</x:t>
         </x:is>
       </x:c>
       <x:c r="J68" s="4" t="inlineStr">
@@ -7426,11 +7474,11 @@
     </x:row>
     <x:row r="69" ht="18" customHeight="1">
       <x:c r="A69" s="9">
-        <x:v>80068</x:v>
+        <x:v>80069</x:v>
       </x:c>
       <x:c r="B69" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">취준좀비 · 색·무늬 꾸미기 · 자세한 부탁</x:t>
+          <x:t xml:space="preserve">취준좀비 · 장식 붙이기 · 자세한 부탁</x:t>
         </x:is>
       </x:c>
       <x:c r="C69" s="4" t="inlineStr">
@@ -7473,11 +7521,11 @@
     </x:row>
     <x:row r="70" ht="18" customHeight="1">
       <x:c r="A70" s="9">
-        <x:v>80069</x:v>
+        <x:v>80070</x:v>
       </x:c>
       <x:c r="B70" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">취준좀비 · 장식 붙이기 · 자세한 부탁</x:t>
+          <x:t xml:space="preserve">샌즈 · 형태 만들기 · 자세한 부탁</x:t>
         </x:is>
       </x:c>
       <x:c r="C70" s="4" t="inlineStr">
@@ -7520,11 +7568,11 @@
     </x:row>
     <x:row r="71" ht="18" customHeight="1">
       <x:c r="A71" s="9">
-        <x:v>80070</x:v>
+        <x:v>80071</x:v>
       </x:c>
       <x:c r="B71" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">샌즈 · 형태 만들기 · 자세한 부탁</x:t>
+          <x:t xml:space="preserve">샌즈 · 색·무늬 꾸미기 · 처음 부탁</x:t>
         </x:is>
       </x:c>
       <x:c r="C71" s="4" t="inlineStr">
@@ -7567,11 +7615,11 @@
     </x:row>
     <x:row r="72" ht="18" customHeight="1">
       <x:c r="A72" s="9">
-        <x:v>80071</x:v>
+        <x:v>80072</x:v>
       </x:c>
       <x:c r="B72" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">샌즈 · 색·무늬 꾸미기 · 처음 부탁</x:t>
+          <x:t xml:space="preserve">샌즈 · 색·무늬 꾸미기 · 자세한 부탁</x:t>
         </x:is>
       </x:c>
       <x:c r="C72" s="4" t="inlineStr">
@@ -7614,11 +7662,11 @@
     </x:row>
     <x:row r="73" ht="18" customHeight="1">
       <x:c r="A73" s="9">
-        <x:v>80072</x:v>
+        <x:v>80073</x:v>
       </x:c>
       <x:c r="B73" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">샌즈 · 색·무늬 꾸미기 · 자세한 부탁</x:t>
+          <x:t xml:space="preserve">샌즈 · 장식 붙이기 · 자세한 부탁</x:t>
         </x:is>
       </x:c>
       <x:c r="C73" s="4" t="inlineStr">
@@ -7661,11 +7709,11 @@
     </x:row>
     <x:row r="74" ht="18" customHeight="1">
       <x:c r="A74" s="9">
-        <x:v>80073</x:v>
+        <x:v>80089</x:v>
       </x:c>
       <x:c r="B74" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">샌즈 · 장식 붙이기 · 자세한 부탁</x:t>
+          <x:t xml:space="preserve">샌즈 · 야차 승리 후 미용실</x:t>
         </x:is>
       </x:c>
       <x:c r="C74" s="4" t="inlineStr">
@@ -7692,7 +7740,7 @@
       </x:c>
       <x:c r="I74" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">미용 대사 연결에서 선택하는 부탁</x:t>
+          <x:t xml:space="preserve">통합 개발실</x:t>
         </x:is>
       </x:c>
       <x:c r="J74" s="4" t="inlineStr">
@@ -7706,8 +7754,713 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="75" ht="18" customHeight="1">
+      <x:c r="A75" s="9">
+        <x:v>80074</x:v>
+      </x:c>
+      <x:c r="B75" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">마왕 부하 · 형태 다듬기 · 처음 부탁</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C75" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">순서대로</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D75" s="5" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E75" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">입력</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F75" s="10">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="G75" s="9">
+        <x:v>1400</x:v>
+      </x:c>
+      <x:c r="H75" s="9">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="I75" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미용 시험용 대사 초안</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J75" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">없음</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K75" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">없음</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="76" ht="18" customHeight="1">
+      <x:c r="A76" s="9">
+        <x:v>80075</x:v>
+      </x:c>
+      <x:c r="B76" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">마왕 부하 · 형태 다듬기 · 자세한 부탁</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C76" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">순서대로</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D76" s="5" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E76" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">입력</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F76" s="10">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="G76" s="9">
+        <x:v>1400</x:v>
+      </x:c>
+      <x:c r="H76" s="9">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="I76" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미용 시험용 대사 초안</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J76" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">없음</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K76" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">없음</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="18" customHeight="1">
+      <x:c r="A77" s="9">
+        <x:v>80076</x:v>
+      </x:c>
+      <x:c r="B77" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">마왕 부하 · 색·무늬 · 처음 부탁</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C77" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">순서대로</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D77" s="5" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E77" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">입력</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F77" s="10">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="G77" s="9">
+        <x:v>1400</x:v>
+      </x:c>
+      <x:c r="H77" s="9">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="I77" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미용 시험용 대사 초안</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J77" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">없음</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K77" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">없음</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="78" ht="18" customHeight="1">
+      <x:c r="A78" s="9">
+        <x:v>80077</x:v>
+      </x:c>
+      <x:c r="B78" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">마왕 부하 · 색·무늬 · 자세한 부탁</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C78" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">순서대로</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D78" s="5" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E78" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">입력</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F78" s="10">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="G78" s="9">
+        <x:v>1400</x:v>
+      </x:c>
+      <x:c r="H78" s="9">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="I78" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미용 시험용 대사 초안</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J78" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">없음</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K78" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">없음</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="79" ht="18" customHeight="1">
+      <x:c r="A79" s="9">
+        <x:v>80078</x:v>
+      </x:c>
+      <x:c r="B79" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">마왕 부하 · 장식 · 처음 부탁</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C79" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">순서대로</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D79" s="5" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E79" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">입력</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F79" s="10">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="G79" s="9">
+        <x:v>1400</x:v>
+      </x:c>
+      <x:c r="H79" s="9">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="I79" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미용 시험용 대사 초안</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J79" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">없음</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K79" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">없음</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="18" customHeight="1">
+      <x:c r="A80" s="9">
+        <x:v>80079</x:v>
+      </x:c>
+      <x:c r="B80" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">마왕 부하 · 장식 · 자세한 부탁</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C80" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">순서대로</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D80" s="5" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E80" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">입력</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F80" s="10">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="G80" s="9">
+        <x:v>1400</x:v>
+      </x:c>
+      <x:c r="H80" s="9">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="I80" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미용 시험용 대사 초안</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J80" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">없음</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K80" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">없음</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="18" customHeight="1">
+      <x:c r="A81" s="9">
+        <x:v>80080</x:v>
+      </x:c>
+      <x:c r="B81" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">마왕 부하 · 손님 등장</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C81" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">순서대로</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D81" s="5" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E81" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">입력</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F81" s="10">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="G81" s="9">
+        <x:v>1400</x:v>
+      </x:c>
+      <x:c r="H81" s="9">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="I81" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">로컬 본편 시연용 임시 대사</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J81" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">없음</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K81" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">없음</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="18" customHeight="1">
+      <x:c r="A82" s="9">
+        <x:v>80081</x:v>
+      </x:c>
+      <x:c r="B82" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">마왕 부하 · 미용 만족</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C82" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">순서대로</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D82" s="5" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E82" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">입력</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F82" s="10">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="G82" s="9">
+        <x:v>1400</x:v>
+      </x:c>
+      <x:c r="H82" s="9">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="I82" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">로컬 본편 시연용 임시 대사</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J82" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">없음</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K82" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">없음</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="83" ht="18" customHeight="1">
+      <x:c r="A83" s="9">
+        <x:v>80082</x:v>
+      </x:c>
+      <x:c r="B83" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">마왕 부하 · 미용 보통</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C83" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">순서대로</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D83" s="5" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E83" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">입력</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F83" s="10">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="G83" s="9">
+        <x:v>1400</x:v>
+      </x:c>
+      <x:c r="H83" s="9">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="I83" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">로컬 본편 시연용 임시 대사</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J83" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">없음</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K83" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">없음</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="84" ht="18" customHeight="1">
+      <x:c r="A84" s="9">
+        <x:v>80083</x:v>
+      </x:c>
+      <x:c r="B84" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">마왕 부하 · 미용 불만족</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C84" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">순서대로</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D84" s="5" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E84" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">입력</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F84" s="10">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="G84" s="9">
+        <x:v>1400</x:v>
+      </x:c>
+      <x:c r="H84" s="9">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="I84" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">로컬 본편 시연용 임시 대사</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J84" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">없음</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K84" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">없음</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="85" ht="18" customHeight="1">
+      <x:c r="A85" s="9">
+        <x:v>80084</x:v>
+      </x:c>
+      <x:c r="B85" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">마왕 부하 · 손님 퇴장</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C85" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">순서대로</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D85" s="5" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E85" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">입력</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F85" s="10">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="G85" s="9">
+        <x:v>1400</x:v>
+      </x:c>
+      <x:c r="H85" s="9">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="I85" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">로컬 본편 시연용 임시 대사</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J85" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">없음</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K85" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">없음</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="86" ht="18" customHeight="1">
+      <x:c r="A86" s="9">
+        <x:v>80085</x:v>
+      </x:c>
+      <x:c r="B86" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">마왕 부하 · 눈에 닿았을 때 · 첫 항의</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C86" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">순서대로</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D86" s="5" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E86" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">자동</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F86" s="10">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="G86" s="9">
+        <x:v>5500</x:v>
+      </x:c>
+      <x:c r="H86" s="9">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="I86" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미용 중 반응 · 조건과 재생 시점은 미용 설정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J86" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">없음</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K86" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">없음</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="87" ht="18" customHeight="1">
+      <x:c r="A87" s="9">
+        <x:v>80086</x:v>
+      </x:c>
+      <x:c r="B87" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">마왕 부하 · 다시 눈에 닿았을 때 · 두 번째 항의</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C87" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">순서대로</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D87" s="5" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E87" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">자동</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F87" s="10">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="G87" s="9">
+        <x:v>5500</x:v>
+      </x:c>
+      <x:c r="H87" s="9">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="I87" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미용 중 반응 · 조건과 재생 시점은 미용 설정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J87" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">없음</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K87" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">없음</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="18" customHeight="1">
+      <x:c r="A88" s="9">
+        <x:v>80087</x:v>
+      </x:c>
+      <x:c r="B88" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">마왕 부하 · 뿔을 줄인 뒤 다시 불어날 때</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C88" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">순서대로</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D88" s="5" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E88" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">자동</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F88" s="10">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="G88" s="9">
+        <x:v>5500</x:v>
+      </x:c>
+      <x:c r="H88" s="9">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="I88" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미용 중 반응 · 조건과 재생 시점은 미용 설정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J88" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">없음</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K88" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">없음</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="18" customHeight="1">
+      <x:c r="A89" s="9">
+        <x:v>80088</x:v>
+      </x:c>
+      <x:c r="B89" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">마왕 부하 · 처음보다 뿔이 더 많아졌을 때</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C89" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">순서대로</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D89" s="5" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E89" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">자동</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F89" s="10">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="G89" s="9">
+        <x:v>5500</x:v>
+      </x:c>
+      <x:c r="H89" s="9">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="I89" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">미용 중 반응 · 조건과 재생 시점은 미용 설정</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J89" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">없음</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K89" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">없음</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="A2:K74">
+  <x:conditionalFormatting sqref="A2:K89">
     <x:cfRule type="expression" dxfId="18" priority="1">
       <x:formula>MOD(ROW(),2)=0</x:formula>
     </x:cfRule>
@@ -14902,56 +15655,243 @@
     <x:row r="194" ht="36" customHeight="1">
       <x:c r="A194" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">보류한 원본 데이터</x:t>
+          <x:t xml:space="preserve">작업 안내 / 마왕 부하 대사</x:t>
         </x:is>
       </x:c>
       <x:c r="B194" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MonsterPhase 10100/1</x:t>
+          <x:t xml:space="preserve">엑셀 편집과 실행 범위</x:t>
         </x:is>
       </x:c>
       <x:c r="C194" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MonsterID=10100; Name=마왕; PhaseID=1; IsInitial=켜기; MaxHP=(빈칸); GaugeMax=(빈칸); ParryGain=(빈칸); GuardGain=(빈칸); DodgeGain=(빈칸); RecoveryMs=(빈칸); AttackSpeed=(빈칸); TransitionTrigger=미정; NextPhaseID=2; PlayerDodgeMissCount=0; EntryDialogueGroupID=(빈칸); PauseForEntryDialogue=켜기; DesignStatus=전환 조건·HP·패턴 미정; OpeningDamageDisplay=(빈칸)</x:t>
+          <x:t xml:space="preserve">MonsterID 10004 마왕 부하의 등장·미용 부탁·상세 부탁·결과·퇴장·항의 문장은 대사/대화 그룹에서 편집합니다. 미용 부탁은 미용 대사 연결 cut/draw/attach에서 연결합니다. 미용 조건과 등장·결과·항의 사건 연결은 통합 프로젝트 JSON에 보관하며 실제 Unity 연결은 별도입니다. 미완성 야차 페이즈는 추가하지 않았습니다.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="195" ht="40" customHeight="1">
       <x:c r="A195" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">보류한 원본 데이터</x:t>
+          <x:t xml:space="preserve">작업 안내 / 마왕 부하 대사</x:t>
         </x:is>
       </x:c>
       <x:c r="B195" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MonsterPhase 10100/2</x:t>
+          <x:t xml:space="preserve">arrival → 80080</x:t>
         </x:is>
       </x:c>
       <x:c r="C195" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MonsterID=10100; Name=마왕; PhaseID=2; IsInitial=끄기; MaxHP=(빈칸); GaugeMax=(빈칸); ParryGain=(빈칸); GuardGain=(빈칸); DodgeGain=(빈칸); RecoveryMs=(빈칸); AttackSpeed=(빈칸); TransitionTrigger=미정; NextPhaseID=3; PlayerDodgeMissCount=0; EntryDialogueGroupID=(빈칸); PauseForEntryDialogue=켜기; DesignStatus=전환 조건·HP·패턴 미정; OpeningDamageDisplay=(빈칸)</x:t>
+          <x:t xml:space="preserve">마왕 부하 · 손님 등장</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="196" ht="36" customHeight="1">
       <x:c r="A196" s="11" t="inlineStr">
         <x:is>
+          <x:t xml:space="preserve">작업 안내 / 마왕 부하 대사</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B196" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">best → 80081</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C196" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">마왕 부하 · 미용 만족</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="197" ht="40" customHeight="1">
+      <x:c r="A197" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">작업 안내 / 마왕 부하 대사</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B197" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">normal → 80082</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C197" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">마왕 부하 · 미용 보통</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="198" ht="36" customHeight="1">
+      <x:c r="A198" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">작업 안내 / 마왕 부하 대사</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B198" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">fail → 80083</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C198" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">마왕 부하 · 미용 불만족</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="199" ht="40" customHeight="1">
+      <x:c r="A199" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">작업 안내 / 마왕 부하 대사</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B199" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">leave → 80084</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C199" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">마왕 부하 · 손님 퇴장</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="200" ht="36" customHeight="1">
+      <x:c r="A200" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">작업 안내 / 마왕 부하 대사</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B200" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">eyeContactLine → 80085</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C200" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">마왕 부하 · 눈에 닿았을 때 · 첫 항의</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="201" ht="40" customHeight="1">
+      <x:c r="A201" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">작업 안내 / 마왕 부하 대사</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B201" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">eyeContactSecondLine → 80086</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C201" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">마왕 부하 · 다시 눈에 닿았을 때 · 두 번째 항의</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="202" ht="36" customHeight="1">
+      <x:c r="A202" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">작업 안내 / 마왕 부하 대사</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B202" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">areaWarningLine → 80087</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C202" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">마왕 부하 · 뿔을 줄인 뒤 다시 불어날 때</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="203" ht="40" customHeight="1">
+      <x:c r="A203" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">작업 안내 / 마왕 부하 대사</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B203" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">areaOverflowLine → 80088</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C203" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">마왕 부하 · 처음보다 뿔이 더 많아졌을 때</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="204" ht="36" customHeight="1">
+      <x:c r="A204" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">작업 안내 / 대사 담당자 검토</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B204" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">담당자 검토본과 마왕 부하 통합</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C204" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-16 저장된 시현님 검토본의 대사·대화 그룹·미용 대사 연결을 반영하고 기존 마왕 부하 대사를 유지했습니다. 겹치는 담당자 추가 그룹80085는80089, 문장900133~900136은900140~900143으로 분리했습니다. 샌즈 야차 승리 후 미용실 대사는 프로젝트의 afterWin에 그룹80089로 연결합니다. 문장 내용·순서는 담당자 검토본을 따릅니다.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="205" ht="40" customHeight="1">
+      <x:c r="A205" s="11" t="inlineStr">
+        <x:is>
           <x:t xml:space="preserve">보류한 원본 데이터</x:t>
         </x:is>
       </x:c>
-      <x:c r="B196" s="11" t="inlineStr">
+      <x:c r="B205" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MonsterPhase 10100/1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C205" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MonsterID=10100; Name=마왕; PhaseID=1; IsInitial=켜기; MaxHP=(빈칸); GaugeMax=(빈칸); ParryGain=(빈칸); GuardGain=(빈칸); DodgeGain=(빈칸); RecoveryMs=(빈칸); AttackSpeed=(빈칸); TransitionTrigger=미정; NextPhaseID=2; PlayerDodgeMissCount=0; EntryDialogueGroupID=(빈칸); PauseForEntryDialogue=켜기; DesignStatus=전환 조건·HP·패턴 미정; OpeningDamageDisplay=(빈칸)</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="206" ht="36" customHeight="1">
+      <x:c r="A206" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">보류한 원본 데이터</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B206" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MonsterPhase 10100/2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C206" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MonsterID=10100; Name=마왕; PhaseID=2; IsInitial=끄기; MaxHP=(빈칸); GaugeMax=(빈칸); ParryGain=(빈칸); GuardGain=(빈칸); DodgeGain=(빈칸); RecoveryMs=(빈칸); AttackSpeed=(빈칸); TransitionTrigger=미정; NextPhaseID=3; PlayerDodgeMissCount=0; EntryDialogueGroupID=(빈칸); PauseForEntryDialogue=켜기; DesignStatus=전환 조건·HP·패턴 미정; OpeningDamageDisplay=(빈칸)</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="207" ht="40" customHeight="1">
+      <x:c r="A207" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">보류한 원본 데이터</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B207" s="11" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">MonsterPhase 10100/3</x:t>
         </x:is>
       </x:c>
-      <x:c r="C196" s="11" t="inlineStr">
+      <x:c r="C207" s="11" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">MonsterID=10100; Name=마왕; PhaseID=3; IsInitial=끄기; MaxHP=(빈칸); GaugeMax=(빈칸); ParryGain=(빈칸); GuardGain=(빈칸); DodgeGain=(빈칸); RecoveryMs=(빈칸); AttackSpeed=(빈칸); TransitionTrigger=없음; NextPhaseID=(빈칸); PlayerDodgeMissCount=0; EntryDialogueGroupID=(빈칸); PauseForEntryDialogue=켜기; DesignStatus=전환 조건·HP·패턴 미정; OpeningDamageDisplay=(빈칸)</x:t>
         </x:is>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="A2:C196">
+  <x:conditionalFormatting sqref="A2:C207">
     <x:cfRule type="expression" dxfId="14" priority="1">
       <x:formula>MOD(ROW(),2)=0</x:formula>
     </x:cfRule>
@@ -15001,7 +15941,7 @@
     </x:row>
     <x:row r="2" ht="48" customHeight="1">
       <x:c r="A2" s="9">
-        <x:v>900002</x:v>
+        <x:v>900005</x:v>
       </x:c>
       <x:c r="B2" s="9">
         <x:v>80001</x:v>
@@ -15016,7 +15956,7 @@
       </x:c>
       <x:c r="E2" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">으어어...안녕하십니까...지원자 11번...아, 미용실이지...</x:t>
+          <x:t xml:space="preserve">&lt;wave=1&gt;으어... &lt;wait=0.35&gt;내, &lt;wait=0.25&gt;내일 언데드 보험회사?&lt;wait=0.25&gt; 면접이 있거든요...&lt;/wave&gt;</x:t>
         </x:is>
       </x:c>
       <x:c r="F2" s="11" t="inlineStr">
@@ -15027,13 +15967,13 @@
     </x:row>
     <x:row r="3" ht="48" customHeight="1">
       <x:c r="A3" s="9">
-        <x:v>900003</x:v>
+        <x:v>900006</x:v>
       </x:c>
       <x:c r="B3" s="9">
         <x:v>80001</x:v>
       </x:c>
       <x:c r="C3" s="9">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D3" s="4" t="inlineStr">
         <x:is>
@@ -15042,7 +15982,7 @@
       </x:c>
       <x:c r="E3" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">얏호―! 어서오세요. 그런데 거긴 거울이에요. 저는 옆에 있는데요?</x:t>
+          <x:t xml:space="preserve">언데드가 보험? &lt;pulse=1.15&gt;이미 죽었는데 보험이 필요 있나?&lt;/pulse&gt;</x:t>
         </x:is>
       </x:c>
       <x:c r="F3" s="11" t="inlineStr">
@@ -15053,13 +15993,13 @@
     </x:row>
     <x:row r="4" ht="48" customHeight="1">
       <x:c r="A4" s="9">
-        <x:v>900004</x:v>
+        <x:v>900007</x:v>
       </x:c>
       <x:c r="B4" s="9">
         <x:v>80001</x:v>
       </x:c>
       <x:c r="C4" s="9">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D4" s="4" t="inlineStr">
         <x:is>
@@ -15068,7 +16008,7 @@
       </x:c>
       <x:c r="E4" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">아… 어쩐지… 같이 인사를 해주시더라니...</x:t>
+          <x:t xml:space="preserve">&lt;wave=1&gt;어, 어허!&lt;wait=0.25&gt; 그건&lt;/wave&gt; &lt;shake=1&gt;종족차별,&lt;wait=0.25&gt; 발언&lt;/shake&gt;&lt;wave=1&gt;입니다...!&lt;/wave&gt;</x:t>
         </x:is>
       </x:c>
       <x:c r="F4" s="11" t="inlineStr">
@@ -15079,22 +16019,22 @@
     </x:row>
     <x:row r="5" ht="48" customHeight="1">
       <x:c r="A5" s="9">
-        <x:v>900005</x:v>
+        <x:v>900008</x:v>
       </x:c>
       <x:c r="B5" s="9">
         <x:v>80001</x:v>
       </x:c>
       <x:c r="C5" s="9">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D5" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">몬스터</x:t>
+          <x:t xml:space="preserve">플레이어</x:t>
         </x:is>
       </x:c>
       <x:c r="E5" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">아무튼… 내일 좀비 보험회사 면접이 있어서요… 죽고 나서 처음 잡힌 면접이에요…</x:t>
+          <x:t xml:space="preserve">알았다구요~ 원하는 스타일은 있나요?</x:t>
         </x:is>
       </x:c>
       <x:c r="F5" s="11" t="inlineStr">
@@ -15105,39 +16045,40 @@
     </x:row>
     <x:row r="6" ht="48" customHeight="1">
       <x:c r="A6" s="9">
-        <x:v>900006</x:v>
+        <x:v>900014</x:v>
       </x:c>
       <x:c r="B6" s="9">
-        <x:v>80001</x:v>
+        <x:v>80002</x:v>
       </x:c>
       <x:c r="C6" s="9">
-        <x:v>5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D6" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">플레이어</x:t>
+          <x:t xml:space="preserve">몬스터</x:t>
         </x:is>
       </x:c>
       <x:c r="E6" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">보험이요...? 좀비는 보험이 필요없지 않나?</x:t>
+          <x:t xml:space="preserve">으어어... 내,&lt;wait=0.25&gt; 내일 면접이니까... &lt;color=#266B4D&gt;앞이 좀 환해지고&lt;/color&gt;,&lt;wait=0.25&gt;
+&lt;color=#9A4935&gt;미, &lt;wait=0.25&gt;민망한 곳은 안 보였으면&lt;/color&gt; 좋겠어요...</x:t>
         </x:is>
       </x:c>
       <x:c r="F6" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">기존 좀비 원문</x:t>
+          <x:t xml:space="preserve">미용 요구 · 선택지 연결</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="7" ht="48" customHeight="1">
       <x:c r="A7" s="9">
-        <x:v>900007</x:v>
+        <x:v>900015</x:v>
       </x:c>
       <x:c r="B7" s="9">
-        <x:v>80001</x:v>
+        <x:v>80003</x:v>
       </x:c>
       <x:c r="C7" s="9">
-        <x:v>6</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D7" s="4" t="inlineStr">
         <x:is>
@@ -15146,33 +16087,34 @@
       </x:c>
       <x:c r="E7" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">어허, 그거 종족차별 발언입니다...! 요새 그런 말 하면... 큰일나요...</x:t>
+          <x:t xml:space="preserve">아, &lt;wait=0.25&gt;앞머리를 좀,&lt;wait=0.25&gt; 잘라서&lt;wait=0.25&gt; &lt;color=#266B4D&gt;두 눈이 잘 보이게&lt;/color&gt;,&lt;wait=0.25&gt; 좀 해 주세요...
+&lt;color=#9A4935&gt;뇌,&lt;wait=0.25&gt; 뇌가 좀 튀어나와서...&lt;wait=0.35&gt; 머리카락으로 가려&lt;/color&gt; 주시고요...&lt;wait=0.35&gt; &lt;wave=1.2&gt;부,&lt;wait=0.25&gt; 부탁드립니다,&lt;wait=0.25&gt; 으어...&lt;/wave&gt;</x:t>
         </x:is>
       </x:c>
       <x:c r="F7" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">기존 좀비 원문</x:t>
+          <x:t xml:space="preserve">미용 요구 · 선택지 연결</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="8" ht="48" customHeight="1">
       <x:c r="A8" s="9">
-        <x:v>900008</x:v>
+        <x:v>900016</x:v>
       </x:c>
       <x:c r="B8" s="9">
-        <x:v>80001</x:v>
+        <x:v>80004</x:v>
       </x:c>
       <x:c r="C8" s="9">
-        <x:v>7</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D8" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">플레이어</x:t>
+          <x:t xml:space="preserve">몬스터</x:t>
         </x:is>
       </x:c>
       <x:c r="E8" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">(별 귀찮은 것도 다 있네~) 알았다구요~ 원하는 스타일은 있나요?</x:t>
+          <x:t xml:space="preserve">아니, 앞이 안 보인다고요! 당장 '가위'를 들어서 내 눈을 가리는 앞머리를 싹 다 잘라달란 말입니다!</x:t>
         </x:is>
       </x:c>
       <x:c r="F8" s="11" t="inlineStr">
@@ -15183,13 +16125,13 @@
     </x:row>
     <x:row r="9" ht="48" customHeight="1">
       <x:c r="A9" s="9">
-        <x:v>900009</x:v>
+        <x:v>900017</x:v>
       </x:c>
       <x:c r="B9" s="9">
-        <x:v>80001</x:v>
+        <x:v>80005</x:v>
       </x:c>
       <x:c r="C9" s="9">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D9" s="4" t="inlineStr">
         <x:is>
@@ -15198,7 +16140,7 @@
       </x:c>
       <x:c r="E9" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">지난번엔 면접관님 눈을 보고 대답하라길래… 한참 열심히 했거든요…</x:t>
+          <x:t xml:space="preserve">으어어…&lt;wait=0.35&gt; 제 눈을 직접 본 건...&lt;wait=0.35&gt; 죽은 뒤로 처음이에요,&lt;wait=0.25&gt; 으어...</x:t>
         </x:is>
       </x:c>
       <x:c r="F9" s="11" t="inlineStr">
@@ -15209,22 +16151,22 @@
     </x:row>
     <x:row r="10" ht="48" customHeight="1">
       <x:c r="A10" s="9">
-        <x:v>900010</x:v>
+        <x:v>900018</x:v>
       </x:c>
       <x:c r="B10" s="9">
-        <x:v>80001</x:v>
+        <x:v>80006</x:v>
       </x:c>
       <x:c r="C10" s="9">
-        <x:v>9</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D10" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">플레이어</x:t>
+          <x:t xml:space="preserve">몬스터</x:t>
         </x:is>
       </x:c>
       <x:c r="E10" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">그런데요?</x:t>
+          <x:t xml:space="preserve">으어어…&lt;wait=0.35&gt; 이, &lt;wait=0.25&gt;일단 앞은 보이네요… &lt;wait=0.35&gt;이 정도면 면접관님은 보이겠어요...&lt;wait=0.35&gt;</x:t>
         </x:is>
       </x:c>
       <x:c r="F10" s="11" t="inlineStr">
@@ -15235,13 +16177,13 @@
     </x:row>
     <x:row r="11" ht="48" customHeight="1">
       <x:c r="A11" s="9">
-        <x:v>900011</x:v>
+        <x:v>900019</x:v>
       </x:c>
       <x:c r="B11" s="9">
-        <x:v>80001</x:v>
+        <x:v>80007</x:v>
       </x:c>
       <x:c r="C11" s="9">
-        <x:v>10</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D11" s="4" t="inlineStr">
         <x:is>
@@ -15250,7 +16192,7 @@
       </x:c>
       <x:c r="E11" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">면접관님은 옆에 계셨대요… 저는 공기청정기한테… 입사 포부를…</x:t>
+          <x:t xml:space="preserve">&lt;shake=1.4&gt;으어... &lt;wait=0.35&gt;으어?&lt;wait=0.35&gt; 으어어어어!!!!!&lt;/shake&gt;</x:t>
         </x:is>
       </x:c>
       <x:c r="F11" s="11" t="inlineStr">
@@ -15261,22 +16203,22 @@
     </x:row>
     <x:row r="12" ht="48" customHeight="1">
       <x:c r="A12" s="9">
-        <x:v>900012</x:v>
+        <x:v>900020</x:v>
       </x:c>
       <x:c r="B12" s="9">
-        <x:v>80001</x:v>
+        <x:v>80008</x:v>
       </x:c>
       <x:c r="C12" s="9">
-        <x:v>11</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D12" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">플레이어</x:t>
+          <x:t xml:space="preserve">몬스터</x:t>
         </x:is>
       </x:c>
       <x:c r="E12" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">O.K~ 이해 완료! 앞이 보이게 해 드리면 되는 거죠?</x:t>
+          <x:t xml:space="preserve">머,&lt;wait=0.25&gt; 머리도 잘 됐는데... &lt;wait=0.35&gt;하,&lt;wait=0.25&gt; 한 번 기세를, &lt;wait=0.25&gt;제 기세를 시험해 주시겠습니까...?&lt;wait=0.35&gt; 으어,&lt;wait=0.25&gt; 면접 때 잘 싸울 수,&lt;wait=0.25&gt; 아,&lt;wait=0.25&gt; 아니 말할 수 있는지......</x:t>
         </x:is>
       </x:c>
       <x:c r="F12" s="11" t="inlineStr">
@@ -15287,13 +16229,13 @@
     </x:row>
     <x:row r="13" ht="48" customHeight="1">
       <x:c r="A13" s="9">
-        <x:v>900013</x:v>
+        <x:v>900021</x:v>
       </x:c>
       <x:c r="B13" s="9">
-        <x:v>80001</x:v>
+        <x:v>80008</x:v>
       </x:c>
       <x:c r="C13" s="9">
-        <x:v>12</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D13" s="4" t="inlineStr">
         <x:is>
@@ -15302,7 +16244,7 @@
       </x:c>
       <x:c r="E13" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">부탁드려요… 이번엔 정말… 산 사람처럼 살고 싶어서요…</x:t>
+          <x:t xml:space="preserve">그, &lt;wait=0.25&gt;그니까 이게,&lt;wait=0.25&gt; 여,&lt;wait=0.25&gt; 연습 야차 상대를...&lt;wait=0.35&gt; 부탁드린다고요... &lt;wait=0.35&gt;이기면 호, &lt;wait=0.25&gt;홍보라도 해 드릴게요...&lt;wait=0.35&gt; 으어...</x:t>
         </x:is>
       </x:c>
       <x:c r="F13" s="11" t="inlineStr">
@@ -15313,10 +16255,10 @@
     </x:row>
     <x:row r="14" ht="48" customHeight="1">
       <x:c r="A14" s="9">
-        <x:v>900014</x:v>
+        <x:v>900022</x:v>
       </x:c>
       <x:c r="B14" s="9">
-        <x:v>80002</x:v>
+        <x:v>80009</x:v>
       </x:c>
       <x:c r="C14" s="9">
         <x:v>1</x:v>
@@ -15328,25 +16270,24 @@
       </x:c>
       <x:c r="E14" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">으어어... 내일 면접인데... &lt;color=#266B4D&gt;앞이 좀 환해지고&lt;/color&gt;,
-&lt;color=#9A4935&gt;민망한 곳은 안 보였으면&lt;/color&gt; 좋겠어요...</x:t>
+          <x:t xml:space="preserve">머리도 됐으니... 제 기세를 한 번 시험해 주시겠어요? 면접 때 자신있게 싸울... 아니 말할 수 있는지 봐주시면 됩니다.</x:t>
         </x:is>
       </x:c>
       <x:c r="F14" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">미용 요구 · 선택지 연결</x:t>
+          <x:t xml:space="preserve">기존 좀비 원문</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="15" ht="48" customHeight="1">
       <x:c r="A15" s="9">
-        <x:v>900015</x:v>
+        <x:v>900023</x:v>
       </x:c>
       <x:c r="B15" s="9">
-        <x:v>80003</x:v>
+        <x:v>80009</x:v>
       </x:c>
       <x:c r="C15" s="9">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D15" s="4" t="inlineStr">
         <x:is>
@@ -15355,22 +16296,21 @@
       </x:c>
       <x:c r="E15" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">&lt;color=#266B4D&gt;두 눈이 잘 보이게&lt;/color&gt; 앞머리를 잘라 주세요...
-아, &lt;color=#9A4935&gt;튀어나온 뇌는 머리카락으로 가려&lt;/color&gt; 주시고요... &lt;wave=1.2&gt;부탁드립니다...&lt;/wave&gt;</x:t>
+          <x:t xml:space="preserve">연습 야차 상대를... 부탁드린다는 뜻입니다...저를 이기시면... 돈은 더 드릴게요…</x:t>
         </x:is>
       </x:c>
       <x:c r="F15" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">미용 요구 · 선택지 연결</x:t>
+          <x:t xml:space="preserve">기존 좀비 원문</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="16" ht="48" customHeight="1">
       <x:c r="A16" s="9">
-        <x:v>900016</x:v>
+        <x:v>900024</x:v>
       </x:c>
       <x:c r="B16" s="9">
-        <x:v>80004</x:v>
+        <x:v>80010</x:v>
       </x:c>
       <x:c r="C16" s="9">
         <x:v>1</x:v>
@@ -15382,7 +16322,7 @@
       </x:c>
       <x:c r="E16" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">아니, 앞이 안 보인다고요! 당장 '가위'를 들어서 내 눈을 가리는 앞머리를 싹 다 잘라달란 말입니다!</x:t>
+          <x:t xml:space="preserve">가위 내려놓으실래요? 제가 면접관이라 생각하고 대답해 보세요. 제 머리... 왜 이렇게 하셨죠?</x:t>
         </x:is>
       </x:c>
       <x:c r="F16" s="11" t="inlineStr">
@@ -15393,13 +16333,13 @@
     </x:row>
     <x:row r="17" ht="48" customHeight="1">
       <x:c r="A17" s="9">
-        <x:v>900017</x:v>
+        <x:v>900025</x:v>
       </x:c>
       <x:c r="B17" s="9">
-        <x:v>80005</x:v>
+        <x:v>80010</x:v>
       </x:c>
       <x:c r="C17" s="9">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D17" s="4" t="inlineStr">
         <x:is>
@@ -15408,7 +16348,7 @@
       </x:c>
       <x:c r="E17" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">으어어… 이게 제 눈이었군요…! 거울 속에 아주 준비된 인재가 한 명 서 있는데요…</x:t>
+          <x:t xml:space="preserve">마왕 법전 제 666조! 야차룰로 정하죠. 제가 이기면... 배상하시는 겁니다!!!</x:t>
         </x:is>
       </x:c>
       <x:c r="F17" s="11" t="inlineStr">
@@ -15419,10 +16359,10 @@
     </x:row>
     <x:row r="18" ht="48" customHeight="1">
       <x:c r="A18" s="9">
-        <x:v>900018</x:v>
+        <x:v>900026</x:v>
       </x:c>
       <x:c r="B18" s="9">
-        <x:v>80006</x:v>
+        <x:v>80011</x:v>
       </x:c>
       <x:c r="C18" s="9">
         <x:v>1</x:v>
@@ -15434,7 +16374,7 @@
       </x:c>
       <x:c r="E18" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">으어어… 일단 앞은 보이네요… 면접관이 한 분만 오시면 딱 좋겠어요…</x:t>
+          <x:t xml:space="preserve">으어어... 제가 대인배라 넘어갑니다... 다른 손님에겐 이렇게 하지 마세요...</x:t>
         </x:is>
       </x:c>
       <x:c r="F18" s="11" t="inlineStr">
@@ -15445,10 +16385,10 @@
     </x:row>
     <x:row r="19" ht="48" customHeight="1">
       <x:c r="A19" s="9">
-        <x:v>900019</x:v>
+        <x:v>900027</x:v>
       </x:c>
       <x:c r="B19" s="9">
-        <x:v>80007</x:v>
+        <x:v>80012</x:v>
       </x:c>
       <x:c r="C19" s="9">
         <x:v>1</x:v>
@@ -15460,7 +16400,7 @@
       </x:c>
       <x:c r="E19" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">으어어어! 이게 머립니까?? 이 꼴을 하고 면접을 가라고요?! 안 되겠다, 이대론 돈 못 냅니다!</x:t>
+          <x:t xml:space="preserve">으... 어쩔 수 없죠. 저도 면접 볼 체력을 아끼는 걸로 할게요. 머리 잘 해주셔서 감사합니다...</x:t>
         </x:is>
       </x:c>
       <x:c r="F19" s="11" t="inlineStr">
@@ -15471,10 +16411,10 @@
     </x:row>
     <x:row r="20" ht="48" customHeight="1">
       <x:c r="A20" s="9">
-        <x:v>900020</x:v>
+        <x:v>900028</x:v>
       </x:c>
       <x:c r="B20" s="9">
-        <x:v>80008</x:v>
+        <x:v>80013</x:v>
       </x:c>
       <x:c r="C20" s="9">
         <x:v>1</x:v>
@@ -15486,7 +16426,7 @@
       </x:c>
       <x:c r="E20" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">머리도 잘 됐겠다, 제 기세를 한 번 시험해 주시겠어요? 면접 때 자신있게 싸울... 아니 말할 수 있는지 봐주시면 됩니다.</x:t>
+          <x:t xml:space="preserve">으... 어쩔 수 없죠. 저도 면접 볼 체력을 아끼는 걸로 할게요. 감사합니다...</x:t>
         </x:is>
       </x:c>
       <x:c r="F20" s="11" t="inlineStr">
@@ -15497,13 +16437,13 @@
     </x:row>
     <x:row r="21" ht="48" customHeight="1">
       <x:c r="A21" s="9">
-        <x:v>900021</x:v>
+        <x:v>900029</x:v>
       </x:c>
       <x:c r="B21" s="9">
-        <x:v>80008</x:v>
+        <x:v>80014</x:v>
       </x:c>
       <x:c r="C21" s="9">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D21" s="4" t="inlineStr">
         <x:is>
@@ -15512,7 +16452,7 @@
       </x:c>
       <x:c r="E21" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">연습 야차 상대를... 부탁드린다는 뜻입니다... 저를 이기시면... 보상은 두둑히 드릴게요...</x:t>
+          <x:t xml:space="preserve">감사합니다…! 실수로 물어도 이해해주세요… 물고 늘어지는 건 제 장점이라...</x:t>
         </x:is>
       </x:c>
       <x:c r="F21" s="11" t="inlineStr">
@@ -15523,10 +16463,10 @@
     </x:row>
     <x:row r="22" ht="48" customHeight="1">
       <x:c r="A22" s="9">
-        <x:v>900022</x:v>
+        <x:v>900030</x:v>
       </x:c>
       <x:c r="B22" s="9">
-        <x:v>80009</x:v>
+        <x:v>80015</x:v>
       </x:c>
       <x:c r="C22" s="9">
         <x:v>1</x:v>
@@ -15538,7 +16478,7 @@
       </x:c>
       <x:c r="E22" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">머리도 됐으니... 제 기세를 한 번 시험해 주시겠어요? 면접 때 자신있게 싸울... 아니 말할 수 있는지 봐주시면 됩니다.</x:t>
+          <x:t xml:space="preserve">감사합니다…! 실수로 물어도 이해해주세요… 물고 늘어지는 건 제 장점이라...</x:t>
         </x:is>
       </x:c>
       <x:c r="F22" s="11" t="inlineStr">
@@ -15549,13 +16489,13 @@
     </x:row>
     <x:row r="23" ht="48" customHeight="1">
       <x:c r="A23" s="9">
-        <x:v>900023</x:v>
+        <x:v>900031</x:v>
       </x:c>
       <x:c r="B23" s="9">
-        <x:v>80009</x:v>
+        <x:v>80016</x:v>
       </x:c>
       <x:c r="C23" s="9">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D23" s="4" t="inlineStr">
         <x:is>
@@ -15564,7 +16504,7 @@
       </x:c>
       <x:c r="E23" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">연습 야차 상대를... 부탁드린다는 뜻입니다...저를 이기시면... 돈은 더 드릴게요…</x:t>
+          <x:t xml:space="preserve">으어어...&lt;wait=0.35&gt; 안녕하십니까…!&lt;wait=0.25&gt; 하,&lt;wait=0.25&gt; 한번 맡은 일은 죽어서도 노, &lt;wait=0.25&gt;놓지 않는 지원자… &lt;wait=0.35&gt;으어어…&lt;wait=0.35&gt; 실제로 죽어봤습니다!</x:t>
         </x:is>
       </x:c>
       <x:c r="F23" s="11" t="inlineStr">
@@ -15575,10 +16515,10 @@
     </x:row>
     <x:row r="24" ht="48" customHeight="1">
       <x:c r="A24" s="9">
-        <x:v>900024</x:v>
+        <x:v>900032</x:v>
       </x:c>
       <x:c r="B24" s="9">
-        <x:v>80010</x:v>
+        <x:v>80017</x:v>
       </x:c>
       <x:c r="C24" s="9">
         <x:v>1</x:v>
@@ -15590,7 +16530,7 @@
       </x:c>
       <x:c r="E24" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">가위 내려놓으실래요? 제가 면접관이라 생각하고 대답해 보세요. 제 머리... 왜 이렇게 하셨죠?</x:t>
+          <x:t xml:space="preserve">변명은 됐습니다…&lt;wait=0.35&gt; 저도 이빨 좀 쓰겠습니다!</x:t>
         </x:is>
       </x:c>
       <x:c r="F24" s="11" t="inlineStr">
@@ -15601,13 +16541,13 @@
     </x:row>
     <x:row r="25" ht="48" customHeight="1">
       <x:c r="A25" s="9">
-        <x:v>900025</x:v>
+        <x:v>900033</x:v>
       </x:c>
       <x:c r="B25" s="9">
-        <x:v>80010</x:v>
+        <x:v>80018</x:v>
       </x:c>
       <x:c r="C25" s="9">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D25" s="4" t="inlineStr">
         <x:is>
@@ -15616,7 +16556,7 @@
       </x:c>
       <x:c r="E25" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">마왕 법전 제 666조! 야차룰로 정하죠. 제가 이기면... 배상하시는 겁니다!!!</x:t>
+          <x:t xml:space="preserve">제, &lt;wait=0.25&gt;제 강점은… &lt;wait=0.35&gt;끈질긴 후속 연락입니다…!</x:t>
         </x:is>
       </x:c>
       <x:c r="F25" s="11" t="inlineStr">
@@ -15627,13 +16567,13 @@
     </x:row>
     <x:row r="26" ht="48" customHeight="1">
       <x:c r="A26" s="9">
-        <x:v>900026</x:v>
+        <x:v>900034</x:v>
       </x:c>
       <x:c r="B26" s="9">
-        <x:v>80011</x:v>
+        <x:v>80018</x:v>
       </x:c>
       <x:c r="C26" s="9">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D26" s="4" t="inlineStr">
         <x:is>
@@ -15642,7 +16582,7 @@
       </x:c>
       <x:c r="E26" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">으어어... 제가 대인배라 넘어갑니다... 다른 손님에겐 이렇게 하지 마세요...</x:t>
+          <x:t xml:space="preserve">정시 출근...&lt;wait=0.35&gt; 아니,&lt;wait=0.25&gt; 정시 타격입니다...!</x:t>
         </x:is>
       </x:c>
       <x:c r="F26" s="11" t="inlineStr">
@@ -15653,10 +16593,10 @@
     </x:row>
     <x:row r="27" ht="48" customHeight="1">
       <x:c r="A27" s="9">
-        <x:v>900027</x:v>
+        <x:v>900035</x:v>
       </x:c>
       <x:c r="B27" s="9">
-        <x:v>80012</x:v>
+        <x:v>80019</x:v>
       </x:c>
       <x:c r="C27" s="9">
         <x:v>1</x:v>
@@ -15668,7 +16608,7 @@
       </x:c>
       <x:c r="E27" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">으... 어쩔 수 없죠. 저도 면접 볼 체력을 아끼는 걸로 할게요. 머리 잘 해주셔서 감사합니다...</x:t>
+          <x:t xml:space="preserve">이건...&lt;wait=0.35&gt; 고객 피드백입니다...!</x:t>
         </x:is>
       </x:c>
       <x:c r="F27" s="11" t="inlineStr">
@@ -15679,13 +16619,13 @@
     </x:row>
     <x:row r="28" ht="48" customHeight="1">
       <x:c r="A28" s="9">
-        <x:v>900028</x:v>
+        <x:v>900036</x:v>
       </x:c>
       <x:c r="B28" s="9">
-        <x:v>80013</x:v>
+        <x:v>80019</x:v>
       </x:c>
       <x:c r="C28" s="9">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D28" s="4" t="inlineStr">
         <x:is>
@@ -15694,7 +16634,7 @@
       </x:c>
       <x:c r="E28" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">으... 어쩔 수 없죠. 저도 면접 볼 체력을 아끼는 걸로 할게요. 감사합니다...</x:t>
+          <x:t xml:space="preserve">서류 30번 떨어진 한...&lt;wait=0.35&gt; 받아라!!</x:t>
         </x:is>
       </x:c>
       <x:c r="F28" s="11" t="inlineStr">
@@ -15705,10 +16645,10 @@
     </x:row>
     <x:row r="29" ht="48" customHeight="1">
       <x:c r="A29" s="9">
-        <x:v>900029</x:v>
+        <x:v>900037</x:v>
       </x:c>
       <x:c r="B29" s="9">
-        <x:v>80014</x:v>
+        <x:v>80020</x:v>
       </x:c>
       <x:c r="C29" s="9">
         <x:v>1</x:v>
@@ -15720,7 +16660,7 @@
       </x:c>
       <x:c r="E29" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">감사합니다…! 실수로 물어도 이해해주세요… 물고 늘어지는 건 제 장점이라...</x:t>
+          <x:t xml:space="preserve">으어어…&lt;wait=0.35&gt; 머리만은 건드리지 말아주세요…!</x:t>
         </x:is>
       </x:c>
       <x:c r="F29" s="11" t="inlineStr">
@@ -15731,10 +16671,10 @@
     </x:row>
     <x:row r="30" ht="48" customHeight="1">
       <x:c r="A30" s="9">
-        <x:v>900030</x:v>
+        <x:v>900038</x:v>
       </x:c>
       <x:c r="B30" s="9">
-        <x:v>80015</x:v>
+        <x:v>80021</x:v>
       </x:c>
       <x:c r="C30" s="9">
         <x:v>1</x:v>
@@ -15746,7 +16686,7 @@
       </x:c>
       <x:c r="E30" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">감사합니다…! 실수로 물어도 이해해주세요… 물고 늘어지는 건 제 장점이라...</x:t>
+          <x:t xml:space="preserve">커헉... &lt;wait=0.35&gt;스펙이 너무 높아...</x:t>
         </x:is>
       </x:c>
       <x:c r="F30" s="11" t="inlineStr">
@@ -15757,10 +16697,10 @@
     </x:row>
     <x:row r="31" ht="48" customHeight="1">
       <x:c r="A31" s="9">
-        <x:v>900031</x:v>
+        <x:v>900039</x:v>
       </x:c>
       <x:c r="B31" s="9">
-        <x:v>80016</x:v>
+        <x:v>80022</x:v>
       </x:c>
       <x:c r="C31" s="9">
         <x:v>1</x:v>
@@ -15772,7 +16712,7 @@
       </x:c>
       <x:c r="E31" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">안녕하십니까…! 한번 맡은 일은 죽어서도 놓지 않는 지원자… 으어어… 실제로 죽어봤습니다!</x:t>
+          <x:t xml:space="preserve">제,&lt;wait=0.25&gt; 제 기세에,&lt;wait=0.25&gt; 압도되셨군요...!</x:t>
         </x:is>
       </x:c>
       <x:c r="F31" s="11" t="inlineStr">
@@ -15783,10 +16723,10 @@
     </x:row>
     <x:row r="32" ht="48" customHeight="1">
       <x:c r="A32" s="9">
-        <x:v>900032</x:v>
+        <x:v>900040</x:v>
       </x:c>
       <x:c r="B32" s="9">
-        <x:v>80017</x:v>
+        <x:v>80023</x:v>
       </x:c>
       <x:c r="C32" s="9">
         <x:v>1</x:v>
@@ -15798,7 +16738,7 @@
       </x:c>
       <x:c r="E32" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">변명은 됐습니다… 저도 이빨 좀 쓰겠습니다!</x:t>
+          <x:t xml:space="preserve">버, &lt;wait=0.25&gt;벌써 지치셨,&lt;wait=0.25&gt; 습니까?&lt;wait=0.35&gt; 감점 들어갑니다.</x:t>
         </x:is>
       </x:c>
       <x:c r="F32" s="11" t="inlineStr">
@@ -15809,10 +16749,10 @@
     </x:row>
     <x:row r="33" ht="48" customHeight="1">
       <x:c r="A33" s="9">
-        <x:v>900033</x:v>
+        <x:v>900041</x:v>
       </x:c>
       <x:c r="B33" s="9">
-        <x:v>80018</x:v>
+        <x:v>80024</x:v>
       </x:c>
       <x:c r="C33" s="9">
         <x:v>1</x:v>
@@ -15824,7 +16764,7 @@
       </x:c>
       <x:c r="E33" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">제 강점은… 끈질긴 후속 연락입니다…!</x:t>
+          <x:t xml:space="preserve">으어어... &lt;wait=0.25&gt;지, &lt;wait=0.25&gt;지금 보니 이 머리도 괜찮네요...</x:t>
         </x:is>
       </x:c>
       <x:c r="F33" s="11" t="inlineStr">
@@ -15835,13 +16775,13 @@
     </x:row>
     <x:row r="34" ht="48" customHeight="1">
       <x:c r="A34" s="9">
-        <x:v>900034</x:v>
+        <x:v>900042</x:v>
       </x:c>
       <x:c r="B34" s="9">
-        <x:v>80018</x:v>
+        <x:v>80025</x:v>
       </x:c>
       <x:c r="C34" s="9">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D34" s="4" t="inlineStr">
         <x:is>
@@ -15850,7 +16790,7 @@
       </x:c>
       <x:c r="E34" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">정시 출근... 아니, 정시 타격입니다!</x:t>
+          <x:t xml:space="preserve">약속대로...&lt;wait=0.35&gt; 돈은 돌려받겠습니다...</x:t>
         </x:is>
       </x:c>
       <x:c r="F34" s="11" t="inlineStr">
@@ -15861,10 +16801,10 @@
     </x:row>
     <x:row r="35" ht="48" customHeight="1">
       <x:c r="A35" s="9">
-        <x:v>900035</x:v>
+        <x:v>900043</x:v>
       </x:c>
       <x:c r="B35" s="9">
-        <x:v>80019</x:v>
+        <x:v>80026</x:v>
       </x:c>
       <x:c r="C35" s="9">
         <x:v>1</x:v>
@@ -15876,7 +16816,7 @@
       </x:c>
       <x:c r="E35" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">이건... 고객 피드백입니다...!</x:t>
+          <x:t xml:space="preserve">여, 역시 이 정도는 되어야... &lt;wait=0.35&gt;취업 성공하는 거군요...&lt;wait=0.35&gt; 리스펙합니다.</x:t>
         </x:is>
       </x:c>
       <x:c r="F35" s="11" t="inlineStr">
@@ -15887,13 +16827,13 @@
     </x:row>
     <x:row r="36" ht="48" customHeight="1">
       <x:c r="A36" s="9">
-        <x:v>900036</x:v>
+        <x:v>900044</x:v>
       </x:c>
       <x:c r="B36" s="9">
-        <x:v>80019</x:v>
+        <x:v>80027</x:v>
       </x:c>
       <x:c r="C36" s="9">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D36" s="4" t="inlineStr">
         <x:is>
@@ -15902,7 +16842,7 @@
       </x:c>
       <x:c r="E36" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">서류 30번 떨어진 한... 받아라!!</x:t>
+          <x:t xml:space="preserve">으어어어! &lt;wait=0.35&gt;이 기세로 합격까지,&lt;wait=0.25&gt; 갑니다!</x:t>
         </x:is>
       </x:c>
       <x:c r="F36" s="11" t="inlineStr">
@@ -15913,10 +16853,10 @@
     </x:row>
     <x:row r="37" ht="48" customHeight="1">
       <x:c r="A37" s="9">
-        <x:v>900037</x:v>
+        <x:v>900048</x:v>
       </x:c>
       <x:c r="B37" s="9">
-        <x:v>80020</x:v>
+        <x:v>80029</x:v>
       </x:c>
       <x:c r="C37" s="9">
         <x:v>1</x:v>
@@ -15928,7 +16868,7 @@
       </x:c>
       <x:c r="E37" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">으어어… 머리만은 건드리지 말아주세요…!</x:t>
+          <x:t xml:space="preserve">으어… 머리도 잘됐고… 태어나서 처음으로 자신감이 생겼어요… 죽은 뒤에 생기긴 했지만…</x:t>
         </x:is>
       </x:c>
       <x:c r="F37" s="11" t="inlineStr">
@@ -15939,22 +16879,22 @@
     </x:row>
     <x:row r="38" ht="48" customHeight="1">
       <x:c r="A38" s="9">
-        <x:v>900038</x:v>
+        <x:v>900049</x:v>
       </x:c>
       <x:c r="B38" s="9">
-        <x:v>80021</x:v>
+        <x:v>80029</x:v>
       </x:c>
       <x:c r="C38" s="9">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D38" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">몬스터</x:t>
+          <x:t xml:space="preserve">플레이어</x:t>
         </x:is>
       </x:c>
       <x:c r="E38" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">커헉... 스펙이 너무 높아...</x:t>
+          <x:t xml:space="preserve">그 자신감으로 내일은 말로 설득 가보자고요~!!</x:t>
         </x:is>
       </x:c>
       <x:c r="F38" s="11" t="inlineStr">
@@ -15965,13 +16905,13 @@
     </x:row>
     <x:row r="39" ht="48" customHeight="1">
       <x:c r="A39" s="9">
-        <x:v>900039</x:v>
+        <x:v>900050</x:v>
       </x:c>
       <x:c r="B39" s="9">
-        <x:v>80022</x:v>
+        <x:v>80029</x:v>
       </x:c>
       <x:c r="C39" s="9">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D39" s="4" t="inlineStr">
         <x:is>
@@ -15980,7 +16920,7 @@
       </x:c>
       <x:c r="E39" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">제 기세에 압도되셨군요...!</x:t>
+          <x:t xml:space="preserve">네... 그럼 안녕히...</x:t>
         </x:is>
       </x:c>
       <x:c r="F39" s="11" t="inlineStr">
@@ -15991,10 +16931,10 @@
     </x:row>
     <x:row r="40" ht="48" customHeight="1">
       <x:c r="A40" s="9">
-        <x:v>900040</x:v>
+        <x:v>900051</x:v>
       </x:c>
       <x:c r="B40" s="9">
-        <x:v>80023</x:v>
+        <x:v>80030</x:v>
       </x:c>
       <x:c r="C40" s="9">
         <x:v>1</x:v>
@@ -16006,7 +16946,7 @@
       </x:c>
       <x:c r="E40" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">벌써 지치셨습니까? 감점 들어갑니다.</x:t>
+          <x:t xml:space="preserve">으어어…머리가 헝클어졌네... 내일도 이러면 어떡하죠…</x:t>
         </x:is>
       </x:c>
       <x:c r="F40" s="11" t="inlineStr">
@@ -16017,22 +16957,22 @@
     </x:row>
     <x:row r="41" ht="48" customHeight="1">
       <x:c r="A41" s="9">
-        <x:v>900041</x:v>
+        <x:v>900052</x:v>
       </x:c>
       <x:c r="B41" s="9">
-        <x:v>80024</x:v>
+        <x:v>80030</x:v>
       </x:c>
       <x:c r="C41" s="9">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D41" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">몬스터</x:t>
+          <x:t xml:space="preserve">플레이어</x:t>
         </x:is>
       </x:c>
       <x:c r="E41" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">이럴 수가... 머리도 잃고 돈도 잃다니... 으어어...</x:t>
+          <x:t xml:space="preserve">초~ 큐트한 키라키라★리본 머리핀 있는데 드릴까요?</x:t>
         </x:is>
       </x:c>
       <x:c r="F41" s="11" t="inlineStr">
@@ -16043,13 +16983,13 @@
     </x:row>
     <x:row r="42" ht="48" customHeight="1">
       <x:c r="A42" s="9">
-        <x:v>900042</x:v>
+        <x:v>900053</x:v>
       </x:c>
       <x:c r="B42" s="9">
-        <x:v>80025</x:v>
+        <x:v>80030</x:v>
       </x:c>
       <x:c r="C42" s="9">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D42" s="4" t="inlineStr">
         <x:is>
@@ -16058,7 +16998,7 @@
       </x:c>
       <x:c r="E42" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">약속대로... 돈은 돌려받겠습니다...</x:t>
+          <x:t xml:space="preserve">아니요... 친근한 인상으로 승부해볼게요...</x:t>
         </x:is>
       </x:c>
       <x:c r="F42" s="11" t="inlineStr">
@@ -16069,13 +17009,13 @@
     </x:row>
     <x:row r="43" ht="48" customHeight="1">
       <x:c r="A43" s="9">
-        <x:v>900043</x:v>
+        <x:v>900054</x:v>
       </x:c>
       <x:c r="B43" s="9">
-        <x:v>80026</x:v>
+        <x:v>80030</x:v>
       </x:c>
       <x:c r="C43" s="9">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D43" s="4" t="inlineStr">
         <x:is>
@@ -16084,7 +17024,7 @@
       </x:c>
       <x:c r="E43" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">역시 이 정도는 되어야... 취업 성공하는 거군요... 리스펙합니다.</x:t>
+          <x:t xml:space="preserve">그럼 안녕히…</x:t>
         </x:is>
       </x:c>
       <x:c r="F43" s="11" t="inlineStr">
@@ -16095,10 +17035,10 @@
     </x:row>
     <x:row r="44" ht="48" customHeight="1">
       <x:c r="A44" s="9">
-        <x:v>900044</x:v>
+        <x:v>900055</x:v>
       </x:c>
       <x:c r="B44" s="9">
-        <x:v>80027</x:v>
+        <x:v>80031</x:v>
       </x:c>
       <x:c r="C44" s="9">
         <x:v>1</x:v>
@@ -16110,7 +17050,7 @@
       </x:c>
       <x:c r="E44" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">으어어! 이 기세로 합격까지 갑니다!</x:t>
+          <x:t xml:space="preserve">으어어… 어찌저찌 이겼으니… 내일 면접도 어떻게든 되겠죠…</x:t>
         </x:is>
       </x:c>
       <x:c r="F44" s="11" t="inlineStr">
@@ -16121,22 +17061,22 @@
     </x:row>
     <x:row r="45" ht="48" customHeight="1">
       <x:c r="A45" s="9">
-        <x:v>900045</x:v>
+        <x:v>900056</x:v>
       </x:c>
       <x:c r="B45" s="9">
-        <x:v>80028</x:v>
+        <x:v>80031</x:v>
       </x:c>
       <x:c r="C45" s="9">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D45" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">몬스터</x:t>
+          <x:t xml:space="preserve">플레이어</x:t>
         </x:is>
       </x:c>
       <x:c r="E45" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">으어어… 머리도 단정하고… 두들겨 맞아서 어깨 힘도 빠졌네요… 면접 준비 끝났어요…</x:t>
+          <x:t xml:space="preserve">에에~ 면접이랑 싸움은 별개쟝~</x:t>
         </x:is>
       </x:c>
       <x:c r="F45" s="11" t="inlineStr">
@@ -16147,22 +17087,22 @@
     </x:row>
     <x:row r="46" ht="48" customHeight="1">
       <x:c r="A46" s="9">
-        <x:v>900046</x:v>
+        <x:v>900057</x:v>
       </x:c>
       <x:c r="B46" s="9">
-        <x:v>80028</x:v>
+        <x:v>80031</x:v>
       </x:c>
       <x:c r="C46" s="9">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D46" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">플레이어</x:t>
+          <x:t xml:space="preserve">몬스터</x:t>
         </x:is>
       </x:c>
       <x:c r="E46" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">긴장 덜고 웃음 MAX로 승부보는 거예요~! 얏호~!</x:t>
+          <x:t xml:space="preserve">그건 그렇죠... 어쨌든 감사합니다...</x:t>
         </x:is>
       </x:c>
       <x:c r="F46" s="11" t="inlineStr">
@@ -16173,13 +17113,13 @@
     </x:row>
     <x:row r="47" ht="48" customHeight="1">
       <x:c r="A47" s="9">
-        <x:v>900047</x:v>
+        <x:v>900058</x:v>
       </x:c>
       <x:c r="B47" s="9">
-        <x:v>80028</x:v>
+        <x:v>80031</x:v>
       </x:c>
       <x:c r="C47" s="9">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D47" s="4" t="inlineStr">
         <x:is>
@@ -16188,7 +17128,7 @@
       </x:c>
       <x:c r="E47" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">네… 계약서는 물지 않고… 서명받겠습니다…</x:t>
+          <x:t xml:space="preserve">그럼 안녕히…</x:t>
         </x:is>
       </x:c>
       <x:c r="F47" s="11" t="inlineStr">
@@ -16199,10 +17139,10 @@
     </x:row>
     <x:row r="48" ht="48" customHeight="1">
       <x:c r="A48" s="9">
-        <x:v>900048</x:v>
+        <x:v>900059</x:v>
       </x:c>
       <x:c r="B48" s="9">
-        <x:v>80029</x:v>
+        <x:v>80032</x:v>
       </x:c>
       <x:c r="C48" s="9">
         <x:v>1</x:v>
@@ -16214,7 +17154,7 @@
       </x:c>
       <x:c r="E48" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">으어… 머리도 잘됐고… 태어나서 처음으로 자신감이 생겼어요… 죽은 뒤에 생기긴 했지만…</x:t>
+          <x:t xml:space="preserve">으어어… 내일 이 머리 얘기가 나오면… 뭐라고 해야 할까요…</x:t>
         </x:is>
       </x:c>
       <x:c r="F48" s="11" t="inlineStr">
@@ -16225,10 +17165,10 @@
     </x:row>
     <x:row r="49" ht="48" customHeight="1">
       <x:c r="A49" s="9">
-        <x:v>900049</x:v>
+        <x:v>900060</x:v>
       </x:c>
       <x:c r="B49" s="9">
-        <x:v>80029</x:v>
+        <x:v>80032</x:v>
       </x:c>
       <x:c r="C49" s="9">
         <x:v>2</x:v>
@@ -16240,7 +17180,7 @@
       </x:c>
       <x:c r="E49" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">그 자신감으로 내일은 말로 설득 가보자고요~!!</x:t>
+          <x:t xml:space="preserve">초- 신선한 유행의 선두주자― 인데스케도 면접관이 사람 보는 눈이 없는 거네~</x:t>
         </x:is>
       </x:c>
       <x:c r="F49" s="11" t="inlineStr">
@@ -16251,10 +17191,10 @@
     </x:row>
     <x:row r="50" ht="48" customHeight="1">
       <x:c r="A50" s="9">
-        <x:v>900050</x:v>
+        <x:v>900061</x:v>
       </x:c>
       <x:c r="B50" s="9">
-        <x:v>80029</x:v>
+        <x:v>80032</x:v>
       </x:c>
       <x:c r="C50" s="9">
         <x:v>3</x:v>
@@ -16266,7 +17206,7 @@
       </x:c>
       <x:c r="E50" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">네... 그럼 안녕히...</x:t>
+          <x:t xml:space="preserve">새로운 시도를 두려워하지 않는다는 거죠... 어떻게든 해볼게요...</x:t>
         </x:is>
       </x:c>
       <x:c r="F50" s="11" t="inlineStr">
@@ -16277,10 +17217,10 @@
     </x:row>
     <x:row r="51" ht="48" customHeight="1">
       <x:c r="A51" s="9">
-        <x:v>900051</x:v>
+        <x:v>900062</x:v>
       </x:c>
       <x:c r="B51" s="9">
-        <x:v>80030</x:v>
+        <x:v>80033</x:v>
       </x:c>
       <x:c r="C51" s="9">
         <x:v>1</x:v>
@@ -16292,7 +17232,7 @@
       </x:c>
       <x:c r="E51" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">으어어…머리가 헝클어졌네... 내일도 이러면 어떡하죠…</x:t>
+          <x:t xml:space="preserve">으어어… 내일 이 머리 얘기가 나오면… 뭐라고 해야 하지…</x:t>
         </x:is>
       </x:c>
       <x:c r="F51" s="11" t="inlineStr">
@@ -16303,10 +17243,10 @@
     </x:row>
     <x:row r="52" ht="48" customHeight="1">
       <x:c r="A52" s="9">
-        <x:v>900052</x:v>
+        <x:v>900063</x:v>
       </x:c>
       <x:c r="B52" s="9">
-        <x:v>80030</x:v>
+        <x:v>80033</x:v>
       </x:c>
       <x:c r="C52" s="9">
         <x:v>2</x:v>
@@ -16318,7 +17258,7 @@
       </x:c>
       <x:c r="E52" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">초~ 큐트한 키라키라★리본 머리핀 있는데 드릴까요?</x:t>
+          <x:t xml:space="preserve">초- 신선한 유행의 선두주자― 인데스케도 면접관이 사람 보는 눈이 없는 거네~</x:t>
         </x:is>
       </x:c>
       <x:c r="F52" s="11" t="inlineStr">
@@ -16329,10 +17269,10 @@
     </x:row>
     <x:row r="53" ht="48" customHeight="1">
       <x:c r="A53" s="9">
-        <x:v>900053</x:v>
+        <x:v>900064</x:v>
       </x:c>
       <x:c r="B53" s="9">
-        <x:v>80030</x:v>
+        <x:v>80033</x:v>
       </x:c>
       <x:c r="C53" s="9">
         <x:v>3</x:v>
@@ -16344,7 +17284,7 @@
       </x:c>
       <x:c r="E53" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">아니요... 친근한 인상으로 승부해볼게요...</x:t>
+          <x:t xml:space="preserve">........상당히 뻔뻔하시네요… 으어어….어떻게든 되겠죠…</x:t>
         </x:is>
       </x:c>
       <x:c r="F53" s="11" t="inlineStr">
@@ -16355,10 +17295,10 @@
     </x:row>
     <x:row r="54" ht="48" customHeight="1">
       <x:c r="A54" s="9">
-        <x:v>900054</x:v>
+        <x:v>900065</x:v>
       </x:c>
       <x:c r="B54" s="9">
-        <x:v>80030</x:v>
+        <x:v>80033</x:v>
       </x:c>
       <x:c r="C54" s="9">
         <x:v>4</x:v>
@@ -16370,7 +17310,7 @@
       </x:c>
       <x:c r="E54" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">그럼 안녕히…</x:t>
+          <x:t xml:space="preserve">이번에도 탈락하면... 대체 언제.....하아…</x:t>
         </x:is>
       </x:c>
       <x:c r="F54" s="11" t="inlineStr">
@@ -16381,10 +17321,10 @@
     </x:row>
     <x:row r="55" ht="48" customHeight="1">
       <x:c r="A55" s="9">
-        <x:v>900055</x:v>
+        <x:v>900066</x:v>
       </x:c>
       <x:c r="B55" s="9">
-        <x:v>80031</x:v>
+        <x:v>80034</x:v>
       </x:c>
       <x:c r="C55" s="9">
         <x:v>1</x:v>
@@ -16396,7 +17336,7 @@
       </x:c>
       <x:c r="E55" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">으어어… 어찌저찌 이겼으니… 내일 면접도 어떻게든 되겠죠…</x:t>
+          <x:t xml:space="preserve">으어... 취직했다... 앞머리도 방구석 생활도 해방됨...... 몇달만에 사람 얼굴 제대로 보는 느낌ㅠㅠ #몬스터헤어살롱 덕분에 붙은 것 같아요 감사합니다. 모두 기 받아가세요! #취업성공 #취준생 #화이팅</x:t>
         </x:is>
       </x:c>
       <x:c r="F55" s="11" t="inlineStr">
@@ -16407,22 +17347,22 @@
     </x:row>
     <x:row r="56" ht="48" customHeight="1">
       <x:c r="A56" s="9">
-        <x:v>900056</x:v>
+        <x:v>900067</x:v>
       </x:c>
       <x:c r="B56" s="9">
-        <x:v>80031</x:v>
+        <x:v>80035</x:v>
       </x:c>
       <x:c r="C56" s="9">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D56" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">플레이어</x:t>
+          <x:t xml:space="preserve">몬스터</x:t>
         </x:is>
       </x:c>
       <x:c r="E56" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">에에~ 면접이랑 싸움은 별개쟝~</x:t>
+          <x:t xml:space="preserve">역시나 면접 떨어졌다….. #취준생 #절규 #미용실저주함 돈도 잃고 머리도 잃음</x:t>
         </x:is>
       </x:c>
       <x:c r="F56" s="11" t="inlineStr">
@@ -16433,13 +17373,13 @@
     </x:row>
     <x:row r="57" ht="48" customHeight="1">
       <x:c r="A57" s="9">
-        <x:v>900057</x:v>
+        <x:v>900068</x:v>
       </x:c>
       <x:c r="B57" s="9">
-        <x:v>80031</x:v>
+        <x:v>80036</x:v>
       </x:c>
       <x:c r="C57" s="9">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D57" s="4" t="inlineStr">
         <x:is>
@@ -16448,24 +17388,24 @@
       </x:c>
       <x:c r="E57" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">그건 그렇죠... 어쨌든 감사합니다...</x:t>
+          <x:t xml:space="preserve">&lt;wave=3 speed=5&gt;&lt;color=#FFD166&gt;&lt;size=24&gt;으하하하!&lt;/size&gt;&lt;/color&gt; 오랜만이구먼, &lt;color=#FFDA8A&gt;제이!!&lt;/color&gt;&lt;/wave&gt;&lt;wait=0.25&gt; 미용실에 불이 켜졌길래... 드디어 돌아온 줄 알았지!</x:t>
         </x:is>
       </x:c>
       <x:c r="F57" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">기존 좀비 원문</x:t>
+          <x:t xml:space="preserve">취객의 가업·제이·몬스터 소울을 떠올리는 단서. 실제 해금·튜토리얼은 야차 이후 미용실에서 진행.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="58" ht="48" customHeight="1">
       <x:c r="A58" s="9">
-        <x:v>900058</x:v>
+        <x:v>900070</x:v>
       </x:c>
       <x:c r="B58" s="9">
-        <x:v>80031</x:v>
+        <x:v>80038</x:v>
       </x:c>
       <x:c r="C58" s="9">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D58" s="4" t="inlineStr">
         <x:is>
@@ -16474,21 +17414,21 @@
       </x:c>
       <x:c r="E58" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">그럼 안녕히…</x:t>
+          <x:t xml:space="preserve">&lt;shake=2 speed=15 dur=0.45&gt;어이쿠!&lt;/shake&gt;&lt;wait=0.3&gt; 손맛 한번 여전하구먼.&lt;wave=2 speed=4&gt; 근데 제이, 자네... 원래 둘이었나?&lt;/wave&gt;</x:t>
         </x:is>
       </x:c>
       <x:c r="F58" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">기존 좀비 원문</x:t>
+          <x:t xml:space="preserve">색·동작 태그는 문자 효과 규칙 시트 참고.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="59" ht="48" customHeight="1">
       <x:c r="A59" s="9">
-        <x:v>900059</x:v>
+        <x:v>900071</x:v>
       </x:c>
       <x:c r="B59" s="9">
-        <x:v>80032</x:v>
+        <x:v>80039</x:v>
       </x:c>
       <x:c r="C59" s="9">
         <x:v>1</x:v>
@@ -16500,50 +17440,50 @@
       </x:c>
       <x:c r="E59" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">으어어… 내일 이 머리 얘기가 나오면… 뭐라고 해야 할까요…</x:t>
+          <x:t xml:space="preserve">어...&lt;wait=0.4&gt; &lt;color=#A9E4DA&gt;이제 한 명으로 보이네.&lt;/color&gt; 제이가... 아니군.&lt;wait=0.45&gt; 미용실에 불이 들어왔길래, 그 녀석인 줄 알았어.</x:t>
         </x:is>
       </x:c>
       <x:c r="F59" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">기존 좀비 원문</x:t>
+          <x:t xml:space="preserve">취객의 가업·제이·몬스터 소울을 떠올리는 단서. 실제 해금·튜토리얼은 야차 이후 미용실에서 진행.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="60" ht="48" customHeight="1">
       <x:c r="A60" s="9">
-        <x:v>900060</x:v>
+        <x:v>900072</x:v>
       </x:c>
       <x:c r="B60" s="9">
-        <x:v>80032</x:v>
+        <x:v>80040</x:v>
       </x:c>
       <x:c r="C60" s="9">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D60" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">플레이어</x:t>
+          <x:t xml:space="preserve">몬스터</x:t>
         </x:is>
       </x:c>
       <x:c r="E60" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">초- 신선한 유행의 선두주자― 인데스케도 면접관이 사람 보는 눈이 없는 거네~</x:t>
+          <x:t xml:space="preserve">허... 막일할 때도 굳어 있던 손이...&lt;wait=0.4&gt; 이 감각, &lt;color=#FFD166&gt;소울을 벼리던 때&lt;/color&gt;랑 닮았구먼.&lt;wait=0.3&gt; 제이가 봤으면 또 실실 웃었겠어!</x:t>
         </x:is>
       </x:c>
       <x:c r="F60" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">기존 좀비 원문</x:t>
+          <x:t xml:space="preserve">취객의 가업·제이·몬스터 소울을 떠올리는 단서. 실제 해금·튜토리얼은 야차 이후 미용실에서 진행.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="61" ht="48" customHeight="1">
       <x:c r="A61" s="9">
-        <x:v>900061</x:v>
+        <x:v>900073</x:v>
       </x:c>
       <x:c r="B61" s="9">
-        <x:v>80032</x:v>
+        <x:v>80041</x:v>
       </x:c>
       <x:c r="C61" s="9">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D61" s="4" t="inlineStr">
         <x:is>
@@ -16552,21 +17492,22 @@
       </x:c>
       <x:c r="E61" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">새로운 시도를 두려워하지 않는다는 거죠... 어떻게든 해볼게요...</x:t>
+          <x:t xml:space="preserve">&lt;shake=2 speed=16 dur=0.4&gt;크하!&lt;/shake&gt; ...&lt;wait=0.4&gt;&lt;color=#B7F4D0&gt;다 깼다, 다 깼어!&lt;/color&gt;
+옛 솜씨도 술에 몽땅 절여진 줄 알았더니! &lt;pulse=1.1 speed=7&gt;아직 쓸 만하구먼! 으하하하!&lt;/pulse&gt;</x:t>
         </x:is>
       </x:c>
       <x:c r="F61" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">기존 좀비 원문</x:t>
+          <x:t xml:space="preserve">취객의 가업·제이·몬스터 소울을 떠올리는 단서. 실제 해금·튜토리얼은 야차 이후 미용실에서 진행.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="62" ht="48" customHeight="1">
       <x:c r="A62" s="9">
-        <x:v>900062</x:v>
+        <x:v>900074</x:v>
       </x:c>
       <x:c r="B62" s="9">
-        <x:v>80033</x:v>
+        <x:v>80042</x:v>
       </x:c>
       <x:c r="C62" s="9">
         <x:v>1</x:v>
@@ -16578,50 +17519,50 @@
       </x:c>
       <x:c r="E62" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">으어어… 내일 이 머리 얘기가 나오면… 뭐라고 해야 하지…</x:t>
+          <x:t xml:space="preserve">우리 집안은 &lt;color=#FFD166&gt;몬스터 소울을 장비와 기술로 벼렸지.&lt;/color&gt; 세상은 바뀌고, 찾는 이도 줄고...&lt;wait=0.4&gt; 제이까지 사라지고 나니 더 붙들 이유가 없더군.</x:t>
         </x:is>
       </x:c>
       <x:c r="F62" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">기존 좀비 원문</x:t>
+          <x:t xml:space="preserve">취객의 가업·제이·몬스터 소울을 떠올리는 단서. 실제 해금·튜토리얼은 야차 이후 미용실에서 진행.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="63" ht="48" customHeight="1">
       <x:c r="A63" s="9">
-        <x:v>900063</x:v>
+        <x:v>900075</x:v>
       </x:c>
       <x:c r="B63" s="9">
-        <x:v>80033</x:v>
+        <x:v>80042</x:v>
       </x:c>
       <x:c r="C63" s="9">
         <x:v>2</x:v>
       </x:c>
       <x:c r="D63" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">플레이어</x:t>
+          <x:t xml:space="preserve">몬스터</x:t>
         </x:is>
       </x:c>
       <x:c r="E63" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">초- 신선한 유행의 선두주자― 인데스케도 면접관이 사람 보는 눈이 없는 거네~</x:t>
+          <x:t xml:space="preserve">그런데 그 미용실에 &lt;color=#B7F4D0&gt;다시 불이 켜졌어.&lt;/color&gt;&lt;wait=0.4&gt; 내 손도 아직 기억하고 있고. 돌아가세. 자네한테 보여줄 게 떠올랐거든! &lt;wave=2 speed=6&gt;&lt;color=#FFD166&gt;으하하하!&lt;/color&gt;&lt;/wave&gt;</x:t>
         </x:is>
       </x:c>
       <x:c r="F63" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">기존 좀비 원문</x:t>
+          <x:t xml:space="preserve">취객의 가업·제이·몬스터 소울을 떠올리는 단서. 실제 해금·튜토리얼은 야차 이후 미용실에서 진행.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="64" ht="48" customHeight="1">
       <x:c r="A64" s="9">
-        <x:v>900064</x:v>
+        <x:v>900069</x:v>
       </x:c>
       <x:c r="B64" s="9">
-        <x:v>80033</x:v>
+        <x:v>80037</x:v>
       </x:c>
       <x:c r="C64" s="9">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D64" s="4" t="inlineStr">
         <x:is>
@@ -16630,24 +17571,24 @@
       </x:c>
       <x:c r="E64" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">........상당히 뻔뻔하시네요… 으어어….어떻게든 되겠죠…</x:t>
+          <x:t xml:space="preserve">헤.&lt;wait=0.35&gt; 오늘은... &lt;wait=0.25&gt;&lt;color=#8BE9FD&gt;가볍게&lt;/color&gt; 가자고,&lt;wait=0.25&gt; 친구. &lt;wait=0.35&gt; 내 &lt;color=#1900d6&gt;파란 공격&lt;/color&gt;은 알고 있겠지?</x:t>
         </x:is>
       </x:c>
       <x:c r="F64" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">기존 좀비 원문</x:t>
+          <x:t xml:space="preserve">색·동작 태그는 문자 효과 규칙 시트 참고.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="65" ht="48" customHeight="1">
       <x:c r="A65" s="9">
-        <x:v>900065</x:v>
+        <x:v>900076</x:v>
       </x:c>
       <x:c r="B65" s="9">
-        <x:v>80033</x:v>
+        <x:v>80043</x:v>
       </x:c>
       <x:c r="C65" s="9">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D65" s="4" t="inlineStr">
         <x:is>
@@ -16656,21 +17597,21 @@
       </x:c>
       <x:c r="E65" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">이번에도 탈락하면... 대체 언제.....하아…</x:t>
+          <x:t xml:space="preserve">뭐야? &lt;wait=0.35&gt;그럼 내가 &lt;wave=2&gt;가만히 서서 맞아줄 줄 알았어?&lt;/wave&gt;</x:t>
         </x:is>
       </x:c>
       <x:c r="F65" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">기존 좀비 원문</x:t>
+          <x:t xml:space="preserve">색·동작 태그는 문자 효과 규칙 시트 참고.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="66" ht="48" customHeight="1">
       <x:c r="A66" s="9">
-        <x:v>900066</x:v>
+        <x:v>900077</x:v>
       </x:c>
       <x:c r="B66" s="9">
-        <x:v>80034</x:v>
+        <x:v>80044</x:v>
       </x:c>
       <x:c r="C66" s="9">
         <x:v>1</x:v>
@@ -16682,21 +17623,21 @@
       </x:c>
       <x:c r="E66" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">으어... 취직했다... 앞머리도 방구석 생활도 해방됨...... 몇달만에 사람 얼굴 제대로 보는 느낌ㅠㅠ #몬스터헤어살롱 덕분에 붙은 것 같아요 감사합니다. 모두 기 받아가세요! #취업성공 #취준생 #화이팅</x:t>
+          <x:t xml:space="preserve">어라? &lt;wait=0.35&gt;&lt;wave=1.4&gt;여기서 맞으면 안 되지 않나?&lt;/wave&gt;</x:t>
         </x:is>
       </x:c>
       <x:c r="F66" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">기존 좀비 원문</x:t>
+          <x:t xml:space="preserve">색·동작 태그는 문자 효과 규칙 시트 참고.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="67" ht="48" customHeight="1">
       <x:c r="A67" s="9">
-        <x:v>900067</x:v>
+        <x:v>900078</x:v>
       </x:c>
       <x:c r="B67" s="9">
-        <x:v>80035</x:v>
+        <x:v>80045</x:v>
       </x:c>
       <x:c r="C67" s="9">
         <x:v>1</x:v>
@@ -16708,21 +17649,21 @@
       </x:c>
       <x:c r="E67" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">역시나 면접 떨어졌다….. #취준생 #절규 #미용실저주함 돈도 잃고 머리도 잃음</x:t>
+          <x:t xml:space="preserve">너, &lt;wait=0.25&gt;그, &lt;wait=0.25&gt;&lt;pulse=1.15&gt;그거 휘두르는 거 진짜 좋아하는구나, &lt;wait=0.25&gt;응?&lt;/pulse&gt;</x:t>
         </x:is>
       </x:c>
       <x:c r="F67" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">기존 좀비 원문</x:t>
+          <x:t xml:space="preserve">색·동작 태그는 문자 효과 규칙 시트 참고.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="68" ht="48" customHeight="1">
       <x:c r="A68" s="9">
-        <x:v>900068</x:v>
+        <x:v>900079</x:v>
       </x:c>
       <x:c r="B68" s="9">
-        <x:v>80036</x:v>
+        <x:v>80046</x:v>
       </x:c>
       <x:c r="C68" s="9">
         <x:v>1</x:v>
@@ -16734,21 +17675,21 @@
       </x:c>
       <x:c r="E68" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">&lt;wave=3 speed=5&gt;&lt;color=#FFD166&gt;&lt;size=24&gt;으하하하!&lt;/size&gt;&lt;/color&gt; 오랜만이구먼, &lt;color=#FFDA8A&gt;제이!!&lt;/color&gt;&lt;/wave&gt;&lt;wait=0.25&gt; 미용실에 불이 켜졌길래... 드디어 돌아온 줄 알았지!</x:t>
+          <x:t xml:space="preserve">&lt;shake=2&gt;으악!!&lt;/shake&gt;&lt;wait=0.5&gt; &lt;wave=1&gt;크흠, &lt;wait=0.25&gt;큼,&lt;wait=0.25&gt; 그러니까, &lt;/wave&gt;&lt;wait=0.35&gt;아무것도 아니었어, 헤.</x:t>
         </x:is>
       </x:c>
       <x:c r="F68" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">취객의 가업·제이·몬스터 소울을 떠올리는 단서. 실제 해금·튜토리얼은 야차 이후 미용실에서 진행.</x:t>
+          <x:t xml:space="preserve">색·동작 태그는 문자 효과 규칙 시트 참고.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="69" ht="48" customHeight="1">
       <x:c r="A69" s="9">
-        <x:v>900070</x:v>
+        <x:v>900080</x:v>
       </x:c>
       <x:c r="B69" s="9">
-        <x:v>80038</x:v>
+        <x:v>80047</x:v>
       </x:c>
       <x:c r="C69" s="9">
         <x:v>1</x:v>
@@ -16760,7 +17701,7 @@
       </x:c>
       <x:c r="E69" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">&lt;shake=2 speed=15 dur=0.45&gt;어이쿠!&lt;/shake&gt;&lt;wait=0.3&gt; 손맛 한번 여전하구먼.&lt;wave=2 speed=4&gt; 근데 제이, 자네... 원래 둘이었나?&lt;/wave&gt;</x:t>
+          <x:t xml:space="preserve">&lt;wave=1&gt;잠깐... &lt;wait=0.25&gt;친구야,&lt;/wave&gt;&lt;wait=0.25&gt; &lt;shake=1.4&gt;나 기억 안 나?&lt;/shake&gt;&lt;wait=0.5&gt; &lt;shake=1.4&gt;그냥 다 잊어버리자고,&lt;wait=0.25&gt; 알겠지?&lt;/shake&gt;</x:t>
         </x:is>
       </x:c>
       <x:c r="F69" s="11" t="inlineStr">
@@ -16771,10 +17712,10 @@
     </x:row>
     <x:row r="70" ht="48" customHeight="1">
       <x:c r="A70" s="9">
-        <x:v>900071</x:v>
+        <x:v>900081</x:v>
       </x:c>
       <x:c r="B70" s="9">
-        <x:v>80039</x:v>
+        <x:v>80048</x:v>
       </x:c>
       <x:c r="C70" s="9">
         <x:v>1</x:v>
@@ -16786,21 +17727,21 @@
       </x:c>
       <x:c r="E70" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">어...&lt;wait=0.4&gt; &lt;color=#A9E4DA&gt;이제 한 명으로 보이네.&lt;/color&gt; 제이가... 아니군.&lt;wait=0.45&gt; 미용실에 불이 들어왔길래, 그 녀석인 줄 알았어.</x:t>
+          <x:t xml:space="preserve">그냥...&lt;wait=0.4&gt; &lt;shake=1.2&gt;닮지 않았다고만 하지 말아줘.&lt;/shake&gt;</x:t>
         </x:is>
       </x:c>
       <x:c r="F70" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">취객의 가업·제이·몬스터 소울을 떠올리는 단서. 실제 해금·튜토리얼은 야차 이후 미용실에서 진행.</x:t>
+          <x:t xml:space="preserve">색·동작 태그는 문자 효과 규칙 시트 참고.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="71" ht="48" customHeight="1">
       <x:c r="A71" s="9">
-        <x:v>900072</x:v>
+        <x:v>900082</x:v>
       </x:c>
       <x:c r="B71" s="9">
-        <x:v>80040</x:v>
+        <x:v>80049</x:v>
       </x:c>
       <x:c r="C71" s="9">
         <x:v>1</x:v>
@@ -16812,24 +17753,24 @@
       </x:c>
       <x:c r="E71" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">허... 막일할 때도 굳어 있던 손이...&lt;wait=0.4&gt; 이 감각, &lt;color=#FFD166&gt;소울을 벼리던 때&lt;/color&gt;랑 닮았구먼.&lt;wait=0.3&gt; 제이가 봤으면 또 실실 웃었겠어!</x:t>
+          <x:t xml:space="preserve">&lt;wave=2 speed=5&gt;&lt;color=#B7F4D0&gt;으어어...&lt;wait=0.35&gt;&lt;/color&gt;&lt;/wave&gt; 손 좀 빌려주세요.&lt;wait=0.35&gt; 아, &lt;wait=0.25&gt;&lt;shake=2 dur=0.4&gt;떼어주시진 말고...!&lt;/shake&gt;</x:t>
         </x:is>
       </x:c>
       <x:c r="F71" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">취객의 가업·제이·몬스터 소울을 떠올리는 단서. 실제 해금·튜토리얼은 야차 이후 미용실에서 진행.</x:t>
+          <x:t xml:space="preserve">전투 중 대사. 등장·미용 과정 대사는 보류.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="72" ht="48" customHeight="1">
       <x:c r="A72" s="9">
-        <x:v>900073</x:v>
+        <x:v>900083</x:v>
       </x:c>
       <x:c r="B72" s="9">
-        <x:v>80041</x:v>
+        <x:v>80049</x:v>
       </x:c>
       <x:c r="C72" s="9">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D72" s="4" t="inlineStr">
         <x:is>
@@ -16838,22 +17779,21 @@
       </x:c>
       <x:c r="E72" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">&lt;shake=2 speed=16 dur=0.4&gt;크하!&lt;/shake&gt; ...&lt;wait=0.4&gt;&lt;color=#B7F4D0&gt;다 깼다, 다 깼어!&lt;/color&gt;
-옛 솜씨도 술에 몽땅 절여진 줄 알았더니! &lt;pulse=1.1 speed=7&gt;아직 쓸 만하구먼! 으하하하!&lt;/pulse&gt;</x:t>
+          <x:t xml:space="preserve">&lt;color=#FFD166&gt;끈기&lt;wait=0.25&gt;&lt;/color&gt;, 하나는 자신 있습니다...!&lt;wait=0.3&gt; &lt;wave=2 speed=5&gt;죽어서도 출근하잖아요...&lt;/wave&gt;</x:t>
         </x:is>
       </x:c>
       <x:c r="F72" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">취객의 가업·제이·몬스터 소울을 떠올리는 단서. 실제 해금·튜토리얼은 야차 이후 미용실에서 진행.</x:t>
+          <x:t xml:space="preserve">전투 중 대사. 등장·미용 과정 대사는 보류.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="73" ht="48" customHeight="1">
       <x:c r="A73" s="9">
-        <x:v>900074</x:v>
+        <x:v>900084</x:v>
       </x:c>
       <x:c r="B73" s="9">
-        <x:v>80042</x:v>
+        <x:v>80050</x:v>
       </x:c>
       <x:c r="C73" s="9">
         <x:v>1</x:v>
@@ -16865,24 +17805,24 @@
       </x:c>
       <x:c r="E73" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">우리 집안은 &lt;color=#FFD166&gt;몬스터 소울을 장비와 기술로 벼렸지.&lt;/color&gt; 세상은 바뀌고, 찾는 이도 줄고...&lt;wait=0.4&gt; 제이까지 사라지고 나니 더 붙들 이유가 없더군.</x:t>
+          <x:t xml:space="preserve">잠깐...&lt;wait=0.25&gt; &lt;shake=2 speed=16 dur=0.5&gt;뼈 때리시면...!&lt;wait=0.25&gt;&lt;/shake&gt; &lt;color=#FFD166&gt;지, &lt;wait=0.25&gt;진짜 뼈 맞는다고요...!&lt;/color&gt;</x:t>
         </x:is>
       </x:c>
       <x:c r="F73" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">취객의 가업·제이·몬스터 소울을 떠올리는 단서. 실제 해금·튜토리얼은 야차 이후 미용실에서 진행.</x:t>
+          <x:t xml:space="preserve">전투 중 대사. 등장·미용 과정 대사는 보류.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="74" ht="48" customHeight="1">
       <x:c r="A74" s="9">
-        <x:v>900075</x:v>
+        <x:v>900085</x:v>
       </x:c>
       <x:c r="B74" s="9">
-        <x:v>80042</x:v>
+        <x:v>80051</x:v>
       </x:c>
       <x:c r="C74" s="9">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D74" s="4" t="inlineStr">
         <x:is>
@@ -16891,24 +17831,25 @@
       </x:c>
       <x:c r="E74" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">그런데 그 미용실에 &lt;color=#B7F4D0&gt;다시 불이 켜졌어.&lt;/color&gt;&lt;wait=0.4&gt; 내 손도 아직 기억하고 있고. 돌아가세. 자네한테 보여줄 게 떠올랐거든! &lt;wave=2 speed=6&gt;&lt;color=#FFD166&gt;으하하하!&lt;/color&gt;&lt;/wave&gt;</x:t>
+          <x:t xml:space="preserve">&lt;cps=15&gt;끝난 줄... 아셨죠?&lt;/cps&gt;&lt;wait=0.5&gt; &lt;color=#B7F4D0&gt;&lt;size=23&gt;좀비는 다시 부활한다구요!&lt;/size&gt;&lt;/color&gt;
+&lt;shake=3 speed=16 dur=0.8&gt;&lt;wave=3 speed=5&gt;으어어어..!&lt;/wave&gt;&lt;/shake&gt;</x:t>
         </x:is>
       </x:c>
       <x:c r="F74" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">취객의 가업·제이·몬스터 소울을 떠올리는 단서. 실제 해금·튜토리얼은 야차 이후 미용실에서 진행.</x:t>
+          <x:t xml:space="preserve">전투 중 대사. 등장·미용 과정 대사는 보류.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="75" ht="48" customHeight="1">
       <x:c r="A75" s="9">
-        <x:v>900069</x:v>
+        <x:v>900086</x:v>
       </x:c>
       <x:c r="B75" s="9">
-        <x:v>80037</x:v>
+        <x:v>80051</x:v>
       </x:c>
       <x:c r="C75" s="9">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D75" s="4" t="inlineStr">
         <x:is>
@@ -16917,21 +17858,21 @@
       </x:c>
       <x:c r="E75" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">헤헤.&lt;wait=0.35&gt; 오늘은... &lt;color=#8BE9FD&gt;가볍게&lt;/color&gt; 가자고, 친구.</x:t>
+          <x:t xml:space="preserve">&lt;color=#FFD166&gt;재도전&lt;/color&gt;에는 자신 있습니다.&lt;wait=0.35&gt; 취업도...&lt;wait=0.5&gt; 이렇게 쉽게 부활하면 좋을 텐데요.</x:t>
         </x:is>
       </x:c>
       <x:c r="F75" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">색·동작 태그는 문자 효과 규칙 시트 참고.</x:t>
+          <x:t xml:space="preserve">전투 중 대사. 등장·미용 과정 대사는 보류.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="76" ht="48" customHeight="1">
       <x:c r="A76" s="9">
-        <x:v>900076</x:v>
+        <x:v>900087</x:v>
       </x:c>
       <x:c r="B76" s="9">
-        <x:v>80043</x:v>
+        <x:v>80052</x:v>
       </x:c>
       <x:c r="C76" s="9">
         <x:v>1</x:v>
@@ -16943,21 +17884,22 @@
       </x:c>
       <x:c r="E76" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">...하하.. 친구..&lt;wait=0.4&gt; 나한텐 &lt;color=#8BE9FD&gt;무용지물&lt;/color&gt;일 텐데..?</x:t>
+          <x:t xml:space="preserve">&lt;wave=2 speed=3&gt;으어어...&lt;/wave&gt;&lt;wait=0.4&gt; 오늘은 여기까지...
+&lt;color=#B7F4D0&gt;재도전도 휴식이 필요하다구요.&lt;/color&gt;</x:t>
         </x:is>
       </x:c>
       <x:c r="F76" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">색·동작 태그는 문자 효과 규칙 시트 참고.</x:t>
+          <x:t xml:space="preserve">전투 중 대사. 등장·미용 과정 대사는 보류.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="77" ht="48" customHeight="1">
       <x:c r="A77" s="9">
-        <x:v>900077</x:v>
+        <x:v>900088</x:v>
       </x:c>
       <x:c r="B77" s="9">
-        <x:v>80044</x:v>
+        <x:v>80053</x:v>
       </x:c>
       <x:c r="C77" s="9">
         <x:v>1</x:v>
@@ -16969,21 +17911,21 @@
       </x:c>
       <x:c r="E77" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">뭐...&lt;wait=0.45&gt; 이 정도는 맞아줄 수 있지.&lt;wait=0.3&gt; &lt;color=#8BE9FD&gt;서비스&lt;/color&gt;라고 해 두자고.</x:t>
+          <x:t xml:space="preserve">&lt;color=#FFD166&gt;끈기 있는 지원자!&lt;/color&gt; 저, 맞죠?&lt;wait=0.3&gt; &lt;wave=2 speed=5&gt;으허허... 아직 쓸 만하네요!&lt;/wave&gt;</x:t>
         </x:is>
       </x:c>
       <x:c r="F77" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">색·동작 태그는 문자 효과 규칙 시트 참고.</x:t>
+          <x:t xml:space="preserve">전투 중 대사. 등장·미용 과정 대사는 보류.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="78" ht="48" customHeight="1">
       <x:c r="A78" s="9">
-        <x:v>900078</x:v>
+        <x:v>900089</x:v>
       </x:c>
       <x:c r="B78" s="9">
-        <x:v>80045</x:v>
+        <x:v>80054</x:v>
       </x:c>
       <x:c r="C78" s="9">
         <x:v>1</x:v>
@@ -16995,21 +17937,22 @@
       </x:c>
       <x:c r="E78" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">헤헤... 같은 수는 두 번 안 통한다고.&lt;wait=0.35&gt; ...방금 건 &lt;color=#8BE9FD&gt;연습&lt;/color&gt;이었지?</x:t>
+          <x:t xml:space="preserve">면접에선,&lt;wait=0.25&gt; 으어,&lt;wait=0.25&gt; 첫인상이 중요하니까요...
+덜 긴, 긴장하려면,&lt;wait=0.25&gt; &lt;color=#9A5B22&gt;&lt;pulse=1.06&gt;단정한 인상&lt;/pulse&gt;&lt;/color&gt;이면 덜 긴장할 것 같아요...&lt;wait=0.35&gt; 으어어...</x:t>
         </x:is>
       </x:c>
       <x:c r="F78" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">색·동작 태그는 문자 효과 규칙 시트 참고.</x:t>
+          <x:t xml:space="preserve">미용 요구 · 선택지 연결</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="79" ht="48" customHeight="1">
       <x:c r="A79" s="9">
-        <x:v>900079</x:v>
+        <x:v>900090</x:v>
       </x:c>
       <x:c r="B79" s="9">
-        <x:v>80046</x:v>
+        <x:v>80055</x:v>
       </x:c>
       <x:c r="C79" s="9">
         <x:v>1</x:v>
@@ -17021,21 +17964,22 @@
       </x:c>
       <x:c r="E79" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">...어라.&lt;wait=0.6&gt; 그 타이밍을 또 맞혔네.&lt;wait=0.35&gt; &lt;shake=1.4 speed=14&gt;좀 쉬엄쉬엄하자고, 친구.&lt;/shake&gt;</x:t>
+          <x:t xml:space="preserve">으어어...&lt;wait=0.35&gt; 염색은 &lt;wave=1.2&gt;&lt;color=#71508F&gt;아무렇게나&lt;/color&gt;&lt;/wave&gt; 괜찮아요...
+저, &lt;wait=0.25&gt;저는,&lt;wait=0.25&gt; &lt;color=#266B4D&gt;지금 머리 색도&lt;/color&gt;,&lt;wait=0.25&gt; 좋아요...</x:t>
         </x:is>
       </x:c>
       <x:c r="F79" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">색·동작 태그는 문자 효과 규칙 시트 참고.</x:t>
+          <x:t xml:space="preserve">미용 요구 · 선택지 연결</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="80" ht="48" customHeight="1">
       <x:c r="A80" s="9">
-        <x:v>900080</x:v>
+        <x:v>900091</x:v>
       </x:c>
       <x:c r="B80" s="9">
-        <x:v>80047</x:v>
+        <x:v>80056</x:v>
       </x:c>
       <x:c r="C80" s="9">
         <x:v>1</x:v>
@@ -17047,22 +17991,21 @@
       </x:c>
       <x:c r="E80" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">잠깐,&lt;wait=0.45&gt; 우리...&lt;wait=0.45&gt; &lt;color=#8BE9FD&gt;친구잖아..?&lt;/color&gt;
-&lt;shake=2.2 speed=20&gt;날 정말 죽일 셈이야..?&lt;/shake&gt;</x:t>
+          <x:t xml:space="preserve">&lt;wave=1&gt;으어어… &lt;wait=0.35&gt;머리도 하고…&lt;wait=0.35&gt; 상쾌하게 몸도 풀고...&lt;wait=0.35&gt; 면접 준비 끝났어요...&lt;/wave&gt;</x:t>
         </x:is>
       </x:c>
       <x:c r="F80" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">색·동작 태그는 문자 효과 규칙 시트 참고.</x:t>
+          <x:t xml:space="preserve">통합 플레이</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="81" ht="48" customHeight="1">
       <x:c r="A81" s="9">
-        <x:v>900081</x:v>
+        <x:v>900092</x:v>
       </x:c>
       <x:c r="B81" s="9">
-        <x:v>80048</x:v>
+        <x:v>80057</x:v>
       </x:c>
       <x:c r="C81" s="9">
         <x:v>1</x:v>
@@ -17074,21 +18017,21 @@
       </x:c>
       <x:c r="E81" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">나는 이래서...&lt;wait=0.65&gt; &lt;cps=16&gt;&lt;shake=1.6 speed=16&gt;&lt;color=#FF9797&gt;눈치 빠른 애송이들이 싫어...&lt;/color&gt;&lt;/shake&gt;&lt;/cps&gt;</x:t>
+          <x:t xml:space="preserve">&lt;wave=1&gt;으어어...&lt;wait=0.35&gt; 연습은 여기까지 하죠...&lt;wait=0.35&gt; 저도 내일 면접이 있어서요.&lt;/wave&gt;</x:t>
         </x:is>
       </x:c>
       <x:c r="F81" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">색·동작 태그는 문자 효과 규칙 시트 참고.</x:t>
+          <x:t xml:space="preserve">통합 플레이</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="82" ht="48" customHeight="1">
       <x:c r="A82" s="9">
-        <x:v>900082</x:v>
+        <x:v>900093</x:v>
       </x:c>
       <x:c r="B82" s="9">
-        <x:v>80049</x:v>
+        <x:v>80058</x:v>
       </x:c>
       <x:c r="C82" s="9">
         <x:v>1</x:v>
@@ -17100,21 +18043,21 @@
       </x:c>
       <x:c r="E82" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">&lt;wave=2 speed=5&gt;&lt;color=#B7F4D0&gt;으어어...&lt;/color&gt;&lt;/wave&gt; 손 좀 빌려주세요.&lt;wait=0.25&gt; 아, &lt;shake=2 dur=0.4&gt;떼어드리진 말구요!&lt;/shake&gt;</x:t>
+          <x:t xml:space="preserve">&lt;shake=2&gt;으하하하!&lt;/shake&gt; 오랜만이구먼, 제이!!</x:t>
         </x:is>
       </x:c>
       <x:c r="F82" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">전투 중 대사. 등장·미용 과정 대사는 보류.</x:t>
+          <x:t xml:space="preserve">통합 플레이</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="83" ht="48" customHeight="1">
       <x:c r="A83" s="9">
-        <x:v>900083</x:v>
+        <x:v>900094</x:v>
       </x:c>
       <x:c r="B83" s="9">
-        <x:v>80049</x:v>
+        <x:v>80058</x:v>
       </x:c>
       <x:c r="C83" s="9">
         <x:v>2</x:v>
@@ -17126,21 +18069,21 @@
       </x:c>
       <x:c r="E83" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">&lt;color=#FFD166&gt;끈기&lt;/color&gt; 하나는 자신 있습니다!&lt;wait=0.3&gt; &lt;wave=2 speed=5&gt;죽어서도 출근하잖아요...&lt;/wave&gt;</x:t>
+          <x:t xml:space="preserve">가게에 불이 켜져 있길래 냅다 뛰어왔지! 이야, 얼굴이 좀... &lt;wave=3&gt;두 개로 보이는구먼!&lt;/wave&gt;</x:t>
         </x:is>
       </x:c>
       <x:c r="F83" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">전투 중 대사. 등장·미용 과정 대사는 보류.</x:t>
+          <x:t xml:space="preserve">통합 플레이</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="84" ht="48" customHeight="1">
       <x:c r="A84" s="9">
-        <x:v>900084</x:v>
+        <x:v>900095</x:v>
       </x:c>
       <x:c r="B84" s="9">
-        <x:v>80050</x:v>
+        <x:v>80059</x:v>
       </x:c>
       <x:c r="C84" s="9">
         <x:v>1</x:v>
@@ -17152,24 +18095,24 @@
       </x:c>
       <x:c r="E84" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">잠깐...&lt;wait=0.25&gt; &lt;shake=2 speed=16 dur=0.5&gt;뼈 때리시면!&lt;/shake&gt; &lt;color=#FFD166&gt;진짜 뼈 맞는다구요!&lt;/color&gt;</x:t>
+          <x:t xml:space="preserve">...자네, 제이가 아니었구먼. 허허. 이제야 제대로 보이는군.</x:t>
         </x:is>
       </x:c>
       <x:c r="F84" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">전투 중 대사. 등장·미용 과정 대사는 보류.</x:t>
+          <x:t xml:space="preserve">통합 플레이</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="85" ht="48" customHeight="1">
       <x:c r="A85" s="9">
-        <x:v>900085</x:v>
+        <x:v>900096</x:v>
       </x:c>
       <x:c r="B85" s="9">
-        <x:v>80051</x:v>
+        <x:v>80059</x:v>
       </x:c>
       <x:c r="C85" s="9">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D85" s="4" t="inlineStr">
         <x:is>
@@ -17178,25 +18121,24 @@
       </x:c>
       <x:c r="E85" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">&lt;cps=15&gt;끝난 줄... 아셨죠?&lt;/cps&gt;&lt;wait=0.5&gt; &lt;color=#B7F4D0&gt;&lt;size=23&gt;좀비는 다시 부활한다구요!&lt;/size&gt;&lt;/color&gt;
-&lt;shake=3 speed=16 dur=0.8&gt;&lt;wave=3 speed=5&gt;으어어어..!&lt;/wave&gt;&lt;/shake&gt;</x:t>
+          <x:t xml:space="preserve">제이가 사라진 뒤로 이 가게도, 내 손끝도 멈춘 줄 알았지. 일용직 일 끝내고 한잔하는 게 하루의 전부였어.</x:t>
         </x:is>
       </x:c>
       <x:c r="F85" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">전투 중 대사. 등장·미용 과정 대사는 보류.</x:t>
+          <x:t xml:space="preserve">통합 플레이</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="86" ht="48" customHeight="1">
       <x:c r="A86" s="9">
-        <x:v>900086</x:v>
+        <x:v>900097</x:v>
       </x:c>
       <x:c r="B86" s="9">
-        <x:v>80051</x:v>
+        <x:v>80059</x:v>
       </x:c>
       <x:c r="C86" s="9">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D86" s="4" t="inlineStr">
         <x:is>
@@ -17205,24 +18147,24 @@
       </x:c>
       <x:c r="E86" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">&lt;color=#FFD166&gt;재도전&lt;/color&gt;에는 자신 있습니다.&lt;wait=0.35&gt; 취업도...&lt;wait=0.5&gt; 이렇게 쉽게 부활하면 좋을 텐데요.</x:t>
+          <x:t xml:space="preserve">우리 집안은 몬스터의 소울에 남은 힘을 &lt;color=#9FE8D1&gt;장비와 기술로 빚어내던&lt;/color&gt; 일을 했네. 아는 이만 찾던 오래된 가업이지.</x:t>
         </x:is>
       </x:c>
       <x:c r="F86" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">전투 중 대사. 등장·미용 과정 대사는 보류.</x:t>
+          <x:t xml:space="preserve">통합 플레이</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="87" ht="48" customHeight="1">
       <x:c r="A87" s="9">
-        <x:v>900087</x:v>
+        <x:v>900098</x:v>
       </x:c>
       <x:c r="B87" s="9">
-        <x:v>80052</x:v>
+        <x:v>80059</x:v>
       </x:c>
       <x:c r="C87" s="9">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D87" s="4" t="inlineStr">
         <x:is>
@@ -17231,25 +18173,24 @@
       </x:c>
       <x:c r="E87" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">&lt;wave=2 speed=3&gt;으어어...&lt;/wave&gt;&lt;wait=0.4&gt; 오늘은 여기까지...
-&lt;color=#B7F4D0&gt;재도전도 휴식이 필요하다구요.&lt;/color&gt;</x:t>
+          <x:t xml:space="preserve">세상이 편리해지니 그 솜씨를 찾는 이도 줄었어. 다시 쓸 일이 없을 줄 알았는데... 자네를 보니, &lt;wave=2&gt;손이 근질근질하구먼!&lt;/wave&gt;</x:t>
         </x:is>
       </x:c>
       <x:c r="F87" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">전투 중 대사. 등장·미용 과정 대사는 보류.</x:t>
+          <x:t xml:space="preserve">통합 플레이</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="88" ht="48" customHeight="1">
       <x:c r="A88" s="9">
-        <x:v>900088</x:v>
+        <x:v>900099</x:v>
       </x:c>
       <x:c r="B88" s="9">
-        <x:v>80053</x:v>
+        <x:v>80059</x:v>
       </x:c>
       <x:c r="C88" s="9">
-        <x:v>1</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D88" s="4" t="inlineStr">
         <x:is>
@@ -17258,21 +18199,21 @@
       </x:c>
       <x:c r="E88" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">&lt;color=#FFD166&gt;끈기 있는 지원자!&lt;/color&gt; 저, 맞죠?&lt;wait=0.3&gt; &lt;wave=2 speed=5&gt;으허허... 아직 쓸 만하네요!&lt;/wave&gt;</x:t>
+          <x:t xml:space="preserve">좋아. 머물러도 된다면 손끝부터 다시 깨워 보지. &lt;color=#FFD166&gt;몬스터 소울을 다루는 법&lt;/color&gt;도 차근차근 알려 주겠네.</x:t>
         </x:is>
       </x:c>
       <x:c r="F88" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">전투 중 대사. 등장·미용 과정 대사는 보류.</x:t>
+          <x:t xml:space="preserve">통합 플레이</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="89" ht="48" customHeight="1">
       <x:c r="A89" s="9">
-        <x:v>900089</x:v>
+        <x:v>900100</x:v>
       </x:c>
       <x:c r="B89" s="9">
-        <x:v>80054</x:v>
+        <x:v>80060</x:v>
       </x:c>
       <x:c r="C89" s="9">
         <x:v>1</x:v>
@@ -17284,22 +18225,21 @@
       </x:c>
       <x:c r="E89" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">면접에선... 첫인상이 중요하다던데요...
-&lt;color=#9A5B22&gt;&lt;pulse=1.06&gt;단정한 인상&lt;/pulse&gt;&lt;/color&gt;이면... 덜 긴장할 것 같아요...</x:t>
+          <x:t xml:space="preserve">허허, 오늘은 술 대신 물 한 잔이면 되겠어. 도구를 챙겨 올 테니, 가게 불은 꺼뜨리지 말게!</x:t>
         </x:is>
       </x:c>
       <x:c r="F89" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">미용 요구 · 선택지 연결</x:t>
+          <x:t xml:space="preserve">통합 플레이</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="90" ht="48" customHeight="1">
       <x:c r="A90" s="9">
-        <x:v>900090</x:v>
+        <x:v>900101</x:v>
       </x:c>
       <x:c r="B90" s="9">
-        <x:v>80055</x:v>
+        <x:v>80061</x:v>
       </x:c>
       <x:c r="C90" s="9">
         <x:v>1</x:v>
@@ -17311,25 +18251,24 @@
       </x:c>
       <x:c r="E90" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">염색이요...? &lt;wave=1.2&gt;&lt;color=#71508F&gt;자유롭게&lt;/color&gt;&lt;/wave&gt; 부탁드려요...
-&lt;color=#266B4D&gt;지금 머리 색도&lt;/color&gt; 저는 좋은데...</x:t>
+          <x:t xml:space="preserve">...헤. &lt;wait=0.35&gt;여기 솜씨가 좋다는 소문을 들었거든.</x:t>
         </x:is>
       </x:c>
       <x:c r="F90" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">미용 요구 · 선택지 연결</x:t>
+          <x:t xml:space="preserve">통합 플레이</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="91" ht="48" customHeight="1">
       <x:c r="A91" s="9">
-        <x:v>900091</x:v>
+        <x:v>900102</x:v>
       </x:c>
       <x:c r="B91" s="9">
-        <x:v>80056</x:v>
+        <x:v>80061</x:v>
       </x:c>
       <x:c r="C91" s="9">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D91" s="4" t="inlineStr">
         <x:is>
@@ -17338,7 +18277,7 @@
       </x:c>
       <x:c r="E91" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">으어어... 머리도 정리하고, 정신도 번쩍 들었네요. 내일은 &lt;color=#FFD166&gt;면접장에 부활&lt;/color&gt;하겠습니다!</x:t>
+          <x:t xml:space="preserve">&lt;pulse=1.15&gt;"뼈"&lt;/pulse&gt; 있는 부탁 하나 해도 될까?&lt;wait=0.35&gt; &lt;color=#FFD166&gt;얼굴 테두리&lt;/color&gt;만 다듬어 줘. &lt;wait=0.35&gt;머리카락은... &lt;wait=0.35&gt;보다시피 휴가 중이야.</x:t>
         </x:is>
       </x:c>
       <x:c r="F91" s="11" t="inlineStr">
@@ -17349,10 +18288,10 @@
     </x:row>
     <x:row r="92" ht="48" customHeight="1">
       <x:c r="A92" s="9">
-        <x:v>900092</x:v>
+        <x:v>900103</x:v>
       </x:c>
       <x:c r="B92" s="9">
-        <x:v>80057</x:v>
+        <x:v>80062</x:v>
       </x:c>
       <x:c r="C92" s="9">
         <x:v>1</x:v>
@@ -17364,21 +18303,22 @@
       </x:c>
       <x:c r="E92" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">으어어... 연습은 여기까지 하죠. 저도 내일 면접이 있어서요.</x:t>
+          <x:t xml:space="preserve">헤. &lt;wait=0.35&gt;오늘은 &lt;color=#52609B&gt;인상 좀 다듬으러&lt;/color&gt; 왔어.&lt;wait=0.35&gt;
+&lt;color=#52609B&gt;각진 데만 가볍게.&lt;wait=0.35&gt;&lt;/color&gt; &lt;wave=1.3&gt;뼈대는 괜찮잖아?&lt;/wave&gt;</x:t>
         </x:is>
       </x:c>
       <x:c r="F92" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">통합 플레이</x:t>
+          <x:t xml:space="preserve">미용 요구 · 선택지 연결</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
       <x:c r="A93" s="9">
-        <x:v>900093</x:v>
+        <x:v>900104</x:v>
       </x:c>
       <x:c r="B93" s="9">
-        <x:v>80058</x:v>
+        <x:v>80063</x:v>
       </x:c>
       <x:c r="C93" s="9">
         <x:v>1</x:v>
@@ -17390,24 +18330,25 @@
       </x:c>
       <x:c r="E93" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">&lt;shake=2&gt;으하하하!&lt;/shake&gt; 오랜만이구먼, 제이!!</x:t>
+          <x:t xml:space="preserve">이번엔 좀 &lt;color=#9A4935&gt;&lt;shake=0.6&gt;만만하지 않은 인상&lt;/shake&gt;&lt;/color&gt;이면 좋겠어.&lt;wait=0.35&gt;
+&lt;color=#9A4935&gt;장식&lt;/color&gt;으로 한 수 보여 줄래?</x:t>
         </x:is>
       </x:c>
       <x:c r="F93" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">통합 플레이</x:t>
+          <x:t xml:space="preserve">미용 요구 · 선택지 연결</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="94" ht="48" customHeight="1">
       <x:c r="A94" s="9">
-        <x:v>900094</x:v>
+        <x:v>900105</x:v>
       </x:c>
       <x:c r="B94" s="9">
-        <x:v>80058</x:v>
+        <x:v>80064</x:v>
       </x:c>
       <x:c r="C94" s="9">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D94" s="4" t="inlineStr">
         <x:is>
@@ -17416,7 +18357,7 @@
       </x:c>
       <x:c r="E94" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">가게에 불이 켜져 있길래 냅다 뛰어왔지! 이야, 얼굴이 좀... &lt;wave=3&gt;두 개로 보이는구먼!&lt;/wave&gt;</x:t>
+          <x:t xml:space="preserve">헤. &lt;wait=0.35&gt;꽤 뼈대 있는 실력이네.&lt;wait=0.35&gt; 그럼... &lt;wait=0.35&gt;몸도 한번 풀어 볼까?</x:t>
         </x:is>
       </x:c>
       <x:c r="F94" s="11" t="inlineStr">
@@ -17427,10 +18368,10 @@
     </x:row>
     <x:row r="95" ht="48" customHeight="1">
       <x:c r="A95" s="9">
-        <x:v>900095</x:v>
+        <x:v>900106</x:v>
       </x:c>
       <x:c r="B95" s="9">
-        <x:v>80059</x:v>
+        <x:v>80065</x:v>
       </x:c>
       <x:c r="C95" s="9">
         <x:v>1</x:v>
@@ -17442,7 +18383,7 @@
       </x:c>
       <x:c r="E95" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">...자네, 제이가 아니었구먼. 허허. 이제야 제대로 보이는군.</x:t>
+          <x:t xml:space="preserve">나쁘지 않네.&lt;wait=0.35&gt; 이번엔 다른 솜씨도 보여 줄래?</x:t>
         </x:is>
       </x:c>
       <x:c r="F95" s="11" t="inlineStr">
@@ -17453,13 +18394,13 @@
     </x:row>
     <x:row r="96" ht="48" customHeight="1">
       <x:c r="A96" s="9">
-        <x:v>900096</x:v>
+        <x:v>900107</x:v>
       </x:c>
       <x:c r="B96" s="9">
-        <x:v>80059</x:v>
+        <x:v>80066</x:v>
       </x:c>
       <x:c r="C96" s="9">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D96" s="4" t="inlineStr">
         <x:is>
@@ -17468,7 +18409,7 @@
       </x:c>
       <x:c r="E96" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">제이가 사라진 뒤로 이 가게도, 내 손끝도 멈춘 줄 알았지. 일용직 일 끝내고 한잔하는 게 하루의 전부였어.</x:t>
+          <x:t xml:space="preserve">...친구, &lt;wait=0.35&gt;이건 좀 &lt;pulse=1.15&gt;"뼈"&lt;/pulse&gt;아픈데.&lt;wait=0.35&gt; 잠깐 밖에서 얘기할까?</x:t>
         </x:is>
       </x:c>
       <x:c r="F96" s="11" t="inlineStr">
@@ -17479,13 +18420,13 @@
     </x:row>
     <x:row r="97" ht="48" customHeight="1">
       <x:c r="A97" s="9">
-        <x:v>900097</x:v>
+        <x:v>900109</x:v>
       </x:c>
       <x:c r="B97" s="9">
-        <x:v>80059</x:v>
+        <x:v>80068</x:v>
       </x:c>
       <x:c r="C97" s="9">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D97" s="4" t="inlineStr">
         <x:is>
@@ -17494,24 +18435,25 @@
       </x:c>
       <x:c r="E97" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">우리 집안은 몬스터의 소울에 남은 힘을 &lt;color=#9FE8D1&gt;장비와 기술로 빚어내던&lt;/color&gt; 일을 했네. 아는 이만 찾던 오래된 가업이지.</x:t>
+          <x:t xml:space="preserve">&lt;color=#71508F&gt;무슨 색이든,&lt;wait=0.25&gt; 무슨 무늬든&lt;/color&gt; 사,&lt;wait=0.25&gt; 상관 없어요...&lt;wait=0.35&gt;
+&lt;color=#266B4D&gt;염색 안 해도 괜찮아요...&lt;/color&gt;&lt;wait=0.35&gt; 지금 머리도 마음에 들어요, &lt;wait=0.25&gt;으어...</x:t>
         </x:is>
       </x:c>
       <x:c r="F97" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">통합 플레이</x:t>
+          <x:t xml:space="preserve">미용 선택지 대사</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="98" ht="48" customHeight="1">
       <x:c r="A98" s="9">
-        <x:v>900098</x:v>
+        <x:v>900110</x:v>
       </x:c>
       <x:c r="B98" s="9">
-        <x:v>80059</x:v>
+        <x:v>80069</x:v>
       </x:c>
       <x:c r="C98" s="9">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D98" s="4" t="inlineStr">
         <x:is>
@@ -17520,24 +18462,25 @@
       </x:c>
       <x:c r="E98" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">세상이 편리해지니 그 솜씨를 찾는 이도 줄었어. 다시 쓸 일이 없을 줄 알았는데... 자네를 보니, &lt;wave=2&gt;손이 근질근질하구먼!&lt;/wave&gt;</x:t>
+          <x:t xml:space="preserve">&lt;color=#9A5B22&gt;단정하고 점잖아 보일 장식&lt;/color&gt;으로...&lt;wait=0.35&gt;
+&lt;color=#9A5B22&gt;하나만&lt;/color&gt;...&lt;wait=0.35&gt; 골라 주시겠어요?&lt;wait=0.35&gt; 으어,&lt;wait=0.25&gt; &lt;wave=1.2&gt;너무 요란, &lt;wait=0.25&gt;하진 않게요...&lt;/wave&gt;</x:t>
         </x:is>
       </x:c>
       <x:c r="F98" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">통합 플레이</x:t>
+          <x:t xml:space="preserve">미용 선택지 대사</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="99" ht="48" customHeight="1">
       <x:c r="A99" s="9">
-        <x:v>900099</x:v>
+        <x:v>900111</x:v>
       </x:c>
       <x:c r="B99" s="9">
-        <x:v>80059</x:v>
+        <x:v>80070</x:v>
       </x:c>
       <x:c r="C99" s="9">
-        <x:v>5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D99" s="4" t="inlineStr">
         <x:is>
@@ -17546,21 +18489,22 @@
       </x:c>
       <x:c r="E99" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">좋아. 머물러도 된다면 손끝부터 다시 깨워 보지. &lt;color=#FFD166&gt;몬스터 소울을 다루는 법&lt;/color&gt;도 차근차근 알려 주겠네.</x:t>
+          <x:t xml:space="preserve">&lt;color=#52609B&gt;얼굴 바깥 테두리만&lt;/color&gt; 망치랑 정으로 톡톡 다듬어 줘.&lt;wait=0.35&gt;
+&lt;color=#9A4935&gt;눈코입은 그대로.&lt;wait=0.35&gt;&lt;/color&gt; &lt;wave=1.2&gt;속까지 시원해질 필요는 없거든.&lt;/wave&gt;</x:t>
         </x:is>
       </x:c>
       <x:c r="F99" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">통합 플레이</x:t>
+          <x:t xml:space="preserve">미용 선택지 대사</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="100" ht="48" customHeight="1">
       <x:c r="A100" s="9">
-        <x:v>900100</x:v>
+        <x:v>900112</x:v>
       </x:c>
       <x:c r="B100" s="9">
-        <x:v>80060</x:v>
+        <x:v>80071</x:v>
       </x:c>
       <x:c r="C100" s="9">
         <x:v>1</x:v>
@@ -17572,21 +18516,22 @@
       </x:c>
       <x:c r="E100" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">허허, 오늘은 술 대신 물 한 잔이면 되겠어. 도구를 챙겨 올 테니, 가게 불은 꺼뜨리지 말게!</x:t>
+          <x:t xml:space="preserve">색은 &lt;color=#71508F&gt;네 감각에 맡길게.&lt;wait=0.35&gt;&lt;/color&gt;
+&lt;color=#52609B&gt;원래 뼈 색&lt;/color&gt;도 꽤 멋지거든.&lt;wait=0.35&gt; &lt;wave=1.2&gt;&lt;pulse=1.15&gt;"뼈"&lt;/pulse&gt;가 있는 색이지.&lt;/wave&gt;</x:t>
         </x:is>
       </x:c>
       <x:c r="F100" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">통합 플레이</x:t>
+          <x:t xml:space="preserve">미용 선택지 대사</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="101" ht="48" customHeight="1">
       <x:c r="A101" s="9">
-        <x:v>900101</x:v>
+        <x:v>900113</x:v>
       </x:c>
       <x:c r="B101" s="9">
-        <x:v>80061</x:v>
+        <x:v>80072</x:v>
       </x:c>
       <x:c r="C101" s="9">
         <x:v>1</x:v>
@@ -17598,24 +18543,25 @@
       </x:c>
       <x:c r="E101" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">...헤. 여기 솜씨가 좋다는 소문을 들었거든.</x:t>
+          <x:t xml:space="preserve">&lt;color=#71508F&gt;더한 뼈와 바깥 테두리&lt;/color&gt;에 마음 가는 색을 칠해 봐.&lt;wait=0.35&gt;
+&lt;color=#52609B&gt;그대로 둬도 좋아.&lt;wait=0.35&gt;&lt;/color&gt; 취향엔 정답이 없으니까. &lt;wait=0.35&gt;헤.</x:t>
         </x:is>
       </x:c>
       <x:c r="F101" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">통합 플레이</x:t>
+          <x:t xml:space="preserve">미용 선택지 대사</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="102" ht="48" customHeight="1">
       <x:c r="A102" s="9">
-        <x:v>900102</x:v>
+        <x:v>900114</x:v>
       </x:c>
       <x:c r="B102" s="9">
-        <x:v>80061</x:v>
+        <x:v>80073</x:v>
       </x:c>
       <x:c r="C102" s="9">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D102" s="4" t="inlineStr">
         <x:is>
@@ -17624,51 +18570,51 @@
       </x:c>
       <x:c r="E102" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">뼈 있는 부탁 하나 해도 될까? &lt;color=#FFD166&gt;얼굴 테두리&lt;/color&gt;만 다듬어 줘. 머리카락은... 보다시피 휴가 중이야.</x:t>
+          <x:t xml:space="preserve">&lt;color=#9A4935&gt;강해 보이는 장식 하나&lt;/color&gt;를 &lt;color=#52609B&gt;얼굴이나 머리 쪽&lt;/color&gt;에 부탁해.&lt;wait=0.35&gt;
+딱 봤을 때 &lt;shake=0.6&gt;쉽게 덤비지는 못하겠다&lt;/shake&gt; 싶은 걸로.</x:t>
         </x:is>
       </x:c>
       <x:c r="F102" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">통합 플레이</x:t>
+          <x:t xml:space="preserve">미용 선택지 대사</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="103" ht="48" customHeight="1">
       <x:c r="A103" s="9">
-        <x:v>900103</x:v>
+        <x:v>900140</x:v>
       </x:c>
       <x:c r="B103" s="9">
-        <x:v>80062</x:v>
+        <x:v>80056</x:v>
       </x:c>
       <x:c r="C103" s="9">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D103" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">몬스터</x:t>
+          <x:t xml:space="preserve">플레이어</x:t>
         </x:is>
       </x:c>
       <x:c r="E103" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">헤. 오늘은 &lt;color=#52609B&gt;인상 좀 다듬으러&lt;/color&gt; 왔어.
-&lt;color=#52609B&gt;각진 데만 가볍게.&lt;/color&gt; &lt;wave=1.3&gt;뼈대는 괜찮잖아?&lt;/wave&gt;</x:t>
+          <x:t xml:space="preserve">두들겨 맞아서 어깨 힘도 다 빠졌죠?</x:t>
         </x:is>
       </x:c>
       <x:c r="F103" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">미용 요구 · 선택지 연결</x:t>
+          <x:t xml:space="preserve">통합 개발실</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="104" ht="48" customHeight="1">
       <x:c r="A104" s="9">
-        <x:v>900104</x:v>
+        <x:v>900141</x:v>
       </x:c>
       <x:c r="B104" s="9">
-        <x:v>80063</x:v>
+        <x:v>80056</x:v>
       </x:c>
       <x:c r="C104" s="9">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D104" s="4" t="inlineStr">
         <x:is>
@@ -17677,25 +18623,24 @@
       </x:c>
       <x:c r="E104" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">이번엔 좀 &lt;color=#9A4935&gt;&lt;shake=0.6&gt;만만하지 않은 인상&lt;/shake&gt;&lt;/color&gt;이면 좋겠어.
-&lt;color=#9A4935&gt;장식&lt;/color&gt;으로 한 수 보여 줄래?</x:t>
+          <x:t xml:space="preserve">&lt;wave=1&gt;그렇네요... &lt;wait=0.35&gt;감사합니다...&lt;/wave&gt;</x:t>
         </x:is>
       </x:c>
       <x:c r="F104" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">미용 요구 · 선택지 연결</x:t>
+          <x:t xml:space="preserve">통합 개발실</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="105" ht="48" customHeight="1">
       <x:c r="A105" s="9">
-        <x:v>900105</x:v>
+        <x:v>900142</x:v>
       </x:c>
       <x:c r="B105" s="9">
-        <x:v>80064</x:v>
+        <x:v>80037</x:v>
       </x:c>
       <x:c r="C105" s="9">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D105" s="4" t="inlineStr">
         <x:is>
@@ -17704,24 +18649,24 @@
       </x:c>
       <x:c r="E105" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">헤. 꽤 뼈대 있는 실력이네. 그럼... 몸도 한번 풀어 볼까?</x:t>
+          <x:t xml:space="preserve">뭐?&lt;wait=0.5&gt; &lt;shake=1&gt;모른다고?&lt;/shake&gt;&lt;wait=0.5&gt;&lt;shake=2&gt; 어떻게 그럴 수가 있지?&lt;/shake&gt; &lt;wait=0.5&gt;와,&lt;wait=0.25&gt; &lt;wave=1.4&gt;샌즈의 &lt;color=#1900d6&gt;파란 공격&lt;/color&gt;은 말이야...&lt;/wave&gt;</x:t>
         </x:is>
       </x:c>
       <x:c r="F105" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">통합 플레이</x:t>
+          <x:t xml:space="preserve">통합 개발실</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="106" ht="48" customHeight="1">
       <x:c r="A106" s="9">
-        <x:v>900106</x:v>
+        <x:v>900143</x:v>
       </x:c>
       <x:c r="B106" s="9">
-        <x:v>80065</x:v>
+        <x:v>80037</x:v>
       </x:c>
       <x:c r="C106" s="9">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D106" s="4" t="inlineStr">
         <x:is>
@@ -17730,24 +18675,24 @@
       </x:c>
       <x:c r="E106" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">나쁘지 않네. 이번엔 다른 솜씨도 보여 줄래?</x:t>
+          <x:t xml:space="preserve">아니야, &lt;wait=0.25&gt;그냥 직접 보여줘야겠어,&lt;wait=0.25&gt; &lt;wait=0.35&gt;헤.</x:t>
         </x:is>
       </x:c>
       <x:c r="F106" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">통합 플레이</x:t>
+          <x:t xml:space="preserve">통합 개발실</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="107" ht="48" customHeight="1">
       <x:c r="A107" s="9">
-        <x:v>900107</x:v>
+        <x:v>900137</x:v>
       </x:c>
       <x:c r="B107" s="9">
-        <x:v>80066</x:v>
+        <x:v>80089</x:v>
       </x:c>
       <x:c r="C107" s="9">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D107" s="4" t="inlineStr">
         <x:is>
@@ -17756,50 +18701,50 @@
       </x:c>
       <x:c r="E107" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">...친구, 이건 좀 뼈아픈데. 잠깐 밖에서 얘기할까?</x:t>
+          <x:t xml:space="preserve">헤.&lt;wait=0.35&gt; 난 &lt;color=#ec6565&gt;그릴비&lt;/color&gt;나 가야겠군.</x:t>
         </x:is>
       </x:c>
       <x:c r="F107" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">통합 플레이</x:t>
+          <x:t xml:space="preserve">통합 개발실</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="108" ht="48" customHeight="1">
       <x:c r="A108" s="9">
-        <x:v>900108</x:v>
+        <x:v>900138</x:v>
       </x:c>
       <x:c r="B108" s="9">
-        <x:v>80067</x:v>
+        <x:v>80089</x:v>
       </x:c>
       <x:c r="C108" s="9">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D108" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">나레이션</x:t>
+          <x:t xml:space="preserve">몬스터</x:t>
         </x:is>
       </x:c>
       <x:c r="E108" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">미용실로 돌아오자, 문에 달린 종이 작게 울렸다. 오늘의 마지막 손님과의 야차가 끝났다.</x:t>
+          <x:t xml:space="preserve">크, &lt;wait=0.25&gt;크흠... &lt;wait=0.35&gt;제법인데, &lt;wait=0.25&gt;꼬마야. &lt;wave=1.4&gt;&lt;pulse=1.15&gt;"뼈"&lt;/pulse&gt;가 시리는 전투였어.&lt;/wave&gt;</x:t>
         </x:is>
       </x:c>
       <x:c r="F108" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">통합 플레이</x:t>
+          <x:t xml:space="preserve">통합 개발실</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="109" ht="48" customHeight="1">
       <x:c r="A109" s="9">
-        <x:v>900109</x:v>
+        <x:v>900139</x:v>
       </x:c>
       <x:c r="B109" s="9">
-        <x:v>80068</x:v>
+        <x:v>80001</x:v>
       </x:c>
       <x:c r="C109" s="9">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D109" s="4" t="inlineStr">
         <x:is>
@@ -17808,22 +18753,21 @@
       </x:c>
       <x:c r="E109" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">&lt;color=#71508F&gt;어떤 색이나 무늬든&lt;/color&gt; 괜찮아요...
-&lt;color=#266B4D&gt;염색하지 않아도 좋아요.&lt;/color&gt; 머리는 지금도 마음에 들어서...</x:t>
+          <x:t xml:space="preserve">&lt;wave=1&gt;주,&lt;wait=0.25&gt; 죽고 나서 면접은,&lt;wait=0.25&gt; 처음이에요...&lt;/wave&gt;</x:t>
         </x:is>
       </x:c>
       <x:c r="F109" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">미용 선택지 대사</x:t>
+          <x:t xml:space="preserve">통합 개발실</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="110" ht="48" customHeight="1">
       <x:c r="A110" s="9">
-        <x:v>900110</x:v>
+        <x:v>900115</x:v>
       </x:c>
       <x:c r="B110" s="9">
-        <x:v>80069</x:v>
+        <x:v>80074</x:v>
       </x:c>
       <x:c r="C110" s="9">
         <x:v>1</x:v>
@@ -17835,25 +18779,24 @@
       </x:c>
       <x:c r="E110" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">면접장에서 &lt;color=#9A5B22&gt;단정하고 점잖아 보일 장식&lt;/color&gt;으로...
-&lt;color=#9A5B22&gt;하나만&lt;/color&gt; 골라 주시겠어요...? &lt;wave=1.2&gt;너무 요란하진 않게요...&lt;/wave&gt;</x:t>
+          <x:t xml:space="preserve">점검은 &lt;color=#52609B&gt;손님의 부탁을 얼마나 정확히 이루어 주는지&lt;/color&gt; 보겠습니다. 제 부탁으로 시험하지요.</x:t>
         </x:is>
       </x:c>
       <x:c r="F110" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">미용 선택지 대사</x:t>
+          <x:t xml:space="preserve">중간 점검: 한 번도 승인되지 않은 반차를 외모 변화로 설득하는 과제. 로컬 검토 초안.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="111" ht="48" customHeight="1">
       <x:c r="A111" s="9">
-        <x:v>900111</x:v>
+        <x:v>900116</x:v>
       </x:c>
       <x:c r="B111" s="9">
-        <x:v>80070</x:v>
+        <x:v>80074</x:v>
       </x:c>
       <x:c r="C111" s="9">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D111" s="4" t="inlineStr">
         <x:is>
@@ -17862,25 +18805,25 @@
       </x:c>
       <x:c r="E111" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">&lt;color=#52609B&gt;얼굴 바깥 테두리만&lt;/color&gt; 망치랑 정으로 톡톡 다듬어 줘.
-&lt;color=#9A4935&gt;눈코입은 그대로.&lt;/color&gt; &lt;wave=1.2&gt;속까지 시원해질 필요는 없거든.&lt;/wave&gt;</x:t>
+          <x:t xml:space="preserve">우선 이 뿔부터입니다. 보고서는 정리했는데, 제 머리 위는 아직이군요.
+눈을 찌르면 점검표도 읽을 수 없습니다.</x:t>
         </x:is>
       </x:c>
       <x:c r="F111" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">미용 선택지 대사</x:t>
+          <x:t xml:space="preserve">중간 점검: 한 번도 승인되지 않은 반차를 외모 변화로 설득하는 과제. 로컬 검토 초안.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="112" ht="48" customHeight="1">
       <x:c r="A112" s="9">
-        <x:v>900112</x:v>
+        <x:v>900117</x:v>
       </x:c>
       <x:c r="B112" s="9">
-        <x:v>80071</x:v>
+        <x:v>80074</x:v>
       </x:c>
       <x:c r="C112" s="9">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D112" s="4" t="inlineStr">
         <x:is>
@@ -17889,22 +18832,22 @@
       </x:c>
       <x:c r="E112" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">색은 &lt;color=#71508F&gt;네 감각에 맡길게.&lt;/color&gt;
-&lt;color=#52609B&gt;원래 뼈 색&lt;/color&gt;도 꽤 멋지거든. &lt;wave=1.2&gt;뼈가 있는 색이지.&lt;/wave&gt;</x:t>
+          <x:t xml:space="preserve">&lt;color=#52609B&gt;눈 세 개는 무사하게, 뿔은 왔을 때보다 가볍게&lt;/color&gt; 부탁드립니다.
+모양은 맡기겠습니다. 정해진 답을 베끼는 시험은 아니니까요.</x:t>
         </x:is>
       </x:c>
       <x:c r="F112" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">미용 선택지 대사</x:t>
+          <x:t xml:space="preserve">중간 점검: 한 번도 승인되지 않은 반차를 외모 변화로 설득하는 과제. 로컬 검토 초안.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="113" ht="48" customHeight="1">
       <x:c r="A113" s="9">
-        <x:v>900113</x:v>
+        <x:v>900118</x:v>
       </x:c>
       <x:c r="B113" s="9">
-        <x:v>80072</x:v>
+        <x:v>80075</x:v>
       </x:c>
       <x:c r="C113" s="9">
         <x:v>1</x:v>
@@ -17916,22 +18859,22 @@
       </x:c>
       <x:c r="E113" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">&lt;color=#71508F&gt;더한 뼈와 바깥 테두리&lt;/color&gt;에 마음 가는 색을 칠해 봐.
-&lt;color=#52609B&gt;그대로 둬도 좋아.&lt;/color&gt; 취향엔 정답이 없으니까. 헤.</x:t>
+          <x:t xml:space="preserve">&lt;color=#52609B&gt;세 눈에 닿지 않게&lt;/color&gt; 뿔을 다듬어 주세요.
+모양은 자유입니다. 다만 전체 양은 처음보다 줄어야 합니다. 줄여 달랬는데 늘어나면 곤란하겠지요.</x:t>
         </x:is>
       </x:c>
       <x:c r="F113" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">미용 선택지 대사</x:t>
+          <x:t xml:space="preserve">중간 점검: 한 번도 승인되지 않은 반차를 외모 변화로 설득하는 과제. 로컬 검토 초안.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="114" ht="48" customHeight="1">
       <x:c r="A114" s="9">
-        <x:v>900114</x:v>
+        <x:v>900120</x:v>
       </x:c>
       <x:c r="B114" s="9">
-        <x:v>80073</x:v>
+        <x:v>80076</x:v>
       </x:c>
       <x:c r="C114" s="9">
         <x:v>1</x:v>
@@ -17943,18 +18886,444 @@
       </x:c>
       <x:c r="E114" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">&lt;color=#9A4935&gt;강해 보이는 장식 하나&lt;/color&gt;를 &lt;color=#52609B&gt;얼굴이나 머리 쪽&lt;/color&gt;에 부탁해.
-딱 봤을 때 &lt;shake=0.6&gt;쉽게 덤비지는 못하겠다&lt;/shake&gt; 싶은 걸로.</x:t>
+          <x:t xml:space="preserve">이제 본시험입니다. 저는 &lt;color=#52609B&gt;666년 동안 단 한 번도 반차를 승인받지 못했습니다.&lt;/color&gt; 무슨 수를 써도 “멀쩡해 보인다”시더군요.
+&lt;color=#52609B&gt;세 눈 아래 모두, 가장 어두운 색으로 다크서클&lt;/color&gt;을 만들어 주십시오. 쉬어야 한다는 말이 얼굴만 봐도 전해지도록요.</x:t>
         </x:is>
       </x:c>
       <x:c r="F114" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">미용 선택지 대사</x:t>
+          <x:t xml:space="preserve">중간 점검: 한 번도 승인되지 않은 반차를 외모 변화로 설득하는 과제. 로컬 검토 초안.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="115" ht="48" customHeight="1">
+      <x:c r="A115" s="9">
+        <x:v>900121</x:v>
+      </x:c>
+      <x:c r="B115" s="9">
+        <x:v>80077</x:v>
+      </x:c>
+      <x:c r="C115" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D115" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">몬스터</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E115" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">&lt;color=#52609B&gt;이마의 눈과 안경 쓴 두 눈, 세 눈 아래를 모두&lt;/color&gt; 짙게 해 주세요.
+눈 자체와 나머지 얼굴은 깔끔하게. 피곤한 인상을 만드는 솜씨를 보는 거지, 보고서를 못 읽게 하는 시험은 아닙니다.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F115" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">중간 점검: 한 번도 승인되지 않은 반차를 외모 변화로 설득하는 과제. 로컬 검토 초안.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="116" ht="48" customHeight="1">
+      <x:c r="A116" s="9">
+        <x:v>900122</x:v>
+      </x:c>
+      <x:c r="B116" s="9">
+        <x:v>80078</x:v>
+      </x:c>
+      <x:c r="C116" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D116" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">몬스터</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E116" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">마지막으로 &lt;color=#D94B4B&gt;코끝에 빨간 코 장식 하나&lt;/color&gt;를 붙여 주십시오.
+마왕님이 제 얼굴을 보고 먼저 “오늘은 쉬어라” 하신다면…… 그보다 확실한 실력 증명이 있겠습니까?</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F116" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">중간 점검: 한 번도 승인되지 않은 반차를 외모 변화로 설득하는 과제. 로컬 검토 초안.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="117" ht="48" customHeight="1">
+      <x:c r="A117" s="9">
+        <x:v>900123</x:v>
+      </x:c>
+      <x:c r="B117" s="9">
+        <x:v>80079</x:v>
+      </x:c>
+      <x:c r="C117" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D117" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">몬스터</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E117" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">&lt;color=#D94B4B&gt;빨간 코는 코 주변에 하나&lt;/color&gt;면 됩니다.
+아파 보이되 우스꽝스럽지는 않게. 반차 신청서이지, 궁정 축제 참가 신청서가 아닙니다.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F117" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">중간 점검: 한 번도 승인되지 않은 반차를 외모 변화로 설득하는 과제. 로컬 검토 초안.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="118" ht="48" customHeight="1">
+      <x:c r="A118" s="9">
+        <x:v>900124</x:v>
+      </x:c>
+      <x:c r="B118" s="9">
+        <x:v>80080</x:v>
+      </x:c>
+      <x:c r="C118" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D118" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">몬스터</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E118" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">실례합니다. 마왕님의 직속 부하입니다. 예고드린 &lt;color=#FFD166&gt;중간 점검&lt;/color&gt;을 하러 왔습니다.
+5일차에 마왕님을 모시려면, 별 세 개에 어울리는 솜씨를 보여 주셔야겠지요.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F118" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">중간 점검: 한 번도 승인되지 않은 반차를 외모 변화로 설득하는 과제. 로컬 검토 초안.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="119" ht="48" customHeight="1">
+      <x:c r="A119" s="9">
+        <x:v>900125</x:v>
+      </x:c>
+      <x:c r="B119" s="9">
+        <x:v>80080</x:v>
+      </x:c>
+      <x:c r="C119" s="9">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D119" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">몬스터</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E119" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">제게는 한 번도 통과하지 못한 결재가 있습니다. &lt;color=#FFD166&gt;반차 신청.&lt;/color&gt;
+저조차 포기한 부탁을 미용으로 이루어 주실 수 있습니까? 오늘은 제가 직접 손님이 되어 확인하겠습니다. 커피는…… 들고 앉아도 되겠지요?</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F119" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">중간 점검: 한 번도 승인되지 않은 반차를 외모 변화로 설득하는 과제. 로컬 검토 초안.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="120" ht="48" customHeight="1">
+      <x:c r="A120" s="9">
+        <x:v>900126</x:v>
+      </x:c>
+      <x:c r="B120" s="9">
+        <x:v>80081</x:v>
+      </x:c>
+      <x:c r="C120" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D120" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">몬스터</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E120" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">&lt;wave=1.2&gt;호오……&lt;/wave&gt; 뿔은 가볍고, 세 눈과 코는 쉬어야 한다는 말을 분명히 전하는군요.
+부탁을 알아듣고 인상을 바꾸는 솜씨, 잘 보았습니다.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F120" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">중간 점검: 한 번도 승인되지 않은 반차를 외모 변화로 설득하는 과제. 로컬 검토 초안.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="121" ht="48" customHeight="1">
+      <x:c r="A121" s="9">
+        <x:v>900127</x:v>
+      </x:c>
+      <x:c r="B121" s="9">
+        <x:v>80081</x:v>
+      </x:c>
+      <x:c r="C121" s="9">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D121" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">몬스터</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E121" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">이번에는 반차 신청서에 제 얼굴도 첨부해야겠습니다.
+중간 점검에는 좋은 평가를 남기지요. 이 솜씨로 별 세 개까지 올라오십시오.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F121" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">중간 점검: 한 번도 승인되지 않은 반차를 외모 변화로 설득하는 과제. 로컬 검토 초안.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="122" ht="48" customHeight="1">
+      <x:c r="A122" s="9">
+        <x:v>900128</x:v>
+      </x:c>
+      <x:c r="B122" s="9">
+        <x:v>80082</x:v>
+      </x:c>
+      <x:c r="C122" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D122" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">몬스터</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E122" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">음…… 의도는 전해집니다. 다만 “당장 쉬어라”보다는 “커피 한 잔 더 마셔라”에 가깝군요.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F122" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">중간 점검: 한 번도 승인되지 않은 반차를 외모 변화로 설득하는 과제. 로컬 검토 초안.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="123" ht="48" customHeight="1">
+      <x:c r="A123" s="9">
+        <x:v>900129</x:v>
+      </x:c>
+      <x:c r="B123" s="9">
+        <x:v>80082</x:v>
+      </x:c>
+      <x:c r="C123" s="9">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D123" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">몬스터</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E123" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">점검 기록에는 조금 더 다듬을 여지가 있다고 적겠습니다.
+5일차까지 손님들의 부탁을 듣고, 그 차이를 익혀 보십시오. 제 반차도 아직 포기하지 않겠습니다.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F123" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">중간 점검: 한 번도 승인되지 않은 반차를 외모 변화로 설득하는 과제. 로컬 검토 초안.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="124" ht="48" customHeight="1">
+      <x:c r="A124" s="9">
+        <x:v>900130</x:v>
+      </x:c>
+      <x:c r="B124" s="9">
+        <x:v>80083</x:v>
+      </x:c>
+      <x:c r="C124" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D124" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">몬스터</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E124" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">&lt;shake=0.8&gt;하아……&lt;/shake&gt; 반차를 설득할 얼굴을 부탁드렸는데, 설명해야 할 부분이 더 늘었군요.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F124" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">중간 점검: 한 번도 승인되지 않은 반차를 외모 변화로 설득하는 과제. 로컬 검토 초안.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="125" ht="48" customHeight="1">
+      <x:c r="A125" s="9">
+        <x:v>900131</x:v>
+      </x:c>
+      <x:c r="B125" s="9">
+        <x:v>80083</x:v>
+      </x:c>
+      <x:c r="C125" s="9">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D125" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">몬스터</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E125" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">중간 점검에는 보완이 필요하다고 남기겠습니다.
+손님이 어떤 모습이 되고 싶은지, 그 말을 놓치지 마십시오. 마왕님을 만날 때도 중요할 겁니다.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F125" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">중간 점검: 한 번도 승인되지 않은 반차를 외모 변화로 설득하는 과제. 로컬 검토 초안.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="126" ht="48" customHeight="1">
+      <x:c r="A126" s="9">
+        <x:v>900132</x:v>
+      </x:c>
+      <x:c r="B126" s="9">
+        <x:v>80084</x:v>
+      </x:c>
+      <x:c r="C126" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D126" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">몬스터</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E126" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">점검은 여기까지입니다. 보고서와 반차 신청서를 함께 올리러 가겠습니다.
+다음에 마왕님을 모시고 올 때는, &lt;color=#FFD166&gt;별 세 개&lt;/color&gt;가 걸려 있기를 기대하지요.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F126" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">중간 점검: 한 번도 승인되지 않은 반차를 외모 변화로 설득하는 과제. 로컬 검토 초안.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="127" ht="48" customHeight="1">
+      <x:c r="A127" s="9">
+        <x:v>900133</x:v>
+      </x:c>
+      <x:c r="B127" s="9">
+        <x:v>80085</x:v>
+      </x:c>
+      <x:c r="C127" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D127" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">몬스터</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E127" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">잠깐! 점검하는 눈입니다. 심사위원을 안 보이게 한다고 통과가 되는 건 아닙니다!</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F127" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">마왕 부하 · 눈에 닿았을 때 · 첫 항의</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="128" ht="48" customHeight="1">
+      <x:c r="A128" s="9">
+        <x:v>900134</x:v>
+      </x:c>
+      <x:c r="B128" s="9">
+        <x:v>80086</x:v>
+      </x:c>
+      <x:c r="C128" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D128" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">몬스터</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E128" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">하아…… 눈은 세 개지만, 재시험 기회까지 세 번인 건 아닙니다.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F128" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">마왕 부하 · 다시 눈에 닿았을 때 · 두 번째 항의</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="129" ht="48" customHeight="1">
+      <x:c r="A129" s="9">
+        <x:v>900135</x:v>
+      </x:c>
+      <x:c r="B129" s="9">
+        <x:v>80087</x:v>
+      </x:c>
+      <x:c r="C129" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D129" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">몬스터</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E129" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">잠깐…… 뿔은 줄여 달라고 말씀드렸습니다. 점검표의 줄 수를 늘릴 생각은 아니시지요?</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F129" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">마왕 부하 · 뿔을 줄인 뒤 다시 불어날 때</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="130" ht="48" customHeight="1">
+      <x:c r="A130" s="9">
+        <x:v>900136</x:v>
+      </x:c>
+      <x:c r="B130" s="9">
+        <x:v>80088</x:v>
+      </x:c>
+      <x:c r="C130" s="9">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D130" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">몬스터</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E130" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">왔을 때보다 뿔이 더 많군요. “요구 이상의 성과”라고 적기에는 방향이 반대입니다만.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F130" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">마왕 부하 · 처음보다 뿔이 더 많아졌을 때</x:t>
         </x:is>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="A2:F114">
+  <x:conditionalFormatting sqref="A2:F130">
     <x:cfRule type="expression" dxfId="16" priority="1">
       <x:formula>MOD(ROW(),2)=0</x:formula>
     </x:cfRule>
@@ -17976,5 +19345,5 @@
 </file>
 
 <file path=customXml/yachaVersion.xml><?xml version="1.0" encoding="utf-8"?>
-<version xmlns="urn:yachacha:table-version">{"format":1,"version":"2026-10-11_14-41-56","parentVersion":"2026-10-11_14-12-42","intent":"플레이어가 네?로 부탁을 더 자세히 듣거나 알겠습니다로 손질을 시작하는 흐름을 엑셀에서 관리하도록, 좀비·샌즈의 최신 미용 대사를 대사 그룹으로 옮기고 미용 대사 연결 6행을 추가. 전투·미용 점수 수치 변경 없음. 기존 80004는 미연결 보관.","snapshot":{"sheets":[{"name":"공격 만들기","keys":["PatternID","Name","RangeMode","ShapePoolID","TilePath","HitMin","HitMax","GapMinMs","GapMaxMs","ResponseMs","ExtraMinMs","ExtraMaxMs","AvoidRepeat","CanDefend","BreakTiles","Notes"],"rows":[{"PatternID":20001,"Name":"랜덤 단일","RangeMode":"범위 반복","ShapePoolID":60001,"TilePath":null,"HitMin":1,"HitMax":1,"GapMinMs":null,"GapMaxMs":null,"ResponseMs":null,"ExtraMinMs":0,"ExtraMaxMs":0,"AvoidRepeat":true,"CanDefend":true,"BreakTiles":false,"Notes":"범위 하나를 뽑아 1회 타격"},{"PatternID":30001,"Name":"랜덤 2~5연속","RangeMode":"범위 반복","ShapePoolID":60001,"TilePath":null,"HitMin":2,"HitMax":5,"GapMinMs":300,"GapMaxMs":600,"ResponseMs":null,"ExtraMinMs":0,"ExtraMaxMs":0,"AvoidRepeat":true,"CanDefend":true,"BreakTiles":false,"Notes":"모든 파란 숫자 예고 후 같은 박자로 타격"},{"PatternID":40001,"Name":"순차 타일","RangeMode":"경로 순차","ShapePoolID":70001,"TilePath":null,"HitMin":null,"HitMax":null,"GapMinMs":300,"GapMaxMs":300,"ResponseMs":null,"ExtraMinMs":0,"ExtraMaxMs":0,"AvoidRepeat":false,"CanDefend":true,"BreakTiles":false,"Notes":"경로 하나 선택 → 타일별 예고 → 모션 1회·순차 타격"},{"PatternID":20002,"Name":"엇박 단일","RangeMode":"범위 반복","ShapePoolID":60001,"TilePath":null,"HitMin":1,"HitMax":1,"GapMinMs":null,"GapMaxMs":null,"ResponseMs":null,"ExtraMinMs":500,"ExtraMaxMs":500,"AvoidRepeat":true,"CanDefend":true,"BreakTiles":false,"Notes":"단일 공격에 500ms 추가 대기"},{"PatternID":20003,"Name":"방어 불가 · 전체 타일 제외","RangeMode":"범위 반복","ShapePoolID":60003,"TilePath":null,"HitMin":1,"HitMax":1,"GapMinMs":null,"GapMaxMs":null,"ResponseMs":null,"ExtraMinMs":0,"ExtraMaxMs":0,"AvoidRepeat":true,"CanDefend":false,"BreakTiles":false,"Notes":"후보 1~8 사용. 전체 9칸 동시 공격 제외. 패링·가드 불가"},{"PatternID":20010,"Name":"타일 파괴 단일","RangeMode":"범위 반복","ShapePoolID":60001,"TilePath":null,"HitMin":1,"HitMax":1,"GapMinMs":null,"GapMaxMs":null,"ResponseMs":null,"ExtraMinMs":0,"ExtraMaxMs":0,"AvoidRepeat":true,"CanDefend":true,"BreakTiles":true,"Notes":"기능 예시. 이 속성은 다른 공격에도 켤 수 있음"},{"PatternID":40002,"Name":"ㄹ자 9칸 순차","RangeMode":"경로 순차","ShapePoolID":null,"TilePath":"1,4,7,8,5,2,3,6,9","HitMin":null,"HitMax":null,"GapMinMs":300,"GapMaxMs":300,"ResponseMs":null,"ExtraMinMs":0,"ExtraMaxMs":0,"AvoidRepeat":false,"CanDefend":true,"BreakTiles":false,"Notes":"경로만 입력. 9타 자동 결정"},{"PatternID":40003,"Name":"대각선 3칸 순차","RangeMode":"경로 순차","ShapePoolID":null,"TilePath":"1,5,9","HitMin":null,"HitMax":null,"GapMinMs":300,"GapMaxMs":300,"ResponseMs":null,"ExtraMinMs":0,"ExtraMaxMs":0,"AvoidRepeat":false,"CanDefend":true,"BreakTiles":false,"Notes":"1→5→9 예고 완료 후 연속 타격"},{"PatternID":50001,"Name":"샌즈 상대 밀치기","RangeMode":"밀친 위치","ShapePoolID":null,"TilePath":null,"HitMin":null,"HitMax":null,"GapMinMs":null,"GapMaxMs":null,"ResponseMs":550,"ExtraMinMs":0,"ExtraMaxMs":0,"AvoidRepeat":false,"CanDefend":true,"BreakTiles":false,"Notes":"방향·시간은 이동·연출에 작성. 수치·방어 임시"},{"PatternID":20020,"Name":"샌즈 블래스터","RangeMode":"범위 반복","ShapePoolID":60001,"TilePath":null,"HitMin":1,"HitMax":1,"GapMinMs":null,"GapMaxMs":null,"ResponseMs":null,"ExtraMinMs":0,"ExtraMaxMs":0,"AvoidRepeat":true,"CanDefend":true,"BreakTiles":false,"Notes":"랜덤 단일 + 이동 없음 + 레이저 연출. 타격 1회"},{"PatternID":30002,"Name":"랜덤 2~3연속","RangeMode":"범위 반복","ShapePoolID":60001,"TilePath":null,"HitMin":2,"HitMax":3,"GapMinMs":300,"GapMaxMs":600,"ResponseMs":null,"ExtraMinMs":0,"ExtraMaxMs":0,"AvoidRepeat":true,"CanDefend":true,"BreakTiles":false,"Notes":"초반 몬스터용 예시. 30001 복사 후 횟수만 변경."},{"PatternID":30003,"Name":"랜덤 4~5연속","RangeMode":"범위 반복","ShapePoolID":60001,"TilePath":null,"HitMin":4,"HitMax":5,"GapMinMs":300,"GapMaxMs":600,"ResponseMs":null,"ExtraMinMs":0,"ExtraMaxMs":0,"AvoidRepeat":true,"CanDefend":true,"BreakTiles":false,"Notes":"후반 몬스터용 예시. 별도 ID로 독립 참조."},{"PatternID":20004,"Name":"단일 · 후보 1~4","RangeMode":"범위 반복","ShapePoolID":60002,"TilePath":null,"HitMin":1,"HitMax":1,"GapMinMs":null,"GapMaxMs":null,"ResponseMs":null,"ExtraMinMs":0,"ExtraMaxMs":0,"AvoidRepeat":true,"CanDefend":true,"BreakTiles":false,"Notes":"20001과 같은 단일, 범위 풀만 60002로 변경."},{"PatternID":20011,"Name":"느긋한 엇박 단일","RangeMode":"범위 반복","ShapePoolID":60001,"TilePath":null,"HitMin":1,"HitMax":1,"GapMinMs":null,"GapMaxMs":null,"ResponseMs":882,"ExtraMinMs":588,"ExtraMaxMs":588,"AvoidRepeat":true,"CanDefend":true,"BreakTiles":false,"Notes":"기존 엇박의 시간만 다른 변형. 필요한 몬스터·페이즈에서 재사용하세요."},{"PatternID":20012,"Name":"빠른 엇박 단일","RangeMode":"범위 반복","ShapePoolID":60001,"TilePath":null,"HitMin":1,"HitMax":1,"GapMinMs":null,"GapMaxMs":null,"ResponseMs":652,"ExtraMinMs":435,"ExtraMaxMs":435,"AvoidRepeat":true,"CanDefend":true,"BreakTiles":false,"Notes":"기존 엇박의 시간만 다른 변형. 필요한 몬스터·페이즈에서 재사용하세요."},{"PatternID":20013,"Name":"더 빠른 엇박 단일","RangeMode":"범위 반복","ShapePoolID":60001,"TilePath":null,"HitMin":1,"HitMax":1,"GapMinMs":null,"GapMaxMs":null,"ResponseMs":577,"ExtraMinMs":385,"ExtraMaxMs":385,"AvoidRepeat":true,"CanDefend":true,"BreakTiles":false,"Notes":"기존 엇박의 시간만 다른 변형. 필요한 몬스터·페이즈에서 재사용하세요."}]},{"name":"이동·연출","keys":["PatternID","PatternName","MoveType","MoveSpeed","MoveDistance","MotionKey","Effect","SoundKey","EffectMs","PushDirection","PushTiles","PushLeadMs","PushMoveMs","Notes"],"rows":[{"PatternID":50001,"PatternName":"샌즈 상대 밀치기","MoveType":"없음","MoveSpeed":null,"MoveDistance":null,"MotionKey":null,"Effect":"기본","SoundKey":null,"EffectMs":null,"PushDirection":"좌우 무작위","PushTiles":1,"PushLeadMs":300,"PushMoveMs":150,"Notes":"예고 300 + 강제이동 150 + 탈출 550ms. 임시값."},{"PatternID":20020,"PatternName":"샌즈 블래스터","MoveType":"없음","MoveSpeed":null,"MoveDistance":null,"MotionKey":null,"Effect":"블래스터 레이저","SoundKey":null,"EffectMs":500,"PushDirection":null,"PushTiles":null,"PushLeadMs":null,"PushMoveMs":null,"Notes":"모션·소리·레이저 프리셋 연결 필요. 표시 500ms 임시."}]},{"name":"몬스터 사용 패턴","keys":["MonsterID","Name","PhaseID","PatternID","PatternName","HitDamage","Weight","Enabled","Notes"],"rows":[{"MonsterID":10001,"Name":"취준좀비","PhaseID":1,"PatternID":20001,"PatternName":"랜덤 단일","HitDamage":20,"Weight":70,"Enabled":true,"Notes":"단일 공격: 70"},{"MonsterID":10001,"Name":"취준좀비","PhaseID":1,"PatternID":40001,"PatternName":"순차 타일","HitDamage":20,"Weight":30,"Enabled":true,"Notes":"순차 공격: 30"},{"MonsterID":10001,"Name":"취준좀비","PhaseID":2,"PatternID":20001,"PatternName":"랜덤 단일","HitDamage":20,"Weight":60,"Enabled":true,"Notes":"단일 공격: 60"},{"MonsterID":10001,"Name":"취준좀비","PhaseID":2,"PatternID":40001,"PatternName":"순차 타일","HitDamage":20,"Weight":40,"Enabled":true,"Notes":"순차 공격: 40"},{"MonsterID":10002,"Name":"취객","PhaseID":1,"PatternID":20001,"PatternName":"랜덤 단일","HitDamage":1,"Weight":40,"Enabled":true,"Notes":"단일 공격: 40"},{"MonsterID":10002,"Name":"취객","PhaseID":1,"PatternID":20011,"PatternName":"느긋한 엇박 단일","HitDamage":1,"Weight":60,"Enabled":true,"Notes":"술 깨기 1/4. 기존 패턴의 피할 시간·엇박 추가 시간으로 속도 조절."},{"MonsterID":10002,"Name":"취객","PhaseID":2,"PatternID":20001,"PatternName":"랜덤 단일","HitDamage":1,"Weight":40,"Enabled":true,"Notes":"단일 공격: 40"},{"MonsterID":10002,"Name":"취객","PhaseID":2,"PatternID":20002,"PatternName":"엇박 단일","HitDamage":1,"Weight":60,"Enabled":true,"Notes":"술 깨기 2/4. 기존 패턴의 피할 시간·엇박 추가 시간으로 속도 조절."},{"MonsterID":10002,"Name":"취객","PhaseID":3,"PatternID":20001,"PatternName":"랜덤 단일","HitDamage":1,"Weight":40,"Enabled":true,"Notes":"단일 공격: 40"},{"MonsterID":10002,"Name":"취객","PhaseID":3,"PatternID":20012,"PatternName":"빠른 엇박 단일","HitDamage":1,"Weight":60,"Enabled":true,"Notes":"술 깨기 3/4. 기존 패턴의 피할 시간·엇박 추가 시간으로 속도 조절."},{"MonsterID":10002,"Name":"취객","PhaseID":4,"PatternID":20001,"PatternName":"랜덤 단일","HitDamage":1,"Weight":40,"Enabled":true,"Notes":"단일 공격: 40"},{"MonsterID":10002,"Name":"취객","PhaseID":4,"PatternID":20013,"PatternName":"더 빠른 엇박 단일","HitDamage":1,"Weight":60,"Enabled":true,"Notes":"술 깨기 4/4. 기존 패턴의 피할 시간·엇박 추가 시간으로 속도 조절."},{"MonsterID":10003,"Name":"샌즈","PhaseID":1,"PatternID":50001,"PatternName":"샌즈 상대 밀치기","HitDamage":20,"Weight":50,"Enabled":true,"Notes":"대사 진행 시험용 초기값: 밀치기/블래스터 각 50, 피해 20. 조절 가능."},{"MonsterID":10001,"Name":"취준좀비","PhaseID":1,"PatternID":40003,"PatternName":"대각선 3칸 순차","HitDamage":20,"Weight":0,"Enabled":false,"Notes":"1→5→9 예시. 기존 70:30 비중 유지 위해 비활성."},{"MonsterID":10003,"Name":"샌즈","PhaseID":1,"PatternID":20020,"PatternName":"샌즈 블래스터","HitDamage":20,"Weight":50,"Enabled":true,"Notes":"대사 진행 시험용 초기값: 밀치기/블래스터 각 50, 피해 20. 조절 가능."},{"MonsterID":10001,"Name":"취준좀비","PhaseID":1,"PatternID":30002,"PatternName":"랜덤 2~3연속","HitDamage":20,"Weight":0,"Enabled":false,"Notes":"연결 예시: 초반 2~3연속. 활성 비중은 유지."},{"MonsterID":10001,"Name":"취준좀비","PhaseID":2,"PatternID":30003,"PatternName":"랜덤 4~5연속","HitDamage":20,"Weight":0,"Enabled":false,"Notes":"연결 예시: 후반 4~5연속. 필요하면 켜고 비중 입력."},{"MonsterID":10001,"Name":"취준좀비","PhaseID":1,"PatternID":20004,"PatternName":"단일 · 후보 1~4","HitDamage":20,"Weight":0,"Enabled":false,"Notes":"연결 예시: 후보 1~4 풀 사용. 필요할 때 활성화."},{"MonsterID":10003,"Name":"샌즈","PhaseID":2,"PatternID":50001,"PatternName":"샌즈 상대 밀치기","HitDamage":20,"Weight":50,"Enabled":true,"Notes":"대사 진행 시험용 초기값: 밀치기/블래스터 각 50, 피해 20. 조절 가능."},{"MonsterID":10003,"Name":"샌즈","PhaseID":2,"PatternID":20020,"PatternName":"샌즈 블래스터","HitDamage":20,"Weight":50,"Enabled":true,"Notes":"대사 진행 시험용 초기값: 밀치기/블래스터 각 50, 피해 20. 조절 가능."},{"MonsterID":10003,"Name":"샌즈","PhaseID":3,"PatternID":50001,"PatternName":"샌즈 상대 밀치기","HitDamage":20,"Weight":50,"Enabled":true,"Notes":"대사 진행 시험용 초기값: 밀치기/블래스터 각 50, 피해 20. 조절 가능."},{"MonsterID":10003,"Name":"샌즈","PhaseID":3,"PatternID":20020,"PatternName":"샌즈 블래스터","HitDamage":20,"Weight":50,"Enabled":true,"Notes":"대사 진행 시험용 초기값: 밀치기/블래스터 각 50, 피해 20. 조절 가능."}]},{"name":"몬스터 페이즈","keys":["MonsterID","Name","PhaseID","IsInitial","MaxHP","GaugeMax","ParryGain","GuardGain","DodgeGain","RecoveryMs","AttackSpeed","TransitionTrigger","NextPhaseID","PlayerDodgeMissCount","EntryDialogueGroupID","PauseForEntryDialogue","DesignStatus","OpeningDamageDisplay"],"rows":[{"MonsterID":10001,"Name":"취준좀비","PhaseID":1,"IsInitial":true,"MaxHP":1000,"GaugeMax":100,"ParryGain":50,"GuardGain":0,"DodgeGain":15,"RecoveryMs":800,"AttackSpeed":1,"TransitionTrigger":"HP 0","NextPhaseID":2,"PlayerDodgeMissCount":0,"EntryDialogueGroupID":null,"PauseForEntryDialogue":true,"DesignStatus":"페이즈 규칙 확정·수치 임시","OpeningDamageDisplay":null},{"MonsterID":10001,"Name":"취준좀비","PhaseID":2,"IsInitial":false,"MaxHP":300,"GaugeMax":100,"ParryGain":50,"GuardGain":0,"DodgeGain":15,"RecoveryMs":800,"AttackSpeed":1.5,"TransitionTrigger":"없음","NextPhaseID":null,"PlayerDodgeMissCount":0,"EntryDialogueGroupID":80051,"PauseForEntryDialogue":true,"DesignStatus":"HP 300 부활. 실제 부활 모션이 끝난 뒤 유머 대사, 입력 후 전투 재개.","OpeningDamageDisplay":null},{"MonsterID":10002,"Name":"취객","PhaseID":1,"IsInitial":true,"MaxHP":750,"GaugeMax":100,"ParryGain":50,"GuardGain":0,"DodgeGain":15,"RecoveryMs":1000,"AttackSpeed":1,"TransitionTrigger":"빈틈공격 성공","NextPhaseID":2,"PlayerDodgeMissCount":0,"EntryDialogueGroupID":null,"PauseForEntryDialogue":false,"DesignStatus":"술 깨기 1/4. 단계당 HP 750. 명중한 빈틈 종료 → 대사 → 다음 페이즈. 엇박 20011.","OpeningDamageDisplay":null},{"MonsterID":10002,"Name":"취객","PhaseID":2,"IsInitial":false,"MaxHP":750,"GaugeMax":100,"ParryGain":50,"GuardGain":0,"DodgeGain":15,"RecoveryMs":1000,"AttackSpeed":1,"TransitionTrigger":"빈틈공격 성공","NextPhaseID":3,"PlayerDodgeMissCount":0,"EntryDialogueGroupID":null,"PauseForEntryDialogue":false,"DesignStatus":"술 깨기 2/4. 단계당 HP 750. 명중한 빈틈 종료 → 대사 → 다음 페이즈. 엇박 20002.","OpeningDamageDisplay":null},{"MonsterID":10002,"Name":"취객","PhaseID":3,"IsInitial":false,"MaxHP":750,"GaugeMax":100,"ParryGain":50,"GuardGain":0,"DodgeGain":15,"RecoveryMs":1000,"AttackSpeed":1,"TransitionTrigger":"빈틈공격 성공","NextPhaseID":4,"PlayerDodgeMissCount":0,"EntryDialogueGroupID":null,"PauseForEntryDialogue":false,"DesignStatus":"술 깨기 3/4. 단계당 HP 750. 명중한 빈틈 종료 → 대사 → 다음 페이즈. 엇박 20012.","OpeningDamageDisplay":null},{"MonsterID":10002,"Name":"취객","PhaseID":4,"IsInitial":false,"MaxHP":750,"GaugeMax":100,"ParryGain":50,"GuardGain":0,"DodgeGain":15,"RecoveryMs":1000,"AttackSpeed":1,"TransitionTrigger":"빈틈공격 성공","NextPhaseID":null,"PlayerDodgeMissCount":0,"EntryDialogueGroupID":null,"PauseForEntryDialogue":false,"DesignStatus":"술 깨기 4/4. 단계당 HP 750. 명중한 빈틈 종료 → 대사 → 전투 승리. 엇박 20013.","OpeningDamageDisplay":null},{"MonsterID":10003,"Name":"샌즈","PhaseID":1,"IsInitial":true,"MaxHP":1,"GaugeMax":100,"ParryGain":50,"GuardGain":0,"DodgeGain":15,"RecoveryMs":800,"AttackSpeed":1,"TransitionTrigger":"HP 0","NextPhaseID":2,"PlayerDodgeMissCount":1,"EntryDialogueGroupID":null,"PauseForEntryDialogue":true,"DesignStatus":"첫 빈틈의 첫 MISS부터 대사(정지 없음). 다음 빈틈은 999999 연타 표시, 종료 후 명중 대사·전환.","OpeningDamageDisplay":999999},{"MonsterID":10003,"Name":"샌즈","PhaseID":2,"IsInitial":false,"MaxHP":1,"GaugeMax":100,"ParryGain":50,"GuardGain":0,"DodgeGain":15,"RecoveryMs":750,"AttackSpeed":1.2,"TransitionTrigger":"HP 0","NextPhaseID":3,"PlayerDodgeMissCount":1,"EntryDialogueGroupID":null,"PauseForEntryDialogue":true,"DesignStatus":"첫 빈틈의 첫 MISS부터 대사(정지 없음). 다음 빈틈은 999999 연타 표시, 종료 후 명중 대사·전환.","OpeningDamageDisplay":999999},{"MonsterID":10003,"Name":"샌즈","PhaseID":3,"IsInitial":false,"MaxHP":1,"GaugeMax":100,"ParryGain":50,"GuardGain":0,"DodgeGain":15,"RecoveryMs":700,"AttackSpeed":1.5,"TransitionTrigger":"HP 0","NextPhaseID":null,"PlayerDodgeMissCount":1,"EntryDialogueGroupID":null,"PauseForEntryDialogue":false,"DesignStatus":"첫 빈틈의 첫 MISS부터 대사(정지 없음). 다음 빈틈은 999999 연타 표시, 종료 후 명중 대사·전환.","OpeningDamageDisplay":999999},{"MonsterID":10100,"Name":"마왕","PhaseID":1,"IsInitial":true,"MaxHP":null,"GaugeMax":null,"ParryGain":null,"GuardGain":null,"DodgeGain":null,"RecoveryMs":null,"AttackSpeed":null,"TransitionTrigger":"미정","NextPhaseID":2,"PlayerDodgeMissCount":0,"EntryDialogueGroupID":null,"PauseForEntryDialogue":true,"DesignStatus":"전환 조건·HP·패턴 미정","OpeningDamageDisplay":null},{"MonsterID":10100,"Name":"마왕","PhaseID":2,"IsInitial":false,"MaxHP":null,"GaugeMax":null,"ParryGain":null,"GuardGain":null,"DodgeGain":null,"RecoveryMs":null,"AttackSpeed":null,"TransitionTrigger":"미정","NextPhaseID":3,"PlayerDodgeMissCount":0,"EntryDialogueGroupID":null,"PauseForEntryDialogue":true,"DesignStatus":"전환 조건·HP·패턴 미정","OpeningDamageDisplay":null},{"MonsterID":10100,"Name":"마왕","PhaseID":3,"IsInitial":false,"MaxHP":null,"GaugeMax":null,"ParryGain":null,"GuardGain":null,"DodgeGain":null,"RecoveryMs":null,"AttackSpeed":null,"TransitionTrigger":"없음","NextPhaseID":null,"PlayerDodgeMissCount":0,"EntryDialogueGroupID":null,"PauseForEntryDialogue":true,"DesignStatus":"전환 조건·HP·패턴 미정","OpeningDamageDisplay":null}]},{"name":"범위 풀","keys":["ShapePoolID","Candidate","SelectMode","Tiles","Weight","Enabled","Notes"],"rows":[{"ShapePoolID":60001,"Candidate":1,"SelectMode":"플레이어 행","Tiles":null,"Weight":25,"Enabled":true,"Notes":"현재 플레이어 행에 맞는 1개 선택"},{"ShapePoolID":60001,"Candidate":2,"SelectMode":"플레이어 열","Tiles":null,"Weight":25,"Enabled":true,"Notes":"현재 플레이어 열에 맞는 1개 선택"},{"ShapePoolID":60001,"Candidate":3,"SelectMode":"직접 입력","Tiles":"1,2,4,5","Weight":5,"Enabled":true,"Notes":"사각형"},{"ShapePoolID":60001,"Candidate":4,"SelectMode":"직접 입력","Tiles":"2,3,5,6","Weight":5,"Enabled":true,"Notes":"사각형"},{"ShapePoolID":60001,"Candidate":5,"SelectMode":"직접 입력","Tiles":"4,5,7,8","Weight":5,"Enabled":true,"Notes":"사각형"},{"ShapePoolID":60001,"Candidate":6,"SelectMode":"직접 입력","Tiles":"5,6,8,9","Weight":5,"Enabled":true,"Notes":"사각형"},{"ShapePoolID":60001,"Candidate":7,"SelectMode":"직접 입력","Tiles":"2,4,5,6,8","Weight":10,"Enabled":true,"Notes":"십자선"},{"ShapePoolID":60001,"Candidate":8,"SelectMode":"직접 입력","Tiles":"1,3,5,7,9","Weight":10,"Enabled":true,"Notes":"X자"},{"ShapePoolID":60001,"Candidate":9,"SelectMode":"직접 입력","Tiles":"1,2,3,4,5,6,7,8,9","Weight":10,"Enabled":true,"Notes":"타일 전체"},{"ShapePoolID":60002,"Candidate":1,"SelectMode":"플레이어 행","Tiles":null,"Weight":25,"Enabled":true,"Notes":"현재 플레이어 행에 맞는 1개 선택"},{"ShapePoolID":60002,"Candidate":2,"SelectMode":"플레이어 열","Tiles":null,"Weight":25,"Enabled":true,"Notes":"현재 플레이어 열에 맞는 1개 선택"},{"ShapePoolID":60002,"Candidate":3,"SelectMode":"직접 입력","Tiles":"1,2,4,5","Weight":5,"Enabled":true,"Notes":"사각형"},{"ShapePoolID":60002,"Candidate":4,"SelectMode":"직접 입력","Tiles":"2,3,5,6","Weight":5,"Enabled":true,"Notes":"사각형"},{"ShapePoolID":70001,"Candidate":1,"SelectMode":"플레이어 행","Tiles":null,"Weight":33,"Enabled":true,"Notes":"현재 플레이어 행 선택"},{"ShapePoolID":70001,"Candidate":2,"SelectMode":"플레이어 열","Tiles":null,"Weight":33,"Enabled":true,"Notes":"현재 플레이어 열 선택"},{"ShapePoolID":70001,"Candidate":3,"SelectMode":"직접 입력","Tiles":"3,5,7","Weight":17,"Enabled":true,"Notes":"대각선"},{"ShapePoolID":70001,"Candidate":4,"SelectMode":"직접 입력","Tiles":"1,5,9","Weight":17,"Enabled":true,"Notes":"대각선"},{"ShapePoolID":60003,"Candidate":1,"SelectMode":"플레이어 행","Tiles":null,"Weight":25,"Enabled":true,"Notes":"현재 플레이어 행에 맞는 1개 선택"},{"ShapePoolID":60003,"Candidate":2,"SelectMode":"플레이어 열","Tiles":null,"Weight":25,"Enabled":true,"Notes":"현재 플레이어 열에 맞는 1개 선택"},{"ShapePoolID":60003,"Candidate":3,"SelectMode":"직접 입력","Tiles":"1,2,4,5","Weight":5,"Enabled":true,"Notes":"사각형"},{"ShapePoolID":60003,"Candidate":4,"SelectMode":"직접 입력","Tiles":"2,3,5,6","Weight":5,"Enabled":true,"Notes":"사각형"},{"ShapePoolID":60003,"Candidate":5,"SelectMode":"직접 입력","Tiles":"4,5,7,8","Weight":5,"Enabled":true,"Notes":"사각형"},{"ShapePoolID":60003,"Candidate":6,"SelectMode":"직접 입력","Tiles":"5,6,8,9","Weight":5,"Enabled":true,"Notes":"사각형"},{"ShapePoolID":60003,"Candidate":7,"SelectMode":"직접 입력","Tiles":"2,4,5,6,8","Weight":10,"Enabled":true,"Notes":"십자선"},{"ShapePoolID":60003,"Candidate":8,"SelectMode":"직접 입력","Tiles":"1,3,5,7,9","Weight":10,"Enabled":true,"Notes":"X자"}]},{"name":"플레이어","keys":["PlayerID","Name","MaxHP","DodgeDamage","GuardMax","ParryMs","GuardHitCost","GuardHoldPerSec","GuardRegenPerSec","GuardBreakSec"],"rows":[{"PlayerID":1,"Name":"주인공","MaxHP":100,"DodgeDamage":30,"GuardMax":100,"ParryMs":200,"GuardHitCost":40,"GuardHoldPerSec":40,"GuardRegenPerSec":30,"GuardBreakSec":2}]},{"name":"공통 규칙","keys":["RuleID","Value","Description"],"rows":[{"RuleID":"DefaultResponseMs","Value":"750","Description":"공격 만들기의 피할 시간이 빈칸이면 750ms."},{"RuleID":"DefaultGapMinMs","Value":"300","Description":"예고 간격 최소가 빈칸이면 300ms."},{"RuleID":"DefaultGapMaxMs","Value":"600","Description":"예고 간격 최대가 빈칸이면 600ms."},{"RuleID":"DefaultPushLeadMs","Value":"300","Description":"밀기 전 예고가 빈칸이면 300ms. 임시."},{"RuleID":"DefaultPushMoveMs","Value":"150","Description":"밀려나는 시간이 빈칸이면 150ms. 임시."},{"RuleID":"AoeExtraResponseMs","Value":"200","Description":"선택된 범위 중 전체 9칸 동시 타격이 하나라도 있으면 반응 여유 200ms 추가. 경로 순차 9타에는 미적용. FFF 원본 기준."},{"RuleID":"TileRestoreSec","Value":"6","Description":"타일 파괴 후 이동 불가. 6초 뒤 복구. 공격속도 배율 제외."},{"RuleID":"GroggyDrainPerSec","Value":"30","Description":"빈틈 공격 중 게이지 초당 감소. 기존값."},{"RuleID":"PostGroggyLockMs","Value":"500","Description":"빈틈 종료 후 공격 제한. 기존값."},{"RuleID":"PushBoundary","Value":"반대쪽 확인 후 취소","Description":"예정 목적지가 경계 밖·파괴 타일이면 반대쪽 같은 거리 확인. 둘 다 불가하면 패턴 취소 후 공격 후 대기. 임시."},{"RuleID":"PushInput","Value":"이동 종료 후 허용","Description":"강제 이동 중 기본 이동 중지. 대기 입력 예약 없이 종료부터 방향키 이동 허용. 강제 이동은 회피 성공으로 세지 않음. 임시."},{"RuleID":"PhaseOrder","Value":"전환 우선","Description":"HP 0이면 다음 페이즈 확인 후 전환, 없으면 승리. 페이즈 진입 HP=MaxHP. 미정 전환은 실행 전 확정."},{"RuleID":"CombatPause","Value":"전투 시간만 정지","Description":"대화로 전투 정지 시 공격·이동·게이지·복구 시간 정지. 대화 넘김은 진행."}]},{"name":"작성 안내","keys":["Group","Topic","Description"],"rows":[{"Group":"시작","Topic":"공격 만들기부터","Description":"비슷한 공격 행을 복사하고 ID·이름을 바꾼 뒤 필요한 값만 수정하세요. 빈칸은 기본값, 회색칸은 해당 방식에서 사용하지 않는 칸입니다."},{"Group":"순서","Topic":"공격 → 몬스터 연결","Description":"공격을 만든 뒤 몬스터 사용 패턴에서 MonsterID·PhaseID·PatternID를 연결하고 피해·비중·사용을 설정하세요."},{"Group":"메모","Topic":"컬럼 제목 설명","Description":"한글 제목(2행)과 영문 이름(3행)에 설명과 예시가 있습니다. Excel의 메모/댓글 표시로 읽을 수 있습니다."},{"Group":"예시","Topic":"단일 또는 1~5연속","Description":"범위 반복에서 최소=최대=1은 단일. 최소=1, 최대=5면 매번 1~5회. 행을 추가할 필요가 없습니다."},{"Group":"예시","Topic":"FFF 연속 공격","Description":"30001은 최소2·최대5, 30002는2~3회, 30003은4~5회입니다. 선택한 횟수만큼 모두 예고한 뒤 같은 범위를 같은 박자로 타격합니다."},{"Group":"예시","Topic":"순차 공격","Description":"경로 순차에서 1,5,9를 입력하면 3타, 1,4,7,8,5,2,3,6,9면 9타입니다. 경로를 풀에서 고를 수도 있어요. 모션은 공격 구간에 한 번입니다."},{"Group":"예시","Topic":"엇박·특성 조합","Description":"타일 파괴와 방어 가능은 어떤 공격에도 적용됩니다. 엇박 추가 대기를 넣으면 같은 공격을 늦은 박자로 바꿀 수 있습니다."},{"Group":"예시","Topic":"샌즈 블래스터","Description":"공격 규칙은 범위 반복 1회. 이동·연출에서 이동 없음과 블래스터 레이저를 선택. 이펙트가 남아 있어도 피해는 한 번입니다."},{"Group":"예시","Topic":"샌즈 밀치기","Description":"공격 방식=밀친 위치. 이동·연출에서 좌우 무작위·1칸. 현재 위치로 목적지 계산 → 예고 → 밀기 → 탈출 시간 → 저장 목적지 타격."},{"Group":"입력","Topic":"반복·경로·밀친 위치","Description":"반복은 풀 필수·횟수1~5. 경로는 풀 또는 직접 경로 중 하나만. 밀친 위치는 풀·경로·횟수를 쓰지 않고 이동·연출 설정이 필수입니다."},{"Group":"입력","Topic":"모든 예고가 먼저","Description":"이번 버전은 전체 예고 후 공격으로 통일했습니다. 매 예고 직후 한 번씩 때리는 방식이 필요하면 별도 동작 규칙을 합의해야 합니다."},{"Group":"입력","Topic":"별도 연출 행은 선택","Description":"이동·연출에 없는 패턴은 이동 없음·몬스터 기본 모션·기본 이펙트와 소리입니다. 특수한 공격만 같은 PatternID로 추가합니다."},{"Group":"시간","Topic":"예고와 타격의 박자","Description":"예고를 0·450·900ms에 보여주고 피할 시간이750이면 타격은1650·2100·2550ms입니다. 서로 다른 간격이면 그 차이를 그대로 복사합니다."},{"Group":"시간","Topic":"속도 조절은 한 배율","Description":"몬스터 페이즈 AttackSpeed로 모든 패턴 시간을 나누고 모션 속도에는 곱합니다. 타일복구·패링시간·공통 빈틈 규칙은 배율 제외."},{"Group":"시간","Topic":"엇박·전체 범위","Description":"추가 대기는 이번 실행에서 한 번 뽑아 모든 타격에 똑같이 더합니다. 전체 9칸 동시 범위가 있으면 공통 여유 200ms도 한 번 더합니다."},{"Group":"샌즈","Topic":"실시간 기준의 뜻","Description":"예고 직전 현재 플레이어 위치를 한 번 읽고 목적지를 저장합니다. 예고 후 이동해도 목적지를 바꾸지 않으며 밀기와 HIT는 같은 타일을 사용합니다."},{"Group":"샌즈","Topic":"경계·파괴 처리","Description":"밀 목적지 불가 → 반대쪽 확인 → 양쪽 불가면 취소. 밀기 시작 전 목적지가 새로 파괴돼도 재선택 없이 취소. 목적지까지 보간 이동하는 초안입니다."},{"Group":"샌즈","Topic":"탈출 시간","Description":"예고300 + 강제이동150 + 피할시간550 = 첫 타격1000ms. 강제 이동 후 입력 허용. 시간과 방어 허용은 임시이며 조정 가능합니다."},{"Group":"실행","Topic":"범위 선택 시점","Description":"반복 공격은 시작 때 모든 범위를 저장합니다. 플레이어 행·열도 그때의 위치 기준. 한 번 예고한 범위를 HIT 직전에 다시 뽑지 않습니다."},{"Group":"실행","Topic":"같은 범위 금지","Description":"같은 타일 집합이면 같은 범위로 봅니다. 직전과 다른 유효 후보에서 비중으로 선택. 후보가 하나뿐이면 반복 허용하며 무한 재추첨하지 않습니다."},{"Group":"실행","Topic":"예고 표시","Description":"범위 반복이 실제2타 이상이면 파란 숫자 N→1. 1타면 기본 예고. 경로 순차는 경로 순서 예고. 연속 예고 표시는 다음 예고가 나오면 교체하지만 선택 범위는 유지합니다."},{"Group":"실행","Topic":"모션·이동 동기화","Description":"한 패턴에 공격 모션 한 번. 실제 클립과 타격 시점의 동기화는 에디터에서 연결합니다. 대상 이동 목적지는 모션 시작 때 고정. 이동 완료가 타격보다 늦으면 이동은 첫 타격 시점에 종료하는 초안입니다."},{"Group":"실행","Topic":"패턴 종료·중단","Description":"마지막 타격·모션·이동이 끝나면 몬스터의 공격 후 대기를 적용. 빈틈·페이즈 전환·전투 종료로 중단되면 남은 예고와 타격, 저장 범위를 모두 폐기합니다."},{"Group":"페이즈","Topic":"샌즈와 초기 MISS","Description":"첫 N번 빈틈 기회 전체를 MISS 처리. 실제 피해로 HP0이 되면 다음 페이즈 확인. 페이즈 전환 또는 최종 승리는 해당 빈틈 기회 종료 때 적용합니다."},{"Group":"피해","Topic":"피해 0과 타일 파괴","Description":"HitDamage=0이면 MISS·피해0이며 가드 소모·빈틈 증가 없음. 타일 파괴는 독립. 파괴된 타일 재타격은 피해·복구시간 갱신 없이 건너뜁니다."},{"Group":"데이터","Topic":"기존 수치 유지","Description":"몬스터9개 페이즈, 플레이어, 기존 활성 패턴6행의 피해·비중 유지. 취객 피해1도 원본 그대로. 샌즈 예시와 대각선 예시는 사용 끄기."},{"Group":"데이터","Topic":"미정 항목","Description":"마왕 HP·게이지·속도·대사와 샌즈 특수 공격 피해·비중은 미정입니다. 빈칸을0으로 해석하지 말고 실행 전에 채워 주세요."},{"Group":"연출","Topic":"연출 프리셋 연결","Description":"블래스터 레이저는 선택한 위험 타일과 방향에 맞게 배치하는 프리셋 이름입니다. 실제 Unity 모션·VFX·소리 연결은 프로그래머와 맞춰야 합니다."},{"Group":"출처","Topic":"기존 파일과 참고","Description":"전투 테이블.xlsx·간격수정.xlsx의 수치와 레이아웃, FFF 전투 프로토타입.html의 연속 예고·타격 순서를 참고했습니다."},{"Group":"출처","Topic":"마스터테이블_스킬.xlsx","Description":"사용기술모션·사용기술어빌리티의 동작/효과 분리 개념 참고. 개별 실행 단계 대신 작업자가 입력할 규칙을 한 행에 모았습니다."},{"Group":"ID 규칙","Topic":"완성된 패턴마다 고유 정수","Description":"PatternID는 종류 이름이 아니라 설정 한 행의 고유 번호입니다. 같은 단일·연속이라도 별도 설정으로 함께 쓸 때는 새 번호를 주세요. 공격 이름은 같아도 되지만 ID는 중복 불가입니다."},{"Group":"ID 규칙","Topic":"20001~29999 단일 계열","Description":"20001 일반 단일 / 20002 엇박 단일 / 20003 방어 불가 단일 / 20010 타일 파괴 단일 / 20020 샌즈 블래스터. 각 행의 실제 설정은 독립입니다."},{"Group":"ID 규칙","Topic":"30001~39999 반복 계열","Description":"30001 랜덤2~5연속 / 30002 랜덤2~3연속 / 30003 랜덤4~5연속. 1~5처럼 단일도 나올 수 있는 반복 규칙도 이 번호대에 둡니다."},{"Group":"ID 규칙","Topic":"40001~49999 경로 순차","Description":"40001 풀에서 경로 선택 / 40002 ㄹ자9칸 / 40003 대각선3칸. 새 경로 변형은 같은 번호대의 사용하지 않는 번호를 선택하세요."},{"Group":"ID 규칙","Topic":"50001~59999 강제 이동 계열","Description":"50001 샌즈 상대 밀치기. 번호대는 정리용이며 코드가 숫자 앞자리로 기능을 추측하지 않습니다. 실제 동작은 범위 사용 방식과 각 설정값을 읽습니다."},{"Group":"ID 규칙","Topic":"기존 패턴 수정과 복사","Description":"공유 패턴 값을 고치면 그 ID를 쓰는 모든 몬스터에게 반영됩니다. 특정 몬스터만 다르게 쓰려면 행을 복사하고 새 ID를 부여한 뒤 그 몬스터의 참조만 바꾸세요."},{"Group":"ID 규칙","Topic":"실제 연결 예시","Description":"몬스터 사용 패턴에서 20010을 선택하면 타일 파괴 단일을 가져옵니다. 30002와30003을 사용하는 초반·후반 연결 예시는 끄기로 추가했습니다. 기존 활성 패턴과 비중은 유지했습니다."},{"Group":"범위 풀 ID","Topic":"60001 전체 9종","Description":"기존 RANDOM_AREA 후보1~9. 60001을 쓰는 모든 공격은 이 후보와 선택 비중을 공유합니다."},{"Group":"범위 풀 ID","Topic":"60002 후보 1~4","Description":"60001에서 후보1~4를 복사해 별도 풀로 등록했습니다. 후보5~9는 이 풀에 없습니다. 기존60001에는 영향을 주지 않습니다."},{"Group":"범위 풀 ID","Topic":"70001 순차 경로 4종","Description":"기존 SEQUENTIAL_PATH의 행·열·대각선 경로 후보4개. 60000번대는 범위 후보, 70000번대는 경로 후보 정리용 번호대입니다. 실제 사용 방식은 공격 설정에서 정합니다."},{"Group":"범위 풀 ID","Topic":"같은 풀 ID의 반복은 정상","Description":"같은 묶음 안의 여러 행은 ShapePoolID가 같아야 합니다. 각 행의 키는 ShapePoolID+Candidate입니다. 다른 풀에서는 후보 번호1·2·3을 다시 사용할 수 있습니다."},{"Group":"범위 풀 ID","Topic":"부분 후보를 쓰는 몬스터","Description":"몬스터 사용 패턴의20004 → 공격 만들기의60002 → 범위 풀의후보1~4. 20001 →60001은 후보1~9입니다. 같은 공격에서 서로 다른 풀을 쓰려면 공격도 복사해 새 PatternID를 주세요."},{"Group":"범위 풀 ID","Topic":"비중은 각 풀 안에서 계산","Description":"60002의 비중25·25·5·5를 그대로 복사했습니다. 합계60으로 나누므로 확률은 약41.67%·41.67%·8.33%·8.33%입니다. 균등하게 하려면 모두1로 바꾸세요."},{"Group":"범위 풀 ID","Topic":"후보와 비중을 다르게 유지","Description":"새 풀을 만들 때 필요한 행을 복사하고 같은 새 ShapePoolID를 지정하세요. 기존 풀을 직접 수정하면 그것을 쓰는 모든 패턴에 영향을 줍니다."},{"Group":"확장 원칙","Topic":"기존 기능부터 조합","Description":"새 요구는 기존 페이즈·패턴 행·대사 조건·연출로 먼저 표현합니다. 전용 컬럼은 기존 구조로 표현할 수 없을 때만 추가합니다."},{"Group":"페이즈","Topic":"취객 네 단계","Description":"단계당 HP 750, 네 단계 합계 3000. 전환 사건은 빈틈공격 성공, 다음 페이즈 2→3→4→빈칸. 연타 시간이 끝나고 대사까지 마쳐야 다음 단계로 갑니다. 무입력·MISS는 진행하지 않습니다."},{"Group":"패턴","Topic":"취객 엇박 조절 위치","Description":"몬스터 사용 패턴에서 1~4페이즈의 엇박은 20011/20002/20012/20013. 공격 만들기의 ResponseMs와 ExtraMinMs·ExtraMaxMs로 조절하세요. 기본 단일과 공격 후 대기는 같습니다."},{"Group":"표시","Topic":"빈틈 피해 숫자","Description":"몬스터 페이즈의 OpeningDamageDisplay는 선택 입력. 빈칸=플레이어 DodgeDamage. 직접 입력=표시만 변경. 실제 피해는 플레이어에서 가져옵니다."},{"Group":"파일","Topic":"작업용·Unity용 한 버전","Description":"작업은 한글 XLSM에서 합니다. 수정한 파일을 시뮬레이터로 불러오고 변경 의도를 적어 버전 저장을 누르면 Unity용 XLSX도 함께 만듭니다."},{"Group":"버전 저장","Topic":"두 파일의 관계","Description":"확정된 게임 데이터는 두 파일이 같습니다. 한글·매크로·3행 제목은 작업용, 영문 시트·1행 제목·TRUE/FALSE는 Unity용입니다."},{"Group":"버전 저장","Topic":"변경 이력","Description":"년-월-일_시-분-초 폴더마다 변경 의도와 시트·행 키·컬럼·이전 값·변경 후 값을 기록합니다. 엑셀 Ctrl+S 후 시뮬레이터에서 불러와 버전 저장하세요."},{"Group":"버전 저장","Topic":"미완성 행과 동시 편집","Description":"미완성 마왕 페이즈는 작업용에 보관합니다. 한 번에는 둘 중 한 파일을 기준으로 수정하세요. 두 파일을 따로 수정한 내용은 자동 병합하지 않습니다."},{"Group":"미용 대사","Topic":"처음 부탁과 네?","Description":"대사에는 실제 문장을, 미용 대사 연결에는 손님 ID·단계·처음 부탁 그룹·자세한 부탁 그룹을 작성합니다. 같은 그룹의 Order는 연속 문장 순서이며 선택 분기가 아닙니다."},{"Group":"미용 대사","Topic":"알겠습니다와 다시 듣기","Description":"처음 부탁의 마지막 문장 뒤 네?/알겠습니다를 표시합니다. 자세한 부탁 뒤에는 알겠습니다만 표시합니다. 이미 들은 단계는 자동 반복하지 않고 다시 듣기로 재생합니다. 되물은 단계는 자세한 부탁을 다시 재생합니다."},{"Group":"미용 대사","Topic":"미용 단계 값","Description":"Stage는 cut(형태 만들기),draw(색·무늬 꾸미기),attach(장식 붙이기). 손님 ID와 Stage 조합은 중복할 수 없습니다. 처음 부탁·자세한 부탁 그룹 모두 존재하는 대사를 참조해야 합니다."},{"Group":"미용 대사","Topic":"엑셀 반영 경로","Description":"수정한 엑셀을 통합 개발실의 야차 편집기에서 불러온 뒤 미용 또는 대사 화면으로 이동하면 같은 대사 데이터로 시험합니다. 버전 저장은 XLSM/XLSX 한 쌍을 만듭니다. 공개 웹 반영은 프로젝트 JSON 내보내기 후 배포가 필요합니다."},{"Group":"미용 대사","Topic":"Unity 연동 범위","Description":"SalonDialogue: MonsterID int,Stage string,RequestGroupID int,DetailGroupID int. 웹 시뮬레이터와 엑셀 양방향 변환에 반영. Unity C# 수신 클래스·선택지 실행 연결은 프로그래머 확인 필요. 미용 영역·점수·그래픽 설정은 프로젝트 JSON에 유지."},{"Group":"미용 대사","Topic":"이전 두 번째 되묻기","Description":"기존 80004 그룹과 대사는 삭제하지 않고 보관. 현재 네? 한 번 흐름에는 연결하지 않음. 재생 여부는 미용 대사 연결에서 결정."}]},{"name":"대사","keys":["DialogueID","GroupID","Order","Speaker","Text","Notes"],"rows":[{"DialogueID":900002,"GroupID":80001,"Order":1,"Speaker":"몬스터","Text":"으어어...안녕하십니까...지원자 11번...아, 미용실이지...","Notes":"기존 좀비 원문"},{"DialogueID":900003,"GroupID":80001,"Order":2,"Speaker":"플레이어","Text":"얏호―! 어서오세요. 그런데 거긴 거울이에요. 저는 옆에 있는데요?","Notes":"기존 좀비 원문"},{"DialogueID":900004,"GroupID":80001,"Order":3,"Speaker":"몬스터","Text":"아… 어쩐지… 같이 인사를 해주시더라니...","Notes":"기존 좀비 원문"},{"DialogueID":900005,"GroupID":80001,"Order":4,"Speaker":"몬스터","Text":"아무튼… 내일 좀비 보험회사 면접이 있어서요… 죽고 나서 처음 잡힌 면접이에요…","Notes":"기존 좀비 원문"},{"DialogueID":900006,"GroupID":80001,"Order":5,"Speaker":"플레이어","Text":"보험이요...? 좀비는 보험이 필요없지 않나?","Notes":"기존 좀비 원문"},{"DialogueID":900007,"GroupID":80001,"Order":6,"Speaker":"몬스터","Text":"어허, 그거 종족차별 발언입니다...! 요새 그런 말 하면... 큰일나요...","Notes":"기존 좀비 원문"},{"DialogueID":900008,"GroupID":80001,"Order":7,"Speaker":"플레이어","Text":"(별 귀찮은 것도 다 있네~) 알았다구요~ 원하는 스타일은 있나요?","Notes":"기존 좀비 원문"},{"DialogueID":900009,"GroupID":80001,"Order":8,"Speaker":"몬스터","Text":"지난번엔 면접관님 눈을 보고 대답하라길래… 한참 열심히 했거든요…","Notes":"기존 좀비 원문"},{"DialogueID":900010,"GroupID":80001,"Order":9,"Speaker":"플레이어","Text":"그런데요?","Notes":"기존 좀비 원문"},{"DialogueID":900011,"GroupID":80001,"Order":10,"Speaker":"몬스터","Text":"면접관님은 옆에 계셨대요… 저는 공기청정기한테… 입사 포부를…","Notes":"기존 좀비 원문"},{"DialogueID":900012,"GroupID":80001,"Order":11,"Speaker":"플레이어","Text":"O.K~ 이해 완료! 앞이 보이게 해 드리면 되는 거죠?","Notes":"기존 좀비 원문"},{"DialogueID":900013,"GroupID":80001,"Order":12,"Speaker":"몬스터","Text":"부탁드려요… 이번엔 정말… 산 사람처럼 살고 싶어서요…","Notes":"기존 좀비 원문"},{"DialogueID":900014,"GroupID":80002,"Order":1,"Speaker":"몬스터","Text":"으어어... 내일 면접인데... &lt;color=#266B4D&gt;앞이 좀 환해지고&lt;/color&gt;,\n&lt;color=#9A4935&gt;민망한 곳은 안 보였으면&lt;/color&gt; 좋겠어요...","Notes":"미용 요구 · 선택지 연결"},{"DialogueID":900015,"GroupID":80003,"Order":1,"Speaker":"몬스터","Text":"&lt;color=#266B4D&gt;두 눈이 잘 보이게&lt;/color&gt; 앞머리를 잘라 주세요...\n아, &lt;color=#9A4935&gt;튀어나온 뇌는 머리카락으로 가려&lt;/color&gt; 주시고요... &lt;wave=1.2&gt;부탁드립니다...&lt;/wave&gt;","Notes":"미용 요구 · 선택지 연결"},{"DialogueID":900016,"GroupID":80004,"Order":1,"Speaker":"몬스터","Text":"아니, 앞이 안 보인다고요! 당장 '가위'를 들어서 내 눈을 가리는 앞머리를 싹 다 잘라달란 말입니다!","Notes":"기존 좀비 원문"},{"DialogueID":900017,"GroupID":80005,"Order":1,"Speaker":"몬스터","Text":"으어어… 이게 제 눈이었군요…! 거울 속에 아주 준비된 인재가 한 명 서 있는데요…","Notes":"기존 좀비 원문"},{"DialogueID":900018,"GroupID":80006,"Order":1,"Speaker":"몬스터","Text":"으어어… 일단 앞은 보이네요… 면접관이 한 분만 오시면 딱 좋겠어요…","Notes":"기존 좀비 원문"},{"DialogueID":900019,"GroupID":80007,"Order":1,"Speaker":"몬스터","Text":"으어어어! 이게 머립니까?? 이 꼴을 하고 면접을 가라고요?! 안 되겠다, 이대론 돈 못 냅니다!","Notes":"기존 좀비 원문"},{"DialogueID":900020,"GroupID":80008,"Order":1,"Speaker":"몬스터","Text":"머리도 잘 됐겠다, 제 기세를 한 번 시험해 주시겠어요? 면접 때 자신있게 싸울... 아니 말할 수 있는지 봐주시면 됩니다.","Notes":"기존 좀비 원문"},{"DialogueID":900021,"GroupID":80008,"Order":2,"Speaker":"몬스터","Text":"연습 야차 상대를... 부탁드린다는 뜻입니다... 저를 이기시면... 보상은 두둑히 드릴게요...","Notes":"기존 좀비 원문"},{"DialogueID":900022,"GroupID":80009,"Order":1,"Speaker":"몬스터","Text":"머리도 됐으니... 제 기세를 한 번 시험해 주시겠어요? 면접 때 자신있게 싸울... 아니 말할 수 있는지 봐주시면 됩니다.","Notes":"기존 좀비 원문"},{"DialogueID":900023,"GroupID":80009,"Order":2,"Speaker":"몬스터","Text":"연습 야차 상대를... 부탁드린다는 뜻입니다...저를 이기시면... 돈은 더 드릴게요…","Notes":"기존 좀비 원문"},{"DialogueID":900024,"GroupID":80010,"Order":1,"Speaker":"몬스터","Text":"가위 내려놓으실래요? 제가 면접관이라 생각하고 대답해 보세요. 제 머리... 왜 이렇게 하셨죠?","Notes":"기존 좀비 원문"},{"DialogueID":900025,"GroupID":80010,"Order":2,"Speaker":"몬스터","Text":"마왕 법전 제 666조! 야차룰로 정하죠. 제가 이기면... 배상하시는 겁니다!!!","Notes":"기존 좀비 원문"},{"DialogueID":900026,"GroupID":80011,"Order":1,"Speaker":"몬스터","Text":"으어어... 제가 대인배라 넘어갑니다... 다른 손님에겐 이렇게 하지 마세요...","Notes":"기존 좀비 원문"},{"DialogueID":900027,"GroupID":80012,"Order":1,"Speaker":"몬스터","Text":"으... 어쩔 수 없죠. 저도 면접 볼 체력을 아끼는 걸로 할게요. 머리 잘 해주셔서 감사합니다...","Notes":"기존 좀비 원문"},{"DialogueID":900028,"GroupID":80013,"Order":1,"Speaker":"몬스터","Text":"으... 어쩔 수 없죠. 저도 면접 볼 체력을 아끼는 걸로 할게요. 감사합니다...","Notes":"기존 좀비 원문"},{"DialogueID":900029,"GroupID":80014,"Order":1,"Speaker":"몬스터","Text":"감사합니다…! 실수로 물어도 이해해주세요… 물고 늘어지는 건 제 장점이라...","Notes":"기존 좀비 원문"},{"DialogueID":900030,"GroupID":80015,"Order":1,"Speaker":"몬스터","Text":"감사합니다…! 실수로 물어도 이해해주세요… 물고 늘어지는 건 제 장점이라...","Notes":"기존 좀비 원문"},{"DialogueID":900031,"GroupID":80016,"Order":1,"Speaker":"몬스터","Text":"안녕하십니까…! 한번 맡은 일은 죽어서도 놓지 않는 지원자… 으어어… 실제로 죽어봤습니다!","Notes":"기존 좀비 원문"},{"DialogueID":900032,"GroupID":80017,"Order":1,"Speaker":"몬스터","Text":"변명은 됐습니다… 저도 이빨 좀 쓰겠습니다!","Notes":"기존 좀비 원문"},{"DialogueID":900033,"GroupID":80018,"Order":1,"Speaker":"몬스터","Text":"제 강점은… 끈질긴 후속 연락입니다…!","Notes":"기존 좀비 원문"},{"DialogueID":900034,"GroupID":80018,"Order":2,"Speaker":"몬스터","Text":"정시 출근... 아니, 정시 타격입니다!","Notes":"기존 좀비 원문"},{"DialogueID":900035,"GroupID":80019,"Order":1,"Speaker":"몬스터","Text":"이건... 고객 피드백입니다...!","Notes":"기존 좀비 원문"},{"DialogueID":900036,"GroupID":80019,"Order":2,"Speaker":"몬스터","Text":"서류 30번 떨어진 한... 받아라!!","Notes":"기존 좀비 원문"},{"DialogueID":900037,"GroupID":80020,"Order":1,"Speaker":"몬스터","Text":"으어어… 머리만은 건드리지 말아주세요…!","Notes":"기존 좀비 원문"},{"DialogueID":900038,"GroupID":80021,"Order":1,"Speaker":"몬스터","Text":"커헉... 스펙이 너무 높아...","Notes":"기존 좀비 원문"},{"DialogueID":900039,"GroupID":80022,"Order":1,"Speaker":"몬스터","Text":"제 기세에 압도되셨군요...!","Notes":"기존 좀비 원문"},{"DialogueID":900040,"GroupID":80023,"Order":1,"Speaker":"몬스터","Text":"벌써 지치셨습니까? 감점 들어갑니다.","Notes":"기존 좀비 원문"},{"DialogueID":900041,"GroupID":80024,"Order":1,"Speaker":"몬스터","Text":"이럴 수가... 머리도 잃고 돈도 잃다니... 으어어...","Notes":"기존 좀비 원문"},{"DialogueID":900042,"GroupID":80025,"Order":1,"Speaker":"몬스터","Text":"약속대로... 돈은 돌려받겠습니다...","Notes":"기존 좀비 원문"},{"DialogueID":900043,"GroupID":80026,"Order":1,"Speaker":"몬스터","Text":"역시 이 정도는 되어야... 취업 성공하는 거군요... 리스펙합니다.","Notes":"기존 좀비 원문"},{"DialogueID":900044,"GroupID":80027,"Order":1,"Speaker":"몬스터","Text":"으어어! 이 기세로 합격까지 갑니다!","Notes":"기존 좀비 원문"},{"DialogueID":900045,"GroupID":80028,"Order":1,"Speaker":"몬스터","Text":"으어어… 머리도 단정하고… 두들겨 맞아서 어깨 힘도 빠졌네요… 면접 준비 끝났어요…","Notes":"기존 좀비 원문"},{"DialogueID":900046,"GroupID":80028,"Order":2,"Speaker":"플레이어","Text":"긴장 덜고 웃음 MAX로 승부보는 거예요~! 얏호~!","Notes":"기존 좀비 원문"},{"DialogueID":900047,"GroupID":80028,"Order":3,"Speaker":"몬스터","Text":"네… 계약서는 물지 않고… 서명받겠습니다…","Notes":"기존 좀비 원문"},{"DialogueID":900048,"GroupID":80029,"Order":1,"Speaker":"몬스터","Text":"으어… 머리도 잘됐고… 태어나서 처음으로 자신감이 생겼어요… 죽은 뒤에 생기긴 했지만…","Notes":"기존 좀비 원문"},{"DialogueID":900049,"GroupID":80029,"Order":2,"Speaker":"플레이어","Text":"그 자신감으로 내일은 말로 설득 가보자고요~!!","Notes":"기존 좀비 원문"},{"DialogueID":900050,"GroupID":80029,"Order":3,"Speaker":"몬스터","Text":"네... 그럼 안녕히...","Notes":"기존 좀비 원문"},{"DialogueID":900051,"GroupID":80030,"Order":1,"Speaker":"몬스터","Text":"으어어…머리가 헝클어졌네... 내일도 이러면 어떡하죠…","Notes":"기존 좀비 원문"},{"DialogueID":900052,"GroupID":80030,"Order":2,"Speaker":"플레이어","Text":"초~ 큐트한 키라키라★리본 머리핀 있는데 드릴까요?","Notes":"기존 좀비 원문"},{"DialogueID":900053,"GroupID":80030,"Order":3,"Speaker":"몬스터","Text":"아니요... 친근한 인상으로 승부해볼게요...","Notes":"기존 좀비 원문"},{"DialogueID":900054,"GroupID":80030,"Order":4,"Speaker":"몬스터","Text":"그럼 안녕히…","Notes":"기존 좀비 원문"},{"DialogueID":900055,"GroupID":80031,"Order":1,"Speaker":"몬스터","Text":"으어어… 어찌저찌 이겼으니… 내일 면접도 어떻게든 되겠죠…","Notes":"기존 좀비 원문"},{"DialogueID":900056,"GroupID":80031,"Order":2,"Speaker":"플레이어","Text":"에에~ 면접이랑 싸움은 별개쟝~","Notes":"기존 좀비 원문"},{"DialogueID":900057,"GroupID":80031,"Order":3,"Speaker":"몬스터","Text":"그건 그렇죠... 어쨌든 감사합니다...","Notes":"기존 좀비 원문"},{"DialogueID":900058,"GroupID":80031,"Order":4,"Speaker":"몬스터","Text":"그럼 안녕히…","Notes":"기존 좀비 원문"},{"DialogueID":900059,"GroupID":80032,"Order":1,"Speaker":"몬스터","Text":"으어어… 내일 이 머리 얘기가 나오면… 뭐라고 해야 할까요…","Notes":"기존 좀비 원문"},{"DialogueID":900060,"GroupID":80032,"Order":2,"Speaker":"플레이어","Text":"초- 신선한 유행의 선두주자― 인데스케도 면접관이 사람 보는 눈이 없는 거네~","Notes":"기존 좀비 원문"},{"DialogueID":900061,"GroupID":80032,"Order":3,"Speaker":"몬스터","Text":"새로운 시도를 두려워하지 않는다는 거죠... 어떻게든 해볼게요...","Notes":"기존 좀비 원문"},{"DialogueID":900062,"GroupID":80033,"Order":1,"Speaker":"몬스터","Text":"으어어… 내일 이 머리 얘기가 나오면… 뭐라고 해야 하지…","Notes":"기존 좀비 원문"},{"DialogueID":900063,"GroupID":80033,"Order":2,"Speaker":"플레이어","Text":"초- 신선한 유행의 선두주자― 인데스케도 면접관이 사람 보는 눈이 없는 거네~","Notes":"기존 좀비 원문"},{"DialogueID":900064,"GroupID":80033,"Order":3,"Speaker":"몬스터","Text":"........상당히 뻔뻔하시네요… 으어어….어떻게든 되겠죠…","Notes":"기존 좀비 원문"},{"DialogueID":900065,"GroupID":80033,"Order":4,"Speaker":"몬스터","Text":"이번에도 탈락하면... 대체 언제.....하아…","Notes":"기존 좀비 원문"},{"DialogueID":900066,"GroupID":80034,"Order":1,"Speaker":"몬스터","Text":"으어... 취직했다... 앞머리도 방구석 생활도 해방됨...... 몇달만에 사람 얼굴 제대로 보는 느낌ㅠㅠ #몬스터헤어살롱 덕분에 붙은 것 같아요 감사합니다. 모두 기 받아가세요! #취업성공 #취준생 #화이팅","Notes":"기존 좀비 원문"},{"DialogueID":900067,"GroupID":80035,"Order":1,"Speaker":"몬스터","Text":"역시나 면접 떨어졌다….. #취준생 #절규 #미용실저주함 돈도 잃고 머리도 잃음","Notes":"기존 좀비 원문"},{"DialogueID":900068,"GroupID":80036,"Order":1,"Speaker":"몬스터","Text":"&lt;wave=3 speed=5&gt;&lt;color=#FFD166&gt;&lt;size=24&gt;으하하하!&lt;/size&gt;&lt;/color&gt; 오랜만이구먼, &lt;color=#FFDA8A&gt;제이!!&lt;/color&gt;&lt;/wave&gt;&lt;wait=0.25&gt; 미용실에 불이 켜졌길래... 드디어 돌아온 줄 알았지!","Notes":"취객의 가업·제이·몬스터 소울을 떠올리는 단서. 실제 해금·튜토리얼은 야차 이후 미용실에서 진행."},{"DialogueID":900070,"GroupID":80038,"Order":1,"Speaker":"몬스터","Text":"&lt;shake=2 speed=15 dur=0.45&gt;어이쿠!&lt;/shake&gt;&lt;wait=0.3&gt; 손맛 한번 여전하구먼.&lt;wave=2 speed=4&gt; 근데 제이, 자네... 원래 둘이었나?&lt;/wave&gt;","Notes":"색·동작 태그는 문자 효과 규칙 시트 참고."},{"DialogueID":900071,"GroupID":80039,"Order":1,"Speaker":"몬스터","Text":"어...&lt;wait=0.4&gt; &lt;color=#A9E4DA&gt;이제 한 명으로 보이네.&lt;/color&gt; 제이가... 아니군.&lt;wait=0.45&gt; 미용실에 불이 들어왔길래, 그 녀석인 줄 알았어.","Notes":"취객의 가업·제이·몬스터 소울을 떠올리는 단서. 실제 해금·튜토리얼은 야차 이후 미용실에서 진행."},{"DialogueID":900072,"GroupID":80040,"Order":1,"Speaker":"몬스터","Text":"허... 막일할 때도 굳어 있던 손이...&lt;wait=0.4&gt; 이 감각, &lt;color=#FFD166&gt;소울을 벼리던 때&lt;/color&gt;랑 닮았구먼.&lt;wait=0.3&gt; 제이가 봤으면 또 실실 웃었겠어!","Notes":"취객의 가업·제이·몬스터 소울을 떠올리는 단서. 실제 해금·튜토리얼은 야차 이후 미용실에서 진행."},{"DialogueID":900073,"GroupID":80041,"Order":1,"Speaker":"몬스터","Text":"&lt;shake=2 speed=16 dur=0.4&gt;크하!&lt;/shake&gt; ...&lt;wait=0.4&gt;&lt;color=#B7F4D0&gt;다 깼다, 다 깼어!&lt;/color&gt;\n옛 솜씨도 술에 몽땅 절여진 줄 알았더니! &lt;pulse=1.1 speed=7&gt;아직 쓸 만하구먼! 으하하하!&lt;/pulse&gt;","Notes":"취객의 가업·제이·몬스터 소울을 떠올리는 단서. 실제 해금·튜토리얼은 야차 이후 미용실에서 진행."},{"DialogueID":900074,"GroupID":80042,"Order":1,"Speaker":"몬스터","Text":"우리 집안은 &lt;color=#FFD166&gt;몬스터 소울을 장비와 기술로 벼렸지.&lt;/color&gt; 세상은 바뀌고, 찾는 이도 줄고...&lt;wait=0.4&gt; 제이까지 사라지고 나니 더 붙들 이유가 없더군.","Notes":"취객의 가업·제이·몬스터 소울을 떠올리는 단서. 실제 해금·튜토리얼은 야차 이후 미용실에서 진행."},{"DialogueID":900075,"GroupID":80042,"Order":2,"Speaker":"몬스터","Text":"그런데 그 미용실에 &lt;color=#B7F4D0&gt;다시 불이 켜졌어.&lt;/color&gt;&lt;wait=0.4&gt; 내 손도 아직 기억하고 있고. 돌아가세. 자네한테 보여줄 게 떠올랐거든! &lt;wave=2 speed=6&gt;&lt;color=#FFD166&gt;으하하하!&lt;/color&gt;&lt;/wave&gt;","Notes":"취객의 가업·제이·몬스터 소울을 떠올리는 단서. 실제 해금·튜토리얼은 야차 이후 미용실에서 진행."},{"DialogueID":900069,"GroupID":80037,"Order":1,"Speaker":"몬스터","Text":"헤헤.&lt;wait=0.35&gt; 오늘은... &lt;color=#8BE9FD&gt;가볍게&lt;/color&gt; 가자고, 친구.","Notes":"색·동작 태그는 문자 효과 규칙 시트 참고."},{"DialogueID":900076,"GroupID":80043,"Order":1,"Speaker":"몬스터","Text":"...하하.. 친구..&lt;wait=0.4&gt; 나한텐 &lt;color=#8BE9FD&gt;무용지물&lt;/color&gt;일 텐데..?","Notes":"색·동작 태그는 문자 효과 규칙 시트 참고."},{"DialogueID":900077,"GroupID":80044,"Order":1,"Speaker":"몬스터","Text":"뭐...&lt;wait=0.45&gt; 이 정도는 맞아줄 수 있지.&lt;wait=0.3&gt; &lt;color=#8BE9FD&gt;서비스&lt;/color&gt;라고 해 두자고.","Notes":"색·동작 태그는 문자 효과 규칙 시트 참고."},{"DialogueID":900078,"GroupID":80045,"Order":1,"Speaker":"몬스터","Text":"헤헤... 같은 수는 두 번 안 통한다고.&lt;wait=0.35&gt; ...방금 건 &lt;color=#8BE9FD&gt;연습&lt;/color&gt;이었지?","Notes":"색·동작 태그는 문자 효과 규칙 시트 참고."},{"DialogueID":900079,"GroupID":80046,"Order":1,"Speaker":"몬스터","Text":"...어라.&lt;wait=0.6&gt; 그 타이밍을 또 맞혔네.&lt;wait=0.35&gt; &lt;shake=1.4 speed=14&gt;좀 쉬엄쉬엄하자고, 친구.&lt;/shake&gt;","Notes":"색·동작 태그는 문자 효과 규칙 시트 참고."},{"DialogueID":900080,"GroupID":80047,"Order":1,"Speaker":"몬스터","Text":"잠깐,&lt;wait=0.45&gt; 우리...&lt;wait=0.45&gt; &lt;color=#8BE9FD&gt;친구잖아..?&lt;/color&gt;\n&lt;shake=2.2 speed=20&gt;날 정말 죽일 셈이야..?&lt;/shake&gt;","Notes":"색·동작 태그는 문자 효과 규칙 시트 참고."},{"DialogueID":900081,"GroupID":80048,"Order":1,"Speaker":"몬스터","Text":"나는 이래서...&lt;wait=0.65&gt; &lt;cps=16&gt;&lt;shake=1.6 speed=16&gt;&lt;color=#FF9797&gt;눈치 빠른 애송이들이 싫어...&lt;/color&gt;&lt;/shake&gt;&lt;/cps&gt;","Notes":"색·동작 태그는 문자 효과 규칙 시트 참고."},{"DialogueID":900082,"GroupID":80049,"Order":1,"Speaker":"몬스터","Text":"&lt;wave=2 speed=5&gt;&lt;color=#B7F4D0&gt;으어어...&lt;/color&gt;&lt;/wave&gt; 손 좀 빌려주세요.&lt;wait=0.25&gt; 아, &lt;shake=2 dur=0.4&gt;떼어드리진 말구요!&lt;/shake&gt;","Notes":"전투 중 대사. 등장·미용 과정 대사는 보류."},{"DialogueID":900083,"GroupID":80049,"Order":2,"Speaker":"몬스터","Text":"&lt;color=#FFD166&gt;끈기&lt;/color&gt; 하나는 자신 있습니다!&lt;wait=0.3&gt; &lt;wave=2 speed=5&gt;죽어서도 출근하잖아요...&lt;/wave&gt;","Notes":"전투 중 대사. 등장·미용 과정 대사는 보류."},{"DialogueID":900084,"GroupID":80050,"Order":1,"Speaker":"몬스터","Text":"잠깐...&lt;wait=0.25&gt; &lt;shake=2 speed=16 dur=0.5&gt;뼈 때리시면!&lt;/shake&gt; &lt;color=#FFD166&gt;진짜 뼈 맞는다구요!&lt;/color&gt;","Notes":"전투 중 대사. 등장·미용 과정 대사는 보류."},{"DialogueID":900085,"GroupID":80051,"Order":1,"Speaker":"몬스터","Text":"&lt;cps=15&gt;끝난 줄... 아셨죠?&lt;/cps&gt;&lt;wait=0.5&gt; &lt;color=#B7F4D0&gt;&lt;size=23&gt;좀비는 다시 부활한다구요!&lt;/size&gt;&lt;/color&gt;\n&lt;shake=3 speed=16 dur=0.8&gt;&lt;wave=3 speed=5&gt;으어어어..!&lt;/wave&gt;&lt;/shake&gt;","Notes":"전투 중 대사. 등장·미용 과정 대사는 보류."},{"DialogueID":900086,"GroupID":80051,"Order":2,"Speaker":"몬스터","Text":"&lt;color=#FFD166&gt;재도전&lt;/color&gt;에는 자신 있습니다.&lt;wait=0.35&gt; 취업도...&lt;wait=0.5&gt; 이렇게 쉽게 부활하면 좋을 텐데요.","Notes":"전투 중 대사. 등장·미용 과정 대사는 보류."},{"DialogueID":900087,"GroupID":80052,"Order":1,"Speaker":"몬스터","Text":"&lt;wave=2 speed=3&gt;으어어...&lt;/wave&gt;&lt;wait=0.4&gt; 오늘은 여기까지...\n&lt;color=#B7F4D0&gt;재도전도 휴식이 필요하다구요.&lt;/color&gt;","Notes":"전투 중 대사. 등장·미용 과정 대사는 보류."},{"DialogueID":900088,"GroupID":80053,"Order":1,"Speaker":"몬스터","Text":"&lt;color=#FFD166&gt;끈기 있는 지원자!&lt;/color&gt; 저, 맞죠?&lt;wait=0.3&gt; &lt;wave=2 speed=5&gt;으허허... 아직 쓸 만하네요!&lt;/wave&gt;","Notes":"전투 중 대사. 등장·미용 과정 대사는 보류."},{"DialogueID":900089,"GroupID":80054,"Order":1,"Speaker":"몬스터","Text":"면접에선... 첫인상이 중요하다던데요...\n&lt;color=#9A5B22&gt;&lt;pulse=1.06&gt;단정한 인상&lt;/pulse&gt;&lt;/color&gt;이면... 덜 긴장할 것 같아요...","Notes":"미용 요구 · 선택지 연결"},{"DialogueID":900090,"GroupID":80055,"Order":1,"Speaker":"몬스터","Text":"염색이요...? &lt;wave=1.2&gt;&lt;color=#71508F&gt;자유롭게&lt;/color&gt;&lt;/wave&gt; 부탁드려요...\n&lt;color=#266B4D&gt;지금 머리 색도&lt;/color&gt; 저는 좋은데...","Notes":"미용 요구 · 선택지 연결"},{"DialogueID":900091,"GroupID":80056,"Order":1,"Speaker":"몬스터","Text":"으어어... 머리도 정리하고, 정신도 번쩍 들었네요. 내일은 &lt;color=#FFD166&gt;면접장에 부활&lt;/color&gt;하겠습니다!","Notes":"통합 플레이"},{"DialogueID":900092,"GroupID":80057,"Order":1,"Speaker":"몬스터","Text":"으어어... 연습은 여기까지 하죠. 저도 내일 면접이 있어서요.","Notes":"통합 플레이"},{"DialogueID":900093,"GroupID":80058,"Order":1,"Speaker":"몬스터","Text":"&lt;shake=2&gt;으하하하!&lt;/shake&gt; 오랜만이구먼, 제이!!","Notes":"통합 플레이"},{"DialogueID":900094,"GroupID":80058,"Order":2,"Speaker":"몬스터","Text":"가게에 불이 켜져 있길래 냅다 뛰어왔지! 이야, 얼굴이 좀... &lt;wave=3&gt;두 개로 보이는구먼!&lt;/wave&gt;","Notes":"통합 플레이"},{"DialogueID":900095,"GroupID":80059,"Order":1,"Speaker":"몬스터","Text":"...자네, 제이가 아니었구먼. 허허. 이제야 제대로 보이는군.","Notes":"통합 플레이"},{"DialogueID":900096,"GroupID":80059,"Order":2,"Speaker":"몬스터","Text":"제이가 사라진 뒤로 이 가게도, 내 손끝도 멈춘 줄 알았지. 일용직 일 끝내고 한잔하는 게 하루의 전부였어.","Notes":"통합 플레이"},{"DialogueID":900097,"GroupID":80059,"Order":3,"Speaker":"몬스터","Text":"우리 집안은 몬스터의 소울에 남은 힘을 &lt;color=#9FE8D1&gt;장비와 기술로 빚어내던&lt;/color&gt; 일을 했네. 아는 이만 찾던 오래된 가업이지.","Notes":"통합 플레이"},{"DialogueID":900098,"GroupID":80059,"Order":4,"Speaker":"몬스터","Text":"세상이 편리해지니 그 솜씨를 찾는 이도 줄었어. 다시 쓸 일이 없을 줄 알았는데... 자네를 보니, &lt;wave=2&gt;손이 근질근질하구먼!&lt;/wave&gt;","Notes":"통합 플레이"},{"DialogueID":900099,"GroupID":80059,"Order":5,"Speaker":"몬스터","Text":"좋아. 머물러도 된다면 손끝부터 다시 깨워 보지. &lt;color=#FFD166&gt;몬스터 소울을 다루는 법&lt;/color&gt;도 차근차근 알려 주겠네.","Notes":"통합 플레이"},{"DialogueID":900100,"GroupID":80060,"Order":1,"Speaker":"몬스터","Text":"허허, 오늘은 술 대신 물 한 잔이면 되겠어. 도구를 챙겨 올 테니, 가게 불은 꺼뜨리지 말게!","Notes":"통합 플레이"},{"DialogueID":900101,"GroupID":80061,"Order":1,"Speaker":"몬스터","Text":"...헤. 여기 솜씨가 좋다는 소문을 들었거든.","Notes":"통합 플레이"},{"DialogueID":900102,"GroupID":80061,"Order":2,"Speaker":"몬스터","Text":"뼈 있는 부탁 하나 해도 될까? &lt;color=#FFD166&gt;얼굴 테두리&lt;/color&gt;만 다듬어 줘. 머리카락은... 보다시피 휴가 중이야.","Notes":"통합 플레이"},{"DialogueID":900103,"GroupID":80062,"Order":1,"Speaker":"몬스터","Text":"헤. 오늘은 &lt;color=#52609B&gt;인상 좀 다듬으러&lt;/color&gt; 왔어.\n&lt;color=#52609B&gt;각진 데만 가볍게.&lt;/color&gt; &lt;wave=1.3&gt;뼈대는 괜찮잖아?&lt;/wave&gt;","Notes":"미용 요구 · 선택지 연결"},{"DialogueID":900104,"GroupID":80063,"Order":1,"Speaker":"몬스터","Text":"이번엔 좀 &lt;color=#9A4935&gt;&lt;shake=0.6&gt;만만하지 않은 인상&lt;/shake&gt;&lt;/color&gt;이면 좋겠어.\n&lt;color=#9A4935&gt;장식&lt;/color&gt;으로 한 수 보여 줄래?","Notes":"미용 요구 · 선택지 연결"},{"DialogueID":900105,"GroupID":80064,"Order":1,"Speaker":"몬스터","Text":"헤. 꽤 뼈대 있는 실력이네. 그럼... 몸도 한번 풀어 볼까?","Notes":"통합 플레이"},{"DialogueID":900106,"GroupID":80065,"Order":1,"Speaker":"몬스터","Text":"나쁘지 않네. 이번엔 다른 솜씨도 보여 줄래?","Notes":"통합 플레이"},{"DialogueID":900107,"GroupID":80066,"Order":1,"Speaker":"몬스터","Text":"...친구, 이건 좀 뼈아픈데. 잠깐 밖에서 얘기할까?","Notes":"통합 플레이"},{"DialogueID":900108,"GroupID":80067,"Order":1,"Speaker":"나레이션","Text":"미용실로 돌아오자, 문에 달린 종이 작게 울렸다. 오늘의 마지막 손님과의 야차가 끝났다.","Notes":"통합 플레이"},{"DialogueID":900109,"GroupID":80068,"Order":1,"Speaker":"몬스터","Text":"&lt;color=#71508F&gt;어떤 색이나 무늬든&lt;/color&gt; 괜찮아요...\n&lt;color=#266B4D&gt;염색하지 않아도 좋아요.&lt;/color&gt; 머리는 지금도 마음에 들어서...","Notes":"미용 선택지 대사"},{"DialogueID":900110,"GroupID":80069,"Order":1,"Speaker":"몬스터","Text":"면접장에서 &lt;color=#9A5B22&gt;단정하고 점잖아 보일 장식&lt;/color&gt;으로...\n&lt;color=#9A5B22&gt;하나만&lt;/color&gt; 골라 주시겠어요...? &lt;wave=1.2&gt;너무 요란하진 않게요...&lt;/wave&gt;","Notes":"미용 선택지 대사"},{"DialogueID":900111,"GroupID":80070,"Order":1,"Speaker":"몬스터","Text":"&lt;color=#52609B&gt;얼굴 바깥 테두리만&lt;/color&gt; 망치랑 정으로 톡톡 다듬어 줘.\n&lt;color=#9A4935&gt;눈코입은 그대로.&lt;/color&gt; &lt;wave=1.2&gt;속까지 시원해질 필요는 없거든.&lt;/wave&gt;","Notes":"미용 선택지 대사"},{"DialogueID":900112,"GroupID":80071,"Order":1,"Speaker":"몬스터","Text":"색은 &lt;color=#71508F&gt;네 감각에 맡길게.&lt;/color&gt;\n&lt;color=#52609B&gt;원래 뼈 색&lt;/color&gt;도 꽤 멋지거든. &lt;wave=1.2&gt;뼈가 있는 색이지.&lt;/wave&gt;","Notes":"미용 선택지 대사"},{"DialogueID":900113,"GroupID":80072,"Order":1,"Speaker":"몬스터","Text":"&lt;color=#71508F&gt;더한 뼈와 바깥 테두리&lt;/color&gt;에 마음 가는 색을 칠해 봐.\n&lt;color=#52609B&gt;그대로 둬도 좋아.&lt;/color&gt; 취향엔 정답이 없으니까. 헤.","Notes":"미용 선택지 대사"},{"DialogueID":900114,"GroupID":80073,"Order":1,"Speaker":"몬스터","Text":"&lt;color=#9A4935&gt;강해 보이는 장식 하나&lt;/color&gt;를 &lt;color=#52609B&gt;얼굴이나 머리 쪽&lt;/color&gt;에 부탁해.\n딱 봤을 때 &lt;shake=0.6&gt;쉽게 덤비지는 못하겠다&lt;/shake&gt; 싶은 걸로.","Notes":"미용 선택지 대사"}]},{"name":"대화 그룹","keys":["GroupID","Name","PlaybackMode","PauseCombat","AdvanceMode","CPS","HoldMs","GapMs","Notes","ActorEffect","FinishEffect"],"rows":[{"GroupID":80001,"Name":"좀비 등장 대화","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80002,"Name":"취준좀비 · 형태 만들기 · 처음 부탁","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"미용 대사 연결에서 선택하는 부탁","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80003,"Name":"취준좀비 · 형태 만들기 · 자세한 부탁","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"미용 대사 연결에서 선택하는 부탁","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80004,"Name":"미용 요청 · 두 번째 되묻기","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80005,"Name":"미용 대성공 · 결과 반응","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80006,"Name":"미용 보통 성공 · 결과 반응","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80007,"Name":"미용 실패 · 결과 반응","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80008,"Name":"미용 대성공 · 야차 제안","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80009,"Name":"미용 보통 성공 · 야차 제안","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80010,"Name":"미용 실패 · 필수 야차 통보","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80011,"Name":"미용 실패 · 배상 완료","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80012,"Name":"미용 대성공 · 야차 거절","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80013,"Name":"미용 보통 성공 · 야차 거절","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80014,"Name":"미용 대성공 · 야차 수락","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80015,"Name":"미용 보통 성공 · 야차 수락","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80016,"Name":"미용 성공 · 전투 시작","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":30,"HoldMs":1500,"GapMs":400,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80017,"Name":"미용 실패 · 전투 시작","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":30,"HoldMs":1500,"GapMs":400,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80018,"Name":"미용 성공 · 전투 중 공격","PlaybackMode":"무작위 한 줄","PauseCombat":false,"AdvanceMode":"자동","CPS":30,"HoldMs":1500,"GapMs":400,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80019,"Name":"미용 실패 · 전투 중 공격","PlaybackMode":"무작위 한 줄","PauseCombat":false,"AdvanceMode":"자동","CPS":30,"HoldMs":1500,"GapMs":400,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80020,"Name":"미용 성공 · 좀비 HP 낮음","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":30,"HoldMs":1500,"GapMs":400,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80021,"Name":"미용 실패 · 좀비 HP 낮음","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":30,"HoldMs":1500,"GapMs":400,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80022,"Name":"미용 성공 · 플레이어 HP 낮음","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":30,"HoldMs":1500,"GapMs":400,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80023,"Name":"미용 실패 · 플레이어 HP 낮음","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":30,"HoldMs":1500,"GapMs":400,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80024,"Name":"미용 실패 · 플레이어 야차 승리","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":30,"HoldMs":1500,"GapMs":400,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80025,"Name":"미용 실패 · 플레이어 야차 패배","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":30,"HoldMs":1500,"GapMs":400,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80026,"Name":"미용 성공 · 플레이어 연습 야차 승리","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":30,"HoldMs":1500,"GapMs":400,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80027,"Name":"미용 성공 · 플레이어 연습 야차 패배","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":30,"HoldMs":1500,"GapMs":400,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80028,"Name":"미용 대성공 · 플레이어 승리 후 퇴장","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80029,"Name":"미용 대성공 · 플레이어 패배 후 퇴장","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80030,"Name":"미용 보통 성공 · 플레이어 승리 후 퇴장","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80031,"Name":"미용 보통 성공 · 플레이어 패배 후 퇴장","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80032,"Name":"미용 실패 · 플레이어 승리 후 퇴장","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80033,"Name":"미용 실패 · 플레이어 패배 후 퇴장","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80034,"Name":"몬스타그램 · 미용 성공 (야차 무관)","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":0,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80035,"Name":"몬스타그램 · 미용 실패 (조건 확인 필요)","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":0,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80036,"Name":"취객 · 제이로 착각","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":29,"HoldMs":1200,"GapMs":250,"Notes":"취객·샌즈 전투 연출 초안. 태그와 시간은 자유롭게 조정 가능.","ActorEffect":"비틀거림","FinishEffect":"없음"},{"GroupID":80037,"Name":"샌즈 · 가볍게 인사","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":23,"HoldMs":900,"GapMs":250,"Notes":"취객·샌즈 전투 연출 초안. 태그와 시간은 자유롭게 조정 가능.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80038,"Name":"취객 · 1단계 아직 두 명으로 보여","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"자동","CPS":27,"HoldMs":1300,"GapMs":250,"Notes":"취객·샌즈 전투 연출 초안. 태그와 시간은 자유롭게 조정 가능.","ActorEffect":"비틀거림","FinishEffect":"없음"},{"GroupID":80039,"Name":"취객 · 2단계 시야가 돌아와","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"자동","CPS":27,"HoldMs":1300,"GapMs":250,"Notes":"취객·샌즈 전투 연출 초안. 태그와 시간은 자유롭게 조정 가능.","ActorEffect":"놀람","FinishEffect":"없음"},{"GroupID":80040,"Name":"취객 · 3단계 제이와 가업","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"자동","CPS":27,"HoldMs":1300,"GapMs":250,"Notes":"취객·샌즈 전투 연출 초안. 태그와 시간은 자유롭게 조정 가능.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80041,"Name":"취객 · 4단계 돌아온 손끝","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"자동","CPS":27,"HoldMs":1300,"GapMs":250,"Notes":"취객·샌즈 전투 연출 초안. 태그와 시간은 자유롭게 조정 가능.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80042,"Name":"취객 · 미용실에서 이어질 이야기","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"자동","CPS":27,"HoldMs":1500,"GapMs":250,"Notes":"전투에서는 해금·지급 연출 없이 귀환을 예고합니다. 소울 해금과 튜토리얼은 이후 미용실 대화에서 진행.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80043,"Name":"샌즈 · 첫 MISS 여유","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":23,"HoldMs":1500,"GapMs":250,"Notes":"첫 MISS와 함께 재생. 말하는 중에도 빈틈 게이지와 연타 진행.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80044,"Name":"샌즈 · 첫 명중 허세","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"자동","CPS":23,"HoldMs":1500,"GapMs":250,"Notes":"취객·샌즈 전투 연출 초안. 태그와 시간은 자유롭게 조정 가능.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80045,"Name":"샌즈 · 두 번째 MISS 농담","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":23,"HoldMs":1500,"GapMs":250,"Notes":"첫 MISS와 함께 재생. 말하는 중에도 빈틈 게이지와 연타 진행.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80046,"Name":"샌즈 · 두 번째 명중 동요","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"자동","CPS":23,"HoldMs":1500,"GapMs":250,"Notes":"취객·샌즈 전투 연출 초안. 태그와 시간은 자유롭게 조정 가능.","ActorEffect":"식은땀","FinishEffect":"없음"},{"GroupID":80047,"Name":"샌즈 · 세 번째 MISS 식은땀","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":23,"HoldMs":1500,"GapMs":250,"Notes":"첫 MISS와 함께 재생. 말하는 중에도 빈틈 게이지와 연타 진행.","ActorEffect":"식은땀","FinishEffect":"없음"},{"GroupID":80048,"Name":"샌즈 · 마지막 말","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"자동","CPS":23,"HoldMs":1500,"GapMs":250,"Notes":"취객·샌즈 전투 연출 초안. 태그와 시간은 자유롭게 조정 가능.","ActorEffect":"식은땀","FinishEffect":"소멸"},{"GroupID":80049,"Name":"좀비 · 끈질긴 공격","PlaybackMode":"무작위 한 줄","PauseCombat":false,"AdvanceMode":"자동","CPS":26,"HoldMs":1400,"GapMs":250,"Notes":"좀비 전투 전용. 기존 문자 효과 태그로 연출.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80050,"Name":"좀비 · 빈틈 농담","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":26,"HoldMs":1400,"GapMs":250,"Notes":"좀비 전투 전용. 기존 문자 효과 태그로 연출.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80051,"Name":"좀비 · 부활 완료 후 한마디","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":26,"HoldMs":1400,"GapMs":250,"Notes":"실제 부활 모션 완료 → 글자 시작 → 다음 대사 입력 후 전투 재개.","ActorEffect":"부활 후 대사","FinishEffect":"없음"},{"GroupID":80052,"Name":"좀비 · 재도전 휴업","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":26,"HoldMs":1400,"GapMs":250,"Notes":"좀비 전투 전용. 기존 문자 효과 태그로 연출.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80053,"Name":"좀비 · 끝까지 버티기","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":26,"HoldMs":1400,"GapMs":250,"Notes":"좀비 전투 전용. 기존 문자 효과 태그로 연출.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80054,"Name":"취준좀비 · 장식 붙이기 · 처음 부탁","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"미용 대사 연결에서 선택하는 부탁","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80055,"Name":"취준좀비 · 색·무늬 꾸미기 · 처음 부탁","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"미용 대사 연결에서 선택하는 부탁","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80056,"Name":"좀비 · 미용실 복귀","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"통합 프로토타입 미용실 대사","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80057,"Name":"좀비 · 연습 종료","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"통합 프로토타입 미용실 대사","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80058,"Name":"취객 · 불 켜진 미용실","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"통합 프로토타입 미용실 대사","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80059,"Name":"취객 · 돌아온 가업","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"통합 프로토타입 미용실 대사","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80060,"Name":"취객 · 잠깐의 외출","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"통합 프로토타입 미용실 대사","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80061,"Name":"샌즈 · 방문","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"통합 프로토타입 미용실 대사","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80062,"Name":"샌즈 · 형태 만들기 · 처음 부탁","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"미용 대사 연결에서 선택하는 부탁","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80063,"Name":"샌즈 · 장식 붙이기 · 처음 부탁","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"미용 대사 연결에서 선택하는 부탁","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80064,"Name":"샌즈 · 미용 만족","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"통합 프로토타입 미용실 대사","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80065,"Name":"샌즈 · 미용 보통","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"통합 프로토타입 미용실 대사","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80066,"Name":"샌즈 · 미용 실패","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"통합 프로토타입 미용실 대사","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80067,"Name":"샌즈 · 야차가 끝난 미용실","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"통합 프로토타입 미용실 대사","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80068,"Name":"취준좀비 · 색·무늬 꾸미기 · 자세한 부탁","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"미용 대사 연결에서 선택하는 부탁","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80069,"Name":"취준좀비 · 장식 붙이기 · 자세한 부탁","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"미용 대사 연결에서 선택하는 부탁","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80070,"Name":"샌즈 · 형태 만들기 · 자세한 부탁","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"미용 대사 연결에서 선택하는 부탁","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80071,"Name":"샌즈 · 색·무늬 꾸미기 · 처음 부탁","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"미용 대사 연결에서 선택하는 부탁","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80072,"Name":"샌즈 · 색·무늬 꾸미기 · 자세한 부탁","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"미용 대사 연결에서 선택하는 부탁","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80073,"Name":"샌즈 · 장식 붙이기 · 자세한 부탁","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"미용 대사 연결에서 선택하는 부탁","ActorEffect":"없음","FinishEffect":"없음"}]},{"name":"전투 대사 연결","keys":["TriggerID","MonsterID","PhaseID","EventType","PatternID","BeautyCondition","GroupID","HPThresholdPct","CooldownMs","MaxPerBattle","Enabled","Notes","EventCount"],"rows":[{"TriggerID":100001,"MonsterID":10001,"PhaseID":null,"EventType":"전투 시작","PatternID":null,"BeautyCondition":"미용 성공","GroupID":80016,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":false,"Notes":"기존 미용 분기 대사 보관. 현재는 전투 전용 공통 연결을 사용하며 등장·미용 흐름은 보류.","EventCount":null},{"TriggerID":100002,"MonsterID":10001,"PhaseID":null,"EventType":"공격 시작","PatternID":null,"BeautyCondition":"미용 성공","GroupID":80018,"HPThresholdPct":null,"CooldownMs":8000,"MaxPerBattle":0,"Enabled":false,"Notes":"기존 미용 분기 대사 보관. 현재는 전투 전용 공통 연결을 사용하며 등장·미용 흐름은 보류.","EventCount":null},{"TriggerID":100003,"MonsterID":10001,"PhaseID":null,"EventType":"몬스터 HP 이하","PatternID":null,"BeautyCondition":"미용 성공","GroupID":80020,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":false,"Notes":"기존 미용 분기 대사 보관. 현재는 전투 전용 공통 연결을 사용하며 등장·미용 흐름은 보류.","EventCount":null},{"TriggerID":100004,"MonsterID":10001,"PhaseID":null,"EventType":"플레이어 HP 이하","PatternID":null,"BeautyCondition":"미용 성공","GroupID":80022,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":false,"Notes":"기존 미용 분기 대사 보관. 현재는 전투 전용 공통 연결을 사용하며 등장·미용 흐름은 보류.","EventCount":null},{"TriggerID":100005,"MonsterID":10001,"PhaseID":null,"EventType":"승리","PatternID":null,"BeautyCondition":"미용 성공","GroupID":80026,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":false,"Notes":"기존 미용 분기 대사 보관. 현재는 전투 전용 공통 연결을 사용하며 등장·미용 흐름은 보류.","EventCount":null},{"TriggerID":100006,"MonsterID":10001,"PhaseID":null,"EventType":"패배","PatternID":null,"BeautyCondition":"미용 성공","GroupID":80027,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":false,"Notes":"기존 미용 분기 대사 보관. 현재는 전투 전용 공통 연결을 사용하며 등장·미용 흐름은 보류.","EventCount":null},{"TriggerID":100007,"MonsterID":10001,"PhaseID":null,"EventType":"전투 시작","PatternID":null,"BeautyCondition":"미용 실패","GroupID":80017,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":false,"Notes":"기존 미용 분기 대사 보관. 현재는 전투 전용 공통 연결을 사용하며 등장·미용 흐름은 보류.","EventCount":null},{"TriggerID":100008,"MonsterID":10001,"PhaseID":null,"EventType":"공격 시작","PatternID":null,"BeautyCondition":"미용 실패","GroupID":80019,"HPThresholdPct":null,"CooldownMs":8000,"MaxPerBattle":0,"Enabled":false,"Notes":"기존 미용 분기 대사 보관. 현재는 전투 전용 공통 연결을 사용하며 등장·미용 흐름은 보류.","EventCount":null},{"TriggerID":100009,"MonsterID":10001,"PhaseID":null,"EventType":"몬스터 HP 이하","PatternID":null,"BeautyCondition":"미용 실패","GroupID":80021,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":false,"Notes":"기존 미용 분기 대사 보관. 현재는 전투 전용 공통 연결을 사용하며 등장·미용 흐름은 보류.","EventCount":null},{"TriggerID":100010,"MonsterID":10001,"PhaseID":null,"EventType":"플레이어 HP 이하","PatternID":null,"BeautyCondition":"미용 실패","GroupID":80023,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":false,"Notes":"기존 미용 분기 대사 보관. 현재는 전투 전용 공통 연결을 사용하며 등장·미용 흐름은 보류.","EventCount":null},{"TriggerID":100011,"MonsterID":10001,"PhaseID":null,"EventType":"승리","PatternID":null,"BeautyCondition":"미용 실패","GroupID":80024,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":false,"Notes":"기존 미용 분기 대사 보관. 현재는 전투 전용 공통 연결을 사용하며 등장·미용 흐름은 보류.","EventCount":null},{"TriggerID":100012,"MonsterID":10001,"PhaseID":null,"EventType":"패배","PatternID":null,"BeautyCondition":"미용 실패","GroupID":80025,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":false,"Notes":"기존 미용 분기 대사 보관. 현재는 전투 전용 공통 연결을 사용하며 등장·미용 흐름은 보류.","EventCount":null},{"TriggerID":100013,"MonsterID":10002,"PhaseID":1,"EventType":"전투 시작","PatternID":null,"BeautyCondition":"공통","GroupID":80036,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":true,"Notes":"사건 발생 시 한 번 재생.","EventCount":null},{"TriggerID":100014,"MonsterID":10003,"PhaseID":1,"EventType":"전투 시작","PatternID":null,"BeautyCondition":"공통","GroupID":80037,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":true,"Notes":"사건 발생 시 한 번 재생.","EventCount":null},{"TriggerID":100015,"MonsterID":10002,"PhaseID":1,"EventType":"빈틈공격 성공","PatternID":null,"BeautyCondition":"공통","GroupID":80038,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":true,"Notes":"해당 페이즈에서 명중한 빈틈이 끝난 뒤 한 번. 대사 후 다음 페이즈 또는 승리.","EventCount":null},{"TriggerID":100016,"MonsterID":10002,"PhaseID":2,"EventType":"빈틈공격 성공","PatternID":null,"BeautyCondition":"공통","GroupID":80039,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":true,"Notes":"해당 페이즈에서 명중한 빈틈이 끝난 뒤 한 번. 대사 후 다음 페이즈 또는 승리.","EventCount":null},{"TriggerID":100017,"MonsterID":10002,"PhaseID":3,"EventType":"빈틈공격 성공","PatternID":null,"BeautyCondition":"공통","GroupID":80040,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":true,"Notes":"해당 페이즈에서 명중한 빈틈이 끝난 뒤 한 번. 대사 후 다음 페이즈 또는 승리.","EventCount":null},{"TriggerID":100018,"MonsterID":10002,"PhaseID":4,"EventType":"빈틈공격 성공","PatternID":null,"BeautyCondition":"공통","GroupID":80041,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":true,"Notes":"해당 페이즈에서 명중한 빈틈이 끝난 뒤 한 번. 대사 후 다음 페이즈 또는 승리.","EventCount":null},{"TriggerID":100019,"MonsterID":10002,"PhaseID":4,"EventType":"승리","PatternID":null,"BeautyCondition":"공통","GroupID":80042,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":true,"Notes":"사건 발생 시 한 번 재생.","EventCount":null},{"TriggerID":100020,"MonsterID":10003,"PhaseID":1,"EventType":"빈틈공격 MISS","PatternID":null,"BeautyCondition":"공통","GroupID":80043,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":true,"Notes":"첫 MISS 순간 대사 시작. 같은 빈틈의 후속 MISS에는 재시작하지 않음. 전투 정지 없음.","EventCount":1},{"TriggerID":100021,"MonsterID":10003,"PhaseID":1,"EventType":"빈틈공격 성공","PatternID":null,"BeautyCondition":"공통","GroupID":80044,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":true,"Notes":"1번째 명중한 빈틈 종료 후 한 번 재생. 연타 개수는 세지 않음.","EventCount":1},{"TriggerID":100022,"MonsterID":10003,"PhaseID":2,"EventType":"빈틈공격 MISS","PatternID":null,"BeautyCondition":"공통","GroupID":80045,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":true,"Notes":"첫 MISS 순간 대사 시작. 같은 빈틈의 후속 MISS에는 재시작하지 않음. 전투 정지 없음.","EventCount":1},{"TriggerID":100023,"MonsterID":10003,"PhaseID":2,"EventType":"빈틈공격 성공","PatternID":null,"BeautyCondition":"공통","GroupID":80046,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":true,"Notes":"1번째 명중한 빈틈 종료 후 한 번 재생. 연타 개수는 세지 않음.","EventCount":1},{"TriggerID":100024,"MonsterID":10003,"PhaseID":3,"EventType":"빈틈공격 MISS","PatternID":null,"BeautyCondition":"공통","GroupID":80047,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":true,"Notes":"첫 MISS 순간 대사 시작. 같은 빈틈의 후속 MISS에는 재시작하지 않음. 전투 정지 없음.","EventCount":1},{"TriggerID":100025,"MonsterID":10003,"PhaseID":3,"EventType":"빈틈공격 성공","PatternID":null,"BeautyCondition":"공통","GroupID":80048,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":true,"Notes":"1번째 명중한 빈틈 종료 후 한 번 재생. 연타 개수는 세지 않음.","EventCount":1},{"TriggerID":100026,"MonsterID":10001,"PhaseID":null,"EventType":"공격 시작","PatternID":null,"BeautyCondition":"공통","GroupID":80049,"HPThresholdPct":null,"CooldownMs":9000,"MaxPerBattle":0,"Enabled":true,"Notes":"등장·미용과 분리한 전투 대사.","EventCount":null},{"TriggerID":100027,"MonsterID":10001,"PhaseID":null,"EventType":"빈틈 발생","PatternID":null,"BeautyCondition":"공통","GroupID":80050,"HPThresholdPct":null,"CooldownMs":12000,"MaxPerBattle":2,"Enabled":true,"Notes":"등장·미용과 분리한 전투 대사.","EventCount":null},{"TriggerID":100028,"MonsterID":10001,"PhaseID":null,"EventType":"승리","PatternID":null,"BeautyCondition":"공통","GroupID":80052,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":true,"Notes":"등장·미용과 분리한 전투 대사.","EventCount":null},{"TriggerID":100029,"MonsterID":10001,"PhaseID":null,"EventType":"패배","PatternID":null,"BeautyCondition":"공통","GroupID":80053,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":true,"Notes":"등장·미용과 분리한 전투 대사.","EventCount":null}]},{"name":"문자 효과 규칙","keys":["Tag","Example","Description"],"rows":[{"Tag":"color","Example":"&lt;color=#FFD166&gt;으하하하!&lt;/color&gt;","Description":"글자색을 바꿉니다. #RRGGBB 또는 white/red 등 기본 색 이름을 씁니다."},{"Tag":"shake","Example":"&lt;shake=2 speed=16 dur=0.5&gt;어이쿠!&lt;/shake&gt;","Description":"글자를 떨리게 합니다. 2는 흔들림 크기, speed는 속도, dur는 지속 초입니다. dur 생략/0이면 대사 동안 계속합니다."},{"Tag":"wave","Example":"&lt;wave=3 speed=5&gt;오랜만이구먼!&lt;/wave&gt;","Description":"글자가 물결처럼 위아래로 움직입니다. 3은 높이, speed는 움직이는 속도입니다."},{"Tag":"wait","Example":"잠깐,&lt;wait=0.4&gt; 우리... 친구잖아?","Description":"이 위치에서 타이핑을 0.4초 쉽니다. 전투 시간을 멈출지는 대화 그룹에서 정합니다."},{"Tag":"cps","Example":"&lt;cps=16&gt;눈치 빠른 애송이들이...&lt;/cps&gt;","Description":"이 구간만 초당 글자 수를 바꿉니다. 0은 즉시 표시입니다."},{"Tag":"speed","Example":"&lt;speed=0.7&gt;천천히&lt;/speed&gt;","Description":"기본 타이핑 속도에 곱합니다. 0.7은 더 느리고 2는 두 배입니다."},{"Tag":"size","Example":"&lt;size=24&gt;으하하하!&lt;/size&gt;","Description":"이 구간의 글자 크기입니다. 화면 픽셀 기준이며 기본 크기는 17입니다."},{"Tag":"pulse","Example":"&lt;pulse=1.1 speed=7&gt;으하하하!&lt;/pulse&gt;","Description":"글자가 1.1배까지 가볍게 커졌다 작아집니다."},{"Tag":"fade","Example":"&lt;fade=0.3&gt;서서히&lt;/fade&gt;","Description":"각 글자가 나타난 뒤 0.3초 동안 천천히 선명해집니다."},{"Tag":"rainbow","Example":"&lt;rainbow=0.6 speed=3&gt;반짝이는 색&lt;/rainbow&gt;","Description":"시간에 따라 글자색을 무지개색으로 바꿉니다. 값은 색의 강도 0~1입니다."},{"Tag":"중첩","Example":"&lt;color=#8BE9FD&gt;&lt;shake=2&gt;친구잖아..?&lt;/shake&gt;&lt;/color&gt;","Description":"효과는 겹쳐 쓸 수 있습니다. 연 태그는 반대 순서로 닫습니다."},{"Tag":"캐릭터 연출","Example":"대화 그룹 → ActorEffect / FinishEffect","Description":"ActorEffect: 비틀거림·놀람·식은땀·부활 후 대사. 부활 후 대사는 모션이 끝나야 글자가 시작됩니다. FinishEffect: 대사 이후 소멸 등 마무리 연출."},{"Tag":"말투 참고","Example":"https://undertale.com/alarmclock/sans/","Description":"샌즈 말투는 공식 대사에서 짧은 말끝·뜸 들임·건조한 농담을 참고. 전투 대사는 사용자 제시 문장과 새 창작 문장으로 구성."}]},{"name":"미용 대사 연결","keys":["MonsterID","Stage","RequestGroupID","DetailGroupID"],"rows":[{"MonsterID":10001,"Stage":"cut","RequestGroupID":80002,"DetailGroupID":80003},{"MonsterID":10001,"Stage":"draw","RequestGroupID":80055,"DetailGroupID":80068},{"MonsterID":10001,"Stage":"attach","RequestGroupID":80054,"DetailGroupID":80069},{"MonsterID":10003,"Stage":"cut","RequestGroupID":80062,"DetailGroupID":80070},{"MonsterID":10003,"Stage":"draw","RequestGroupID":80071,"DetailGroupID":80072},{"MonsterID":10003,"Stage":"attach","RequestGroupID":80063,"DetailGroupID":80073}]}]},"drafts":[{"MonsterID":10100,"PhaseID":1},{"MonsterID":10100,"PhaseID":2},{"MonsterID":10100,"PhaseID":3}]}</version>
+<version xmlns="urn:yachacha:table-version">{"format":1,"version":"2026-10-17_02-47-36","parentVersion":"2026-10-17_02-33-50","intent":"대사 담당자가 검토한 비마왕부하 대사의 문장·화자·순서·삭제 및 추가를 반영하고, 기존 마왕 부하의 21문장을 보존해 같은 버전에서 편집하게 했습니다. 담당자 파일과 겹친 그룹80085→80089, 문장900133~900136→900140~900143만 분리했고 샌즈 전투 승리 후 대사도 연결했습니다. 전투·미용·보상 수치 변경은 없습니다.","snapshot":{"sheets":[{"name":"공격 만들기","keys":["PatternID","Name","RangeMode","ShapePoolID","TilePath","HitMin","HitMax","GapMinMs","GapMaxMs","ResponseMs","ExtraMinMs","ExtraMaxMs","AvoidRepeat","CanDefend","BreakTiles","Notes"],"rows":[{"PatternID":20001,"Name":"랜덤 단일","RangeMode":"범위 반복","ShapePoolID":60001,"TilePath":null,"HitMin":1,"HitMax":1,"GapMinMs":null,"GapMaxMs":null,"ResponseMs":null,"ExtraMinMs":0,"ExtraMaxMs":0,"AvoidRepeat":true,"CanDefend":true,"BreakTiles":false,"Notes":"범위 하나를 뽑아 1회 타격"},{"PatternID":30001,"Name":"랜덤 2~5연속","RangeMode":"범위 반복","ShapePoolID":60001,"TilePath":null,"HitMin":2,"HitMax":5,"GapMinMs":300,"GapMaxMs":600,"ResponseMs":null,"ExtraMinMs":0,"ExtraMaxMs":0,"AvoidRepeat":true,"CanDefend":true,"BreakTiles":false,"Notes":"모든 파란 숫자 예고 후 같은 박자로 타격"},{"PatternID":40001,"Name":"순차 타일","RangeMode":"경로 순차","ShapePoolID":70001,"TilePath":null,"HitMin":null,"HitMax":null,"GapMinMs":300,"GapMaxMs":300,"ResponseMs":null,"ExtraMinMs":0,"ExtraMaxMs":0,"AvoidRepeat":false,"CanDefend":true,"BreakTiles":false,"Notes":"경로 하나 선택 → 타일별 예고 → 모션 1회·순차 타격"},{"PatternID":20002,"Name":"엇박 단일","RangeMode":"범위 반복","ShapePoolID":60001,"TilePath":null,"HitMin":1,"HitMax":1,"GapMinMs":null,"GapMaxMs":null,"ResponseMs":null,"ExtraMinMs":500,"ExtraMaxMs":500,"AvoidRepeat":true,"CanDefend":true,"BreakTiles":false,"Notes":"단일 공격에 500ms 추가 대기"},{"PatternID":20003,"Name":"방어 불가 · 전체 타일 제외","RangeMode":"범위 반복","ShapePoolID":60003,"TilePath":null,"HitMin":1,"HitMax":1,"GapMinMs":null,"GapMaxMs":null,"ResponseMs":null,"ExtraMinMs":0,"ExtraMaxMs":0,"AvoidRepeat":true,"CanDefend":false,"BreakTiles":false,"Notes":"후보 1~8 사용. 전체 9칸 동시 공격 제외. 패링·가드 불가"},{"PatternID":20010,"Name":"타일 파괴 단일","RangeMode":"범위 반복","ShapePoolID":60001,"TilePath":null,"HitMin":1,"HitMax":1,"GapMinMs":null,"GapMaxMs":null,"ResponseMs":null,"ExtraMinMs":0,"ExtraMaxMs":0,"AvoidRepeat":true,"CanDefend":true,"BreakTiles":true,"Notes":"기능 예시. 이 속성은 다른 공격에도 켤 수 있음"},{"PatternID":40002,"Name":"ㄹ자 9칸 순차","RangeMode":"경로 순차","ShapePoolID":null,"TilePath":"1,4,7,8,5,2,3,6,9","HitMin":null,"HitMax":null,"GapMinMs":300,"GapMaxMs":300,"ResponseMs":null,"ExtraMinMs":0,"ExtraMaxMs":0,"AvoidRepeat":false,"CanDefend":true,"BreakTiles":false,"Notes":"경로만 입력. 9타 자동 결정"},{"PatternID":40003,"Name":"대각선 3칸 순차","RangeMode":"경로 순차","ShapePoolID":null,"TilePath":"1,5,9","HitMin":null,"HitMax":null,"GapMinMs":300,"GapMaxMs":300,"ResponseMs":null,"ExtraMinMs":0,"ExtraMaxMs":0,"AvoidRepeat":false,"CanDefend":true,"BreakTiles":false,"Notes":"1→5→9 예고 완료 후 연속 타격"},{"PatternID":50001,"Name":"샌즈 상대 밀치기","RangeMode":"밀친 위치","ShapePoolID":null,"TilePath":null,"HitMin":null,"HitMax":null,"GapMinMs":null,"GapMaxMs":null,"ResponseMs":550,"ExtraMinMs":0,"ExtraMaxMs":0,"AvoidRepeat":false,"CanDefend":true,"BreakTiles":false,"Notes":"방향·시간은 이동·연출에 작성. 수치·방어 임시"},{"PatternID":20020,"Name":"샌즈 블래스터","RangeMode":"범위 반복","ShapePoolID":60001,"TilePath":null,"HitMin":1,"HitMax":1,"GapMinMs":null,"GapMaxMs":null,"ResponseMs":null,"ExtraMinMs":0,"ExtraMaxMs":0,"AvoidRepeat":true,"CanDefend":true,"BreakTiles":false,"Notes":"랜덤 단일 + 이동 없음 + 레이저 연출. 타격 1회"},{"PatternID":30002,"Name":"랜덤 2~3연속","RangeMode":"범위 반복","ShapePoolID":60001,"TilePath":null,"HitMin":2,"HitMax":3,"GapMinMs":300,"GapMaxMs":600,"ResponseMs":null,"ExtraMinMs":0,"ExtraMaxMs":0,"AvoidRepeat":true,"CanDefend":true,"BreakTiles":false,"Notes":"초반 몬스터용 예시. 30001 복사 후 횟수만 변경."},{"PatternID":30003,"Name":"랜덤 4~5연속","RangeMode":"범위 반복","ShapePoolID":60001,"TilePath":null,"HitMin":4,"HitMax":5,"GapMinMs":300,"GapMaxMs":600,"ResponseMs":null,"ExtraMinMs":0,"ExtraMaxMs":0,"AvoidRepeat":true,"CanDefend":true,"BreakTiles":false,"Notes":"후반 몬스터용 예시. 별도 ID로 독립 참조."},{"PatternID":20004,"Name":"단일 · 후보 1~4","RangeMode":"범위 반복","ShapePoolID":60002,"TilePath":null,"HitMin":1,"HitMax":1,"GapMinMs":null,"GapMaxMs":null,"ResponseMs":null,"ExtraMinMs":0,"ExtraMaxMs":0,"AvoidRepeat":true,"CanDefend":true,"BreakTiles":false,"Notes":"20001과 같은 단일, 범위 풀만 60002로 변경."},{"PatternID":20011,"Name":"느긋한 엇박 단일","RangeMode":"범위 반복","ShapePoolID":60001,"TilePath":null,"HitMin":1,"HitMax":1,"GapMinMs":null,"GapMaxMs":null,"ResponseMs":882,"ExtraMinMs":588,"ExtraMaxMs":588,"AvoidRepeat":true,"CanDefend":true,"BreakTiles":false,"Notes":"기존 엇박의 시간만 다른 변형. 필요한 몬스터·페이즈에서 재사용하세요."},{"PatternID":20012,"Name":"빠른 엇박 단일","RangeMode":"범위 반복","ShapePoolID":60001,"TilePath":null,"HitMin":1,"HitMax":1,"GapMinMs":null,"GapMaxMs":null,"ResponseMs":652,"ExtraMinMs":435,"ExtraMaxMs":435,"AvoidRepeat":true,"CanDefend":true,"BreakTiles":false,"Notes":"기존 엇박의 시간만 다른 변형. 필요한 몬스터·페이즈에서 재사용하세요."},{"PatternID":20013,"Name":"더 빠른 엇박 단일","RangeMode":"범위 반복","ShapePoolID":60001,"TilePath":null,"HitMin":1,"HitMax":1,"GapMinMs":null,"GapMaxMs":null,"ResponseMs":577,"ExtraMinMs":385,"ExtraMaxMs":385,"AvoidRepeat":true,"CanDefend":true,"BreakTiles":false,"Notes":"기존 엇박의 시간만 다른 변형. 필요한 몬스터·페이즈에서 재사용하세요."}]},{"name":"이동·연출","keys":["PatternID","PatternName","MoveType","MoveSpeed","MoveDistance","MotionKey","Effect","SoundKey","EffectMs","PushDirection","PushTiles","PushLeadMs","PushMoveMs","Notes"],"rows":[{"PatternID":50001,"PatternName":"샌즈 상대 밀치기","MoveType":"없음","MoveSpeed":null,"MoveDistance":null,"MotionKey":null,"Effect":"기본","SoundKey":null,"EffectMs":null,"PushDirection":"좌우 무작위","PushTiles":1,"PushLeadMs":300,"PushMoveMs":150,"Notes":"예고 300 + 강제이동 150 + 탈출 550ms. 임시값."},{"PatternID":20020,"PatternName":"샌즈 블래스터","MoveType":"없음","MoveSpeed":null,"MoveDistance":null,"MotionKey":null,"Effect":"블래스터 레이저","SoundKey":null,"EffectMs":500,"PushDirection":null,"PushTiles":null,"PushLeadMs":null,"PushMoveMs":null,"Notes":"모션·소리·레이저 프리셋 연결 필요. 표시 500ms 임시."}]},{"name":"몬스터 사용 패턴","keys":["MonsterID","Name","PhaseID","PatternID","PatternName","HitDamage","Weight","Enabled","Notes"],"rows":[{"MonsterID":10001,"Name":"취준좀비","PhaseID":1,"PatternID":20001,"PatternName":"랜덤 단일","HitDamage":20,"Weight":70,"Enabled":true,"Notes":"단일 공격: 70"},{"MonsterID":10001,"Name":"취준좀비","PhaseID":1,"PatternID":40001,"PatternName":"순차 타일","HitDamage":20,"Weight":30,"Enabled":true,"Notes":"순차 공격: 30"},{"MonsterID":10001,"Name":"취준좀비","PhaseID":2,"PatternID":20001,"PatternName":"랜덤 단일","HitDamage":20,"Weight":60,"Enabled":true,"Notes":"단일 공격: 60"},{"MonsterID":10001,"Name":"취준좀비","PhaseID":2,"PatternID":40001,"PatternName":"순차 타일","HitDamage":20,"Weight":40,"Enabled":true,"Notes":"순차 공격: 40"},{"MonsterID":10002,"Name":"취객","PhaseID":1,"PatternID":20001,"PatternName":"랜덤 단일","HitDamage":1,"Weight":40,"Enabled":true,"Notes":"단일 공격: 40"},{"MonsterID":10002,"Name":"취객","PhaseID":1,"PatternID":20011,"PatternName":"느긋한 엇박 단일","HitDamage":1,"Weight":60,"Enabled":true,"Notes":"술 깨기 1/4. 기존 패턴의 피할 시간·엇박 추가 시간으로 속도 조절."},{"MonsterID":10002,"Name":"취객","PhaseID":2,"PatternID":20001,"PatternName":"랜덤 단일","HitDamage":1,"Weight":40,"Enabled":true,"Notes":"단일 공격: 40"},{"MonsterID":10002,"Name":"취객","PhaseID":2,"PatternID":20002,"PatternName":"엇박 단일","HitDamage":1,"Weight":60,"Enabled":true,"Notes":"술 깨기 2/4. 기존 패턴의 피할 시간·엇박 추가 시간으로 속도 조절."},{"MonsterID":10002,"Name":"취객","PhaseID":3,"PatternID":20001,"PatternName":"랜덤 단일","HitDamage":1,"Weight":40,"Enabled":true,"Notes":"단일 공격: 40"},{"MonsterID":10002,"Name":"취객","PhaseID":3,"PatternID":20012,"PatternName":"빠른 엇박 단일","HitDamage":1,"Weight":60,"Enabled":true,"Notes":"술 깨기 3/4. 기존 패턴의 피할 시간·엇박 추가 시간으로 속도 조절."},{"MonsterID":10002,"Name":"취객","PhaseID":4,"PatternID":20001,"PatternName":"랜덤 단일","HitDamage":1,"Weight":40,"Enabled":true,"Notes":"단일 공격: 40"},{"MonsterID":10002,"Name":"취객","PhaseID":4,"PatternID":20013,"PatternName":"더 빠른 엇박 단일","HitDamage":1,"Weight":60,"Enabled":true,"Notes":"술 깨기 4/4. 기존 패턴의 피할 시간·엇박 추가 시간으로 속도 조절."},{"MonsterID":10003,"Name":"샌즈","PhaseID":1,"PatternID":50001,"PatternName":"샌즈 상대 밀치기","HitDamage":20,"Weight":50,"Enabled":true,"Notes":"대사 진행 시험용 초기값: 밀치기/블래스터 각 50, 피해 20. 조절 가능."},{"MonsterID":10001,"Name":"취준좀비","PhaseID":1,"PatternID":40003,"PatternName":"대각선 3칸 순차","HitDamage":20,"Weight":0,"Enabled":false,"Notes":"1→5→9 예시. 기존 70:30 비중 유지 위해 비활성."},{"MonsterID":10003,"Name":"샌즈","PhaseID":1,"PatternID":20020,"PatternName":"샌즈 블래스터","HitDamage":20,"Weight":50,"Enabled":true,"Notes":"대사 진행 시험용 초기값: 밀치기/블래스터 각 50, 피해 20. 조절 가능."},{"MonsterID":10001,"Name":"취준좀비","PhaseID":1,"PatternID":30002,"PatternName":"랜덤 2~3연속","HitDamage":20,"Weight":0,"Enabled":false,"Notes":"연결 예시: 초반 2~3연속. 활성 비중은 유지."},{"MonsterID":10001,"Name":"취준좀비","PhaseID":2,"PatternID":30003,"PatternName":"랜덤 4~5연속","HitDamage":20,"Weight":0,"Enabled":false,"Notes":"연결 예시: 후반 4~5연속. 필요하면 켜고 비중 입력."},{"MonsterID":10001,"Name":"취준좀비","PhaseID":1,"PatternID":20004,"PatternName":"단일 · 후보 1~4","HitDamage":20,"Weight":0,"Enabled":false,"Notes":"연결 예시: 후보 1~4 풀 사용. 필요할 때 활성화."},{"MonsterID":10003,"Name":"샌즈","PhaseID":2,"PatternID":50001,"PatternName":"샌즈 상대 밀치기","HitDamage":20,"Weight":50,"Enabled":true,"Notes":"대사 진행 시험용 초기값: 밀치기/블래스터 각 50, 피해 20. 조절 가능."},{"MonsterID":10003,"Name":"샌즈","PhaseID":2,"PatternID":20020,"PatternName":"샌즈 블래스터","HitDamage":20,"Weight":50,"Enabled":true,"Notes":"대사 진행 시험용 초기값: 밀치기/블래스터 각 50, 피해 20. 조절 가능."},{"MonsterID":10003,"Name":"샌즈","PhaseID":3,"PatternID":50001,"PatternName":"샌즈 상대 밀치기","HitDamage":20,"Weight":50,"Enabled":true,"Notes":"대사 진행 시험용 초기값: 밀치기/블래스터 각 50, 피해 20. 조절 가능."},{"MonsterID":10003,"Name":"샌즈","PhaseID":3,"PatternID":20020,"PatternName":"샌즈 블래스터","HitDamage":20,"Weight":50,"Enabled":true,"Notes":"대사 진행 시험용 초기값: 밀치기/블래스터 각 50, 피해 20. 조절 가능."}]},{"name":"몬스터 페이즈","keys":["MonsterID","Name","PhaseID","IsInitial","MaxHP","GaugeMax","ParryGain","GuardGain","DodgeGain","RecoveryMs","AttackSpeed","TransitionTrigger","NextPhaseID","PlayerDodgeMissCount","EntryDialogueGroupID","PauseForEntryDialogue","DesignStatus","OpeningDamageDisplay"],"rows":[{"MonsterID":10001,"Name":"취준좀비","PhaseID":1,"IsInitial":true,"MaxHP":1000,"GaugeMax":100,"ParryGain":50,"GuardGain":0,"DodgeGain":15,"RecoveryMs":800,"AttackSpeed":1,"TransitionTrigger":"HP 0","NextPhaseID":2,"PlayerDodgeMissCount":0,"EntryDialogueGroupID":null,"PauseForEntryDialogue":true,"DesignStatus":"페이즈 규칙 확정·수치 임시","OpeningDamageDisplay":null},{"MonsterID":10001,"Name":"취준좀비","PhaseID":2,"IsInitial":false,"MaxHP":300,"GaugeMax":100,"ParryGain":50,"GuardGain":0,"DodgeGain":15,"RecoveryMs":800,"AttackSpeed":1.5,"TransitionTrigger":"없음","NextPhaseID":null,"PlayerDodgeMissCount":0,"EntryDialogueGroupID":80051,"PauseForEntryDialogue":true,"DesignStatus":"HP 300 부활. 실제 부활 모션이 끝난 뒤 유머 대사, 입력 후 전투 재개.","OpeningDamageDisplay":null},{"MonsterID":10002,"Name":"취객","PhaseID":1,"IsInitial":true,"MaxHP":750,"GaugeMax":100,"ParryGain":50,"GuardGain":0,"DodgeGain":15,"RecoveryMs":1000,"AttackSpeed":1,"TransitionTrigger":"빈틈공격 성공","NextPhaseID":2,"PlayerDodgeMissCount":0,"EntryDialogueGroupID":null,"PauseForEntryDialogue":false,"DesignStatus":"술 깨기 1/4. 단계당 HP 750. 명중한 빈틈 종료 → 대사 → 다음 페이즈. 엇박 20011.","OpeningDamageDisplay":null},{"MonsterID":10002,"Name":"취객","PhaseID":2,"IsInitial":false,"MaxHP":750,"GaugeMax":100,"ParryGain":50,"GuardGain":0,"DodgeGain":15,"RecoveryMs":1000,"AttackSpeed":1,"TransitionTrigger":"빈틈공격 성공","NextPhaseID":3,"PlayerDodgeMissCount":0,"EntryDialogueGroupID":null,"PauseForEntryDialogue":false,"DesignStatus":"술 깨기 2/4. 단계당 HP 750. 명중한 빈틈 종료 → 대사 → 다음 페이즈. 엇박 20002.","OpeningDamageDisplay":null},{"MonsterID":10002,"Name":"취객","PhaseID":3,"IsInitial":false,"MaxHP":750,"GaugeMax":100,"ParryGain":50,"GuardGain":0,"DodgeGain":15,"RecoveryMs":1000,"AttackSpeed":1,"TransitionTrigger":"빈틈공격 성공","NextPhaseID":4,"PlayerDodgeMissCount":0,"EntryDialogueGroupID":null,"PauseForEntryDialogue":false,"DesignStatus":"술 깨기 3/4. 단계당 HP 750. 명중한 빈틈 종료 → 대사 → 다음 페이즈. 엇박 20012.","OpeningDamageDisplay":null},{"MonsterID":10002,"Name":"취객","PhaseID":4,"IsInitial":false,"MaxHP":750,"GaugeMax":100,"ParryGain":50,"GuardGain":0,"DodgeGain":15,"RecoveryMs":1000,"AttackSpeed":1,"TransitionTrigger":"빈틈공격 성공","NextPhaseID":null,"PlayerDodgeMissCount":0,"EntryDialogueGroupID":null,"PauseForEntryDialogue":false,"DesignStatus":"술 깨기 4/4. 단계당 HP 750. 명중한 빈틈 종료 → 대사 → 전투 승리. 엇박 20013.","OpeningDamageDisplay":null},{"MonsterID":10003,"Name":"샌즈","PhaseID":1,"IsInitial":true,"MaxHP":1,"GaugeMax":100,"ParryGain":50,"GuardGain":0,"DodgeGain":15,"RecoveryMs":800,"AttackSpeed":1,"TransitionTrigger":"HP 0","NextPhaseID":2,"PlayerDodgeMissCount":1,"EntryDialogueGroupID":null,"PauseForEntryDialogue":true,"DesignStatus":"첫 빈틈의 첫 MISS부터 대사(정지 없음). 다음 빈틈은 999999 연타 표시, 종료 후 명중 대사·전환.","OpeningDamageDisplay":999999},{"MonsterID":10003,"Name":"샌즈","PhaseID":2,"IsInitial":false,"MaxHP":1,"GaugeMax":100,"ParryGain":50,"GuardGain":0,"DodgeGain":15,"RecoveryMs":750,"AttackSpeed":1.2,"TransitionTrigger":"HP 0","NextPhaseID":3,"PlayerDodgeMissCount":1,"EntryDialogueGroupID":null,"PauseForEntryDialogue":true,"DesignStatus":"첫 빈틈의 첫 MISS부터 대사(정지 없음). 다음 빈틈은 999999 연타 표시, 종료 후 명중 대사·전환.","OpeningDamageDisplay":999999},{"MonsterID":10003,"Name":"샌즈","PhaseID":3,"IsInitial":false,"MaxHP":1,"GaugeMax":100,"ParryGain":50,"GuardGain":0,"DodgeGain":15,"RecoveryMs":700,"AttackSpeed":1.5,"TransitionTrigger":"HP 0","NextPhaseID":null,"PlayerDodgeMissCount":1,"EntryDialogueGroupID":null,"PauseForEntryDialogue":false,"DesignStatus":"첫 빈틈의 첫 MISS부터 대사(정지 없음). 다음 빈틈은 999999 연타 표시, 종료 후 명중 대사·전환.","OpeningDamageDisplay":999999},{"MonsterID":10100,"Name":"마왕","PhaseID":1,"IsInitial":true,"MaxHP":null,"GaugeMax":null,"ParryGain":null,"GuardGain":null,"DodgeGain":null,"RecoveryMs":null,"AttackSpeed":null,"TransitionTrigger":"미정","NextPhaseID":2,"PlayerDodgeMissCount":0,"EntryDialogueGroupID":null,"PauseForEntryDialogue":true,"DesignStatus":"전환 조건·HP·패턴 미정","OpeningDamageDisplay":null},{"MonsterID":10100,"Name":"마왕","PhaseID":2,"IsInitial":false,"MaxHP":null,"GaugeMax":null,"ParryGain":null,"GuardGain":null,"DodgeGain":null,"RecoveryMs":null,"AttackSpeed":null,"TransitionTrigger":"미정","NextPhaseID":3,"PlayerDodgeMissCount":0,"EntryDialogueGroupID":null,"PauseForEntryDialogue":true,"DesignStatus":"전환 조건·HP·패턴 미정","OpeningDamageDisplay":null},{"MonsterID":10100,"Name":"마왕","PhaseID":3,"IsInitial":false,"MaxHP":null,"GaugeMax":null,"ParryGain":null,"GuardGain":null,"DodgeGain":null,"RecoveryMs":null,"AttackSpeed":null,"TransitionTrigger":"없음","NextPhaseID":null,"PlayerDodgeMissCount":0,"EntryDialogueGroupID":null,"PauseForEntryDialogue":true,"DesignStatus":"전환 조건·HP·패턴 미정","OpeningDamageDisplay":null}]},{"name":"범위 풀","keys":["ShapePoolID","Candidate","SelectMode","Tiles","Weight","Enabled","Notes"],"rows":[{"ShapePoolID":60001,"Candidate":1,"SelectMode":"플레이어 행","Tiles":null,"Weight":25,"Enabled":true,"Notes":"현재 플레이어 행에 맞는 1개 선택"},{"ShapePoolID":60001,"Candidate":2,"SelectMode":"플레이어 열","Tiles":null,"Weight":25,"Enabled":true,"Notes":"현재 플레이어 열에 맞는 1개 선택"},{"ShapePoolID":60001,"Candidate":3,"SelectMode":"직접 입력","Tiles":"1,2,4,5","Weight":5,"Enabled":true,"Notes":"사각형"},{"ShapePoolID":60001,"Candidate":4,"SelectMode":"직접 입력","Tiles":"2,3,5,6","Weight":5,"Enabled":true,"Notes":"사각형"},{"ShapePoolID":60001,"Candidate":5,"SelectMode":"직접 입력","Tiles":"4,5,7,8","Weight":5,"Enabled":true,"Notes":"사각형"},{"ShapePoolID":60001,"Candidate":6,"SelectMode":"직접 입력","Tiles":"5,6,8,9","Weight":5,"Enabled":true,"Notes":"사각형"},{"ShapePoolID":60001,"Candidate":7,"SelectMode":"직접 입력","Tiles":"2,4,5,6,8","Weight":10,"Enabled":true,"Notes":"십자선"},{"ShapePoolID":60001,"Candidate":8,"SelectMode":"직접 입력","Tiles":"1,3,5,7,9","Weight":10,"Enabled":true,"Notes":"X자"},{"ShapePoolID":60001,"Candidate":9,"SelectMode":"직접 입력","Tiles":"1,2,3,4,5,6,7,8,9","Weight":10,"Enabled":true,"Notes":"타일 전체"},{"ShapePoolID":60002,"Candidate":1,"SelectMode":"플레이어 행","Tiles":null,"Weight":25,"Enabled":true,"Notes":"현재 플레이어 행에 맞는 1개 선택"},{"ShapePoolID":60002,"Candidate":2,"SelectMode":"플레이어 열","Tiles":null,"Weight":25,"Enabled":true,"Notes":"현재 플레이어 열에 맞는 1개 선택"},{"ShapePoolID":60002,"Candidate":3,"SelectMode":"직접 입력","Tiles":"1,2,4,5","Weight":5,"Enabled":true,"Notes":"사각형"},{"ShapePoolID":60002,"Candidate":4,"SelectMode":"직접 입력","Tiles":"2,3,5,6","Weight":5,"Enabled":true,"Notes":"사각형"},{"ShapePoolID":70001,"Candidate":1,"SelectMode":"플레이어 행","Tiles":null,"Weight":33,"Enabled":true,"Notes":"현재 플레이어 행 선택"},{"ShapePoolID":70001,"Candidate":2,"SelectMode":"플레이어 열","Tiles":null,"Weight":33,"Enabled":true,"Notes":"현재 플레이어 열 선택"},{"ShapePoolID":70001,"Candidate":3,"SelectMode":"직접 입력","Tiles":"3,5,7","Weight":17,"Enabled":true,"Notes":"대각선"},{"ShapePoolID":70001,"Candidate":4,"SelectMode":"직접 입력","Tiles":"1,5,9","Weight":17,"Enabled":true,"Notes":"대각선"},{"ShapePoolID":60003,"Candidate":1,"SelectMode":"플레이어 행","Tiles":null,"Weight":25,"Enabled":true,"Notes":"현재 플레이어 행에 맞는 1개 선택"},{"ShapePoolID":60003,"Candidate":2,"SelectMode":"플레이어 열","Tiles":null,"Weight":25,"Enabled":true,"Notes":"현재 플레이어 열에 맞는 1개 선택"},{"ShapePoolID":60003,"Candidate":3,"SelectMode":"직접 입력","Tiles":"1,2,4,5","Weight":5,"Enabled":true,"Notes":"사각형"},{"ShapePoolID":60003,"Candidate":4,"SelectMode":"직접 입력","Tiles":"2,3,5,6","Weight":5,"Enabled":true,"Notes":"사각형"},{"ShapePoolID":60003,"Candidate":5,"SelectMode":"직접 입력","Tiles":"4,5,7,8","Weight":5,"Enabled":true,"Notes":"사각형"},{"ShapePoolID":60003,"Candidate":6,"SelectMode":"직접 입력","Tiles":"5,6,8,9","Weight":5,"Enabled":true,"Notes":"사각형"},{"ShapePoolID":60003,"Candidate":7,"SelectMode":"직접 입력","Tiles":"2,4,5,6,8","Weight":10,"Enabled":true,"Notes":"십자선"},{"ShapePoolID":60003,"Candidate":8,"SelectMode":"직접 입력","Tiles":"1,3,5,7,9","Weight":10,"Enabled":true,"Notes":"X자"}]},{"name":"플레이어","keys":["PlayerID","Name","MaxHP","DodgeDamage","GuardMax","ParryMs","GuardHitCost","GuardHoldPerSec","GuardRegenPerSec","GuardBreakSec"],"rows":[{"PlayerID":1,"Name":"주인공","MaxHP":100,"DodgeDamage":30,"GuardMax":100,"ParryMs":200,"GuardHitCost":40,"GuardHoldPerSec":40,"GuardRegenPerSec":30,"GuardBreakSec":2}]},{"name":"공통 규칙","keys":["RuleID","Value","Description"],"rows":[{"RuleID":"DefaultResponseMs","Value":"750","Description":"공격 만들기의 피할 시간이 빈칸이면 750ms."},{"RuleID":"DefaultGapMinMs","Value":"300","Description":"예고 간격 최소가 빈칸이면 300ms."},{"RuleID":"DefaultGapMaxMs","Value":"600","Description":"예고 간격 최대가 빈칸이면 600ms."},{"RuleID":"DefaultPushLeadMs","Value":"300","Description":"밀기 전 예고가 빈칸이면 300ms. 임시."},{"RuleID":"DefaultPushMoveMs","Value":"150","Description":"밀려나는 시간이 빈칸이면 150ms. 임시."},{"RuleID":"AoeExtraResponseMs","Value":"200","Description":"선택된 범위 중 전체 9칸 동시 타격이 하나라도 있으면 반응 여유 200ms 추가. 경로 순차 9타에는 미적용. FFF 원본 기준."},{"RuleID":"TileRestoreSec","Value":"6","Description":"타일 파괴 후 이동 불가. 6초 뒤 복구. 공격속도 배율 제외."},{"RuleID":"GroggyDrainPerSec","Value":"30","Description":"빈틈 공격 중 게이지 초당 감소. 기존값."},{"RuleID":"PostGroggyLockMs","Value":"500","Description":"빈틈 종료 후 공격 제한. 기존값."},{"RuleID":"PushBoundary","Value":"반대쪽 확인 후 취소","Description":"예정 목적지가 경계 밖·파괴 타일이면 반대쪽 같은 거리 확인. 둘 다 불가하면 패턴 취소 후 공격 후 대기. 임시."},{"RuleID":"PushInput","Value":"이동 종료 후 허용","Description":"강제 이동 중 기본 이동 중지. 대기 입력 예약 없이 종료부터 방향키 이동 허용. 강제 이동은 회피 성공으로 세지 않음. 임시."},{"RuleID":"PhaseOrder","Value":"전환 우선","Description":"HP 0이면 다음 페이즈 확인 후 전환, 없으면 승리. 페이즈 진입 HP=MaxHP. 미정 전환은 실행 전 확정."},{"RuleID":"CombatPause","Value":"전투 시간만 정지","Description":"대화로 전투 정지 시 공격·이동·게이지·복구 시간 정지. 대화 넘김은 진행."}]},{"name":"작성 안내","keys":["Group","Topic","Description"],"rows":[{"Group":"시작","Topic":"공격 만들기부터","Description":"비슷한 공격 행을 복사하고 ID·이름을 바꾼 뒤 필요한 값만 수정하세요. 빈칸은 기본값, 회색칸은 해당 방식에서 사용하지 않는 칸입니다."},{"Group":"순서","Topic":"공격 → 몬스터 연결","Description":"공격을 만든 뒤 몬스터 사용 패턴에서 MonsterID·PhaseID·PatternID를 연결하고 피해·비중·사용을 설정하세요."},{"Group":"메모","Topic":"컬럼 제목 설명","Description":"한글 제목(2행)과 영문 이름(3행)에 설명과 예시가 있습니다. Excel의 메모/댓글 표시로 읽을 수 있습니다."},{"Group":"예시","Topic":"단일 또는 1~5연속","Description":"범위 반복에서 최소=최대=1은 단일. 최소=1, 최대=5면 매번 1~5회. 행을 추가할 필요가 없습니다."},{"Group":"예시","Topic":"FFF 연속 공격","Description":"30001은 최소2·최대5, 30002는2~3회, 30003은4~5회입니다. 선택한 횟수만큼 모두 예고한 뒤 같은 범위를 같은 박자로 타격합니다."},{"Group":"예시","Topic":"순차 공격","Description":"경로 순차에서 1,5,9를 입력하면 3타, 1,4,7,8,5,2,3,6,9면 9타입니다. 경로를 풀에서 고를 수도 있어요. 모션은 공격 구간에 한 번입니다."},{"Group":"예시","Topic":"엇박·특성 조합","Description":"타일 파괴와 방어 가능은 어떤 공격에도 적용됩니다. 엇박 추가 대기를 넣으면 같은 공격을 늦은 박자로 바꿀 수 있습니다."},{"Group":"예시","Topic":"샌즈 블래스터","Description":"공격 규칙은 범위 반복 1회. 이동·연출에서 이동 없음과 블래스터 레이저를 선택. 이펙트가 남아 있어도 피해는 한 번입니다."},{"Group":"예시","Topic":"샌즈 밀치기","Description":"공격 방식=밀친 위치. 이동·연출에서 좌우 무작위·1칸. 현재 위치로 목적지 계산 → 예고 → 밀기 → 탈출 시간 → 저장 목적지 타격."},{"Group":"입력","Topic":"반복·경로·밀친 위치","Description":"반복은 풀 필수·횟수1~5. 경로는 풀 또는 직접 경로 중 하나만. 밀친 위치는 풀·경로·횟수를 쓰지 않고 이동·연출 설정이 필수입니다."},{"Group":"입력","Topic":"모든 예고가 먼저","Description":"이번 버전은 전체 예고 후 공격으로 통일했습니다. 매 예고 직후 한 번씩 때리는 방식이 필요하면 별도 동작 규칙을 합의해야 합니다."},{"Group":"입력","Topic":"별도 연출 행은 선택","Description":"이동·연출에 없는 패턴은 이동 없음·몬스터 기본 모션·기본 이펙트와 소리입니다. 특수한 공격만 같은 PatternID로 추가합니다."},{"Group":"시간","Topic":"예고와 타격의 박자","Description":"예고를 0·450·900ms에 보여주고 피할 시간이750이면 타격은1650·2100·2550ms입니다. 서로 다른 간격이면 그 차이를 그대로 복사합니다."},{"Group":"시간","Topic":"속도 조절은 한 배율","Description":"몬스터 페이즈 AttackSpeed로 모든 패턴 시간을 나누고 모션 속도에는 곱합니다. 타일복구·패링시간·공통 빈틈 규칙은 배율 제외."},{"Group":"시간","Topic":"엇박·전체 범위","Description":"추가 대기는 이번 실행에서 한 번 뽑아 모든 타격에 똑같이 더합니다. 전체 9칸 동시 범위가 있으면 공통 여유 200ms도 한 번 더합니다."},{"Group":"샌즈","Topic":"실시간 기준의 뜻","Description":"예고 직전 현재 플레이어 위치를 한 번 읽고 목적지를 저장합니다. 예고 후 이동해도 목적지를 바꾸지 않으며 밀기와 HIT는 같은 타일을 사용합니다."},{"Group":"샌즈","Topic":"경계·파괴 처리","Description":"밀 목적지 불가 → 반대쪽 확인 → 양쪽 불가면 취소. 밀기 시작 전 목적지가 새로 파괴돼도 재선택 없이 취소. 목적지까지 보간 이동하는 초안입니다."},{"Group":"샌즈","Topic":"탈출 시간","Description":"예고300 + 강제이동150 + 피할시간550 = 첫 타격1000ms. 강제 이동 후 입력 허용. 시간과 방어 허용은 임시이며 조정 가능합니다."},{"Group":"실행","Topic":"범위 선택 시점","Description":"반복 공격은 시작 때 모든 범위를 저장합니다. 플레이어 행·열도 그때의 위치 기준. 한 번 예고한 범위를 HIT 직전에 다시 뽑지 않습니다."},{"Group":"실행","Topic":"같은 범위 금지","Description":"같은 타일 집합이면 같은 범위로 봅니다. 직전과 다른 유효 후보에서 비중으로 선택. 후보가 하나뿐이면 반복 허용하며 무한 재추첨하지 않습니다."},{"Group":"실행","Topic":"예고 표시","Description":"범위 반복이 실제2타 이상이면 파란 숫자 N→1. 1타면 기본 예고. 경로 순차는 경로 순서 예고. 연속 예고 표시는 다음 예고가 나오면 교체하지만 선택 범위는 유지합니다."},{"Group":"실행","Topic":"모션·이동 동기화","Description":"한 패턴에 공격 모션 한 번. 실제 클립과 타격 시점의 동기화는 에디터에서 연결합니다. 대상 이동 목적지는 모션 시작 때 고정. 이동 완료가 타격보다 늦으면 이동은 첫 타격 시점에 종료하는 초안입니다."},{"Group":"실행","Topic":"패턴 종료·중단","Description":"마지막 타격·모션·이동이 끝나면 몬스터의 공격 후 대기를 적용. 빈틈·페이즈 전환·전투 종료로 중단되면 남은 예고와 타격, 저장 범위를 모두 폐기합니다."},{"Group":"페이즈","Topic":"샌즈와 초기 MISS","Description":"첫 N번 빈틈 기회 전체를 MISS 처리. 실제 피해로 HP0이 되면 다음 페이즈 확인. 페이즈 전환 또는 최종 승리는 해당 빈틈 기회 종료 때 적용합니다."},{"Group":"피해","Topic":"피해 0과 타일 파괴","Description":"HitDamage=0이면 MISS·피해0이며 가드 소모·빈틈 증가 없음. 타일 파괴는 독립. 파괴된 타일 재타격은 피해·복구시간 갱신 없이 건너뜁니다."},{"Group":"데이터","Topic":"기존 수치 유지","Description":"몬스터9개 페이즈, 플레이어, 기존 활성 패턴6행의 피해·비중 유지. 취객 피해1도 원본 그대로. 샌즈 예시와 대각선 예시는 사용 끄기."},{"Group":"데이터","Topic":"미정 항목","Description":"마왕 HP·게이지·속도·대사와 샌즈 특수 공격 피해·비중은 미정입니다. 빈칸을0으로 해석하지 말고 실행 전에 채워 주세요."},{"Group":"연출","Topic":"연출 프리셋 연결","Description":"블래스터 레이저는 선택한 위험 타일과 방향에 맞게 배치하는 프리셋 이름입니다. 실제 Unity 모션·VFX·소리 연결은 프로그래머와 맞춰야 합니다."},{"Group":"출처","Topic":"기존 파일과 참고","Description":"전투 테이블.xlsx·간격수정.xlsx의 수치와 레이아웃, FFF 전투 프로토타입.html의 연속 예고·타격 순서를 참고했습니다."},{"Group":"출처","Topic":"마스터테이블_스킬.xlsx","Description":"사용기술모션·사용기술어빌리티의 동작/효과 분리 개념 참고. 개별 실행 단계 대신 작업자가 입력할 규칙을 한 행에 모았습니다."},{"Group":"ID 규칙","Topic":"완성된 패턴마다 고유 정수","Description":"PatternID는 종류 이름이 아니라 설정 한 행의 고유 번호입니다. 같은 단일·연속이라도 별도 설정으로 함께 쓸 때는 새 번호를 주세요. 공격 이름은 같아도 되지만 ID는 중복 불가입니다."},{"Group":"ID 규칙","Topic":"20001~29999 단일 계열","Description":"20001 일반 단일 / 20002 엇박 단일 / 20003 방어 불가 단일 / 20010 타일 파괴 단일 / 20020 샌즈 블래스터. 각 행의 실제 설정은 독립입니다."},{"Group":"ID 규칙","Topic":"30001~39999 반복 계열","Description":"30001 랜덤2~5연속 / 30002 랜덤2~3연속 / 30003 랜덤4~5연속. 1~5처럼 단일도 나올 수 있는 반복 규칙도 이 번호대에 둡니다."},{"Group":"ID 규칙","Topic":"40001~49999 경로 순차","Description":"40001 풀에서 경로 선택 / 40002 ㄹ자9칸 / 40003 대각선3칸. 새 경로 변형은 같은 번호대의 사용하지 않는 번호를 선택하세요."},{"Group":"ID 규칙","Topic":"50001~59999 강제 이동 계열","Description":"50001 샌즈 상대 밀치기. 번호대는 정리용이며 코드가 숫자 앞자리로 기능을 추측하지 않습니다. 실제 동작은 범위 사용 방식과 각 설정값을 읽습니다."},{"Group":"ID 규칙","Topic":"기존 패턴 수정과 복사","Description":"공유 패턴 값을 고치면 그 ID를 쓰는 모든 몬스터에게 반영됩니다. 특정 몬스터만 다르게 쓰려면 행을 복사하고 새 ID를 부여한 뒤 그 몬스터의 참조만 바꾸세요."},{"Group":"ID 규칙","Topic":"실제 연결 예시","Description":"몬스터 사용 패턴에서 20010을 선택하면 타일 파괴 단일을 가져옵니다. 30002와30003을 사용하는 초반·후반 연결 예시는 끄기로 추가했습니다. 기존 활성 패턴과 비중은 유지했습니다."},{"Group":"범위 풀 ID","Topic":"60001 전체 9종","Description":"기존 RANDOM_AREA 후보1~9. 60001을 쓰는 모든 공격은 이 후보와 선택 비중을 공유합니다."},{"Group":"범위 풀 ID","Topic":"60002 후보 1~4","Description":"60001에서 후보1~4를 복사해 별도 풀로 등록했습니다. 후보5~9는 이 풀에 없습니다. 기존60001에는 영향을 주지 않습니다."},{"Group":"범위 풀 ID","Topic":"70001 순차 경로 4종","Description":"기존 SEQUENTIAL_PATH의 행·열·대각선 경로 후보4개. 60000번대는 범위 후보, 70000번대는 경로 후보 정리용 번호대입니다. 실제 사용 방식은 공격 설정에서 정합니다."},{"Group":"범위 풀 ID","Topic":"같은 풀 ID의 반복은 정상","Description":"같은 묶음 안의 여러 행은 ShapePoolID가 같아야 합니다. 각 행의 키는 ShapePoolID+Candidate입니다. 다른 풀에서는 후보 번호1·2·3을 다시 사용할 수 있습니다."},{"Group":"범위 풀 ID","Topic":"부분 후보를 쓰는 몬스터","Description":"몬스터 사용 패턴의20004 → 공격 만들기의60002 → 범위 풀의후보1~4. 20001 →60001은 후보1~9입니다. 같은 공격에서 서로 다른 풀을 쓰려면 공격도 복사해 새 PatternID를 주세요."},{"Group":"범위 풀 ID","Topic":"비중은 각 풀 안에서 계산","Description":"60002의 비중25·25·5·5를 그대로 복사했습니다. 합계60으로 나누므로 확률은 약41.67%·41.67%·8.33%·8.33%입니다. 균등하게 하려면 모두1로 바꾸세요."},{"Group":"범위 풀 ID","Topic":"후보와 비중을 다르게 유지","Description":"새 풀을 만들 때 필요한 행을 복사하고 같은 새 ShapePoolID를 지정하세요. 기존 풀을 직접 수정하면 그것을 쓰는 모든 패턴에 영향을 줍니다."},{"Group":"확장 원칙","Topic":"기존 기능부터 조합","Description":"새 요구는 기존 페이즈·패턴 행·대사 조건·연출로 먼저 표현합니다. 전용 컬럼은 기존 구조로 표현할 수 없을 때만 추가합니다."},{"Group":"페이즈","Topic":"취객 네 단계","Description":"단계당 HP 750, 네 단계 합계 3000. 전환 사건은 빈틈공격 성공, 다음 페이즈 2→3→4→빈칸. 연타 시간이 끝나고 대사까지 마쳐야 다음 단계로 갑니다. 무입력·MISS는 진행하지 않습니다."},{"Group":"패턴","Topic":"취객 엇박 조절 위치","Description":"몬스터 사용 패턴에서 1~4페이즈의 엇박은 20011/20002/20012/20013. 공격 만들기의 ResponseMs와 ExtraMinMs·ExtraMaxMs로 조절하세요. 기본 단일과 공격 후 대기는 같습니다."},{"Group":"표시","Topic":"빈틈 피해 숫자","Description":"몬스터 페이즈의 OpeningDamageDisplay는 선택 입력. 빈칸=플레이어 DodgeDamage. 직접 입력=표시만 변경. 실제 피해는 플레이어에서 가져옵니다."},{"Group":"파일","Topic":"작업용·Unity용 한 버전","Description":"작업은 한글 XLSM에서 합니다. 수정한 파일을 시뮬레이터로 불러오고 변경 의도를 적어 버전 저장을 누르면 Unity용 XLSX도 함께 만듭니다."},{"Group":"버전 저장","Topic":"두 파일의 관계","Description":"확정된 게임 데이터는 두 파일이 같습니다. 한글·매크로·3행 제목은 작업용, 영문 시트·1행 제목·TRUE/FALSE는 Unity용입니다."},{"Group":"버전 저장","Topic":"변경 이력","Description":"년-월-일_시-분-초 폴더마다 변경 의도와 시트·행 키·컬럼·이전 값·변경 후 값을 기록합니다. 엑셀 Ctrl+S 후 시뮬레이터에서 불러와 버전 저장하세요."},{"Group":"버전 저장","Topic":"미완성 행과 동시 편집","Description":"미완성 마왕 페이즈는 작업용에 보관합니다. 한 번에는 둘 중 한 파일을 기준으로 수정하세요. 두 파일을 따로 수정한 내용은 자동 병합하지 않습니다."},{"Group":"미용 대사","Topic":"처음 부탁과 네?","Description":"대사에는 실제 문장을, 미용 대사 연결에는 손님 ID·단계·처음 부탁 그룹·자세한 부탁 그룹을 작성합니다. 같은 그룹의 Order는 연속 문장 순서이며 선택 분기가 아닙니다."},{"Group":"미용 대사","Topic":"알겠습니다와 다시 듣기","Description":"처음 부탁의 마지막 문장 뒤 네?/알겠습니다를 표시합니다. 자세한 부탁 뒤에는 알겠습니다만 표시합니다. 이미 들은 단계는 자동 반복하지 않고 다시 듣기로 재생합니다. 되물은 단계는 자세한 부탁을 다시 재생합니다."},{"Group":"미용 대사","Topic":"미용 단계 값","Description":"Stage는 cut(형태 만들기),draw(색·무늬 꾸미기),attach(장식 붙이기). 손님 ID와 Stage 조합은 중복할 수 없습니다. 처음 부탁·자세한 부탁 그룹 모두 존재하는 대사를 참조해야 합니다."},{"Group":"미용 대사","Topic":"엑셀 반영 경로","Description":"수정한 엑셀을 통합 개발실의 야차 편집기에서 불러온 뒤 미용 또는 대사 화면으로 이동하면 같은 대사 데이터로 시험합니다. 버전 저장은 XLSM/XLSX 한 쌍을 만듭니다. 공개 웹 반영은 프로젝트 JSON 내보내기 후 배포가 필요합니다."},{"Group":"미용 대사","Topic":"Unity 연동 범위","Description":"SalonDialogue: MonsterID int,Stage string,RequestGroupID int,DetailGroupID int. 웹 시뮬레이터와 엑셀 양방향 변환에 반영. Unity C# 수신 클래스·선택지 실행 연결은 프로그래머 확인 필요. 미용 영역·점수·그래픽 설정은 프로젝트 JSON에 유지."},{"Group":"미용 대사","Topic":"이전 두 번째 되묻기","Description":"기존 80004 그룹과 대사는 삭제하지 않고 보관. 현재 네? 한 번 흐름에는 연결하지 않음. 재생 여부는 미용 대사 연결에서 결정."},{"Group":"마왕 부하 대사","Topic":"엑셀 편집과 실행 범위","Description":"MonsterID 10004 마왕 부하의 등장·미용 부탁·상세 부탁·결과·퇴장·항의 문장은 대사/대화 그룹에서 편집합니다. 미용 부탁은 미용 대사 연결 cut/draw/attach에서 연결합니다. 미용 조건과 등장·결과·항의 사건 연결은 통합 프로젝트 JSON에 보관하며 실제 Unity 연결은 별도입니다. 미완성 야차 페이즈는 추가하지 않았습니다."},{"Group":"마왕 부하 대사","Topic":"arrival → 80080","Description":"마왕 부하 · 손님 등장"},{"Group":"마왕 부하 대사","Topic":"best → 80081","Description":"마왕 부하 · 미용 만족"},{"Group":"마왕 부하 대사","Topic":"normal → 80082","Description":"마왕 부하 · 미용 보통"},{"Group":"마왕 부하 대사","Topic":"fail → 80083","Description":"마왕 부하 · 미용 불만족"},{"Group":"마왕 부하 대사","Topic":"leave → 80084","Description":"마왕 부하 · 손님 퇴장"},{"Group":"마왕 부하 대사","Topic":"eyeContactLine → 80085","Description":"마왕 부하 · 눈에 닿았을 때 · 첫 항의"},{"Group":"마왕 부하 대사","Topic":"eyeContactSecondLine → 80086","Description":"마왕 부하 · 다시 눈에 닿았을 때 · 두 번째 항의"},{"Group":"마왕 부하 대사","Topic":"areaWarningLine → 80087","Description":"마왕 부하 · 뿔을 줄인 뒤 다시 불어날 때"},{"Group":"마왕 부하 대사","Topic":"areaOverflowLine → 80088","Description":"마왕 부하 · 처음보다 뿔이 더 많아졌을 때"},{"Group":"대사 담당자 검토","Topic":"담당자 검토본과 마왕 부하 통합","Description":"2026-10-16 저장된 시현님 검토본의 대사·대화 그룹·미용 대사 연결을 반영하고 기존 마왕 부하 대사를 유지했습니다. 겹치는 담당자 추가 그룹80085는80089, 문장900133~900136은900140~900143으로 분리했습니다. 샌즈 야차 승리 후 미용실 대사는 프로젝트의 afterWin에 그룹80089로 연결합니다. 문장 내용·순서는 담당자 검토본을 따릅니다."}]},{"name":"대사","keys":["DialogueID","GroupID","Order","Speaker","Text","Notes"],"rows":[{"DialogueID":900005,"GroupID":80001,"Order":1,"Speaker":"몬스터","Text":"&lt;wave=1&gt;으어... &lt;wait=0.35&gt;내, &lt;wait=0.25&gt;내일 언데드 보험회사?&lt;wait=0.25&gt; 면접이 있거든요...&lt;/wave&gt;","Notes":"기존 좀비 원문"},{"DialogueID":900006,"GroupID":80001,"Order":3,"Speaker":"플레이어","Text":"언데드가 보험? &lt;pulse=1.15&gt;이미 죽었는데 보험이 필요 있나?&lt;/pulse&gt;","Notes":"기존 좀비 원문"},{"DialogueID":900007,"GroupID":80001,"Order":4,"Speaker":"몬스터","Text":"&lt;wave=1&gt;어, 어허!&lt;wait=0.25&gt; 그건&lt;/wave&gt; &lt;shake=1&gt;종족차별,&lt;wait=0.25&gt; 발언&lt;/shake&gt;&lt;wave=1&gt;입니다...!&lt;/wave&gt;","Notes":"기존 좀비 원문"},{"DialogueID":900008,"GroupID":80001,"Order":5,"Speaker":"플레이어","Text":"알았다구요~ 원하는 스타일은 있나요?","Notes":"기존 좀비 원문"},{"DialogueID":900014,"GroupID":80002,"Order":1,"Speaker":"몬스터","Text":"으어어... 내,&lt;wait=0.25&gt; 내일 면접이니까... &lt;color=#266B4D&gt;앞이 좀 환해지고&lt;/color&gt;,&lt;wait=0.25&gt;\n&lt;color=#9A4935&gt;미, &lt;wait=0.25&gt;민망한 곳은 안 보였으면&lt;/color&gt; 좋겠어요...","Notes":"미용 요구 · 선택지 연결"},{"DialogueID":900015,"GroupID":80003,"Order":1,"Speaker":"몬스터","Text":"아, &lt;wait=0.25&gt;앞머리를 좀,&lt;wait=0.25&gt; 잘라서&lt;wait=0.25&gt; &lt;color=#266B4D&gt;두 눈이 잘 보이게&lt;/color&gt;,&lt;wait=0.25&gt; 좀 해 주세요...\n&lt;color=#9A4935&gt;뇌,&lt;wait=0.25&gt; 뇌가 좀 튀어나와서...&lt;wait=0.35&gt; 머리카락으로 가려&lt;/color&gt; 주시고요...&lt;wait=0.35&gt; &lt;wave=1.2&gt;부,&lt;wait=0.25&gt; 부탁드립니다,&lt;wait=0.25&gt; 으어...&lt;/wave&gt;","Notes":"미용 요구 · 선택지 연결"},{"DialogueID":900016,"GroupID":80004,"Order":1,"Speaker":"몬스터","Text":"아니, 앞이 안 보인다고요! 당장 '가위'를 들어서 내 눈을 가리는 앞머리를 싹 다 잘라달란 말입니다!","Notes":"기존 좀비 원문"},{"DialogueID":900017,"GroupID":80005,"Order":1,"Speaker":"몬스터","Text":"으어어…&lt;wait=0.35&gt; 제 눈을 직접 본 건...&lt;wait=0.35&gt; 죽은 뒤로 처음이에요,&lt;wait=0.25&gt; 으어...","Notes":"기존 좀비 원문"},{"DialogueID":900018,"GroupID":80006,"Order":1,"Speaker":"몬스터","Text":"으어어…&lt;wait=0.35&gt; 이, &lt;wait=0.25&gt;일단 앞은 보이네요… &lt;wait=0.35&gt;이 정도면 면접관님은 보이겠어요...&lt;wait=0.35&gt;","Notes":"기존 좀비 원문"},{"DialogueID":900019,"GroupID":80007,"Order":1,"Speaker":"몬스터","Text":"&lt;shake=1.4&gt;으어... &lt;wait=0.35&gt;으어?&lt;wait=0.35&gt; 으어어어어!!!!!&lt;/shake&gt;","Notes":"기존 좀비 원문"},{"DialogueID":900020,"GroupID":80008,"Order":1,"Speaker":"몬스터","Text":"머,&lt;wait=0.25&gt; 머리도 잘 됐는데... &lt;wait=0.35&gt;하,&lt;wait=0.25&gt; 한 번 기세를, &lt;wait=0.25&gt;제 기세를 시험해 주시겠습니까...?&lt;wait=0.35&gt; 으어,&lt;wait=0.25&gt; 면접 때 잘 싸울 수,&lt;wait=0.25&gt; 아,&lt;wait=0.25&gt; 아니 말할 수 있는지......","Notes":"기존 좀비 원문"},{"DialogueID":900021,"GroupID":80008,"Order":2,"Speaker":"몬스터","Text":"그, &lt;wait=0.25&gt;그니까 이게,&lt;wait=0.25&gt; 여,&lt;wait=0.25&gt; 연습 야차 상대를...&lt;wait=0.35&gt; 부탁드린다고요... &lt;wait=0.35&gt;이기면 호, &lt;wait=0.25&gt;홍보라도 해 드릴게요...&lt;wait=0.35&gt; 으어...","Notes":"기존 좀비 원문"},{"DialogueID":900022,"GroupID":80009,"Order":1,"Speaker":"몬스터","Text":"머리도 됐으니... 제 기세를 한 번 시험해 주시겠어요? 면접 때 자신있게 싸울... 아니 말할 수 있는지 봐주시면 됩니다.","Notes":"기존 좀비 원문"},{"DialogueID":900023,"GroupID":80009,"Order":2,"Speaker":"몬스터","Text":"연습 야차 상대를... 부탁드린다는 뜻입니다...저를 이기시면... 돈은 더 드릴게요…","Notes":"기존 좀비 원문"},{"DialogueID":900024,"GroupID":80010,"Order":1,"Speaker":"몬스터","Text":"가위 내려놓으실래요? 제가 면접관이라 생각하고 대답해 보세요. 제 머리... 왜 이렇게 하셨죠?","Notes":"기존 좀비 원문"},{"DialogueID":900025,"GroupID":80010,"Order":2,"Speaker":"몬스터","Text":"마왕 법전 제 666조! 야차룰로 정하죠. 제가 이기면... 배상하시는 겁니다!!!","Notes":"기존 좀비 원문"},{"DialogueID":900026,"GroupID":80011,"Order":1,"Speaker":"몬스터","Text":"으어어... 제가 대인배라 넘어갑니다... 다른 손님에겐 이렇게 하지 마세요...","Notes":"기존 좀비 원문"},{"DialogueID":900027,"GroupID":80012,"Order":1,"Speaker":"몬스터","Text":"으... 어쩔 수 없죠. 저도 면접 볼 체력을 아끼는 걸로 할게요. 머리 잘 해주셔서 감사합니다...","Notes":"기존 좀비 원문"},{"DialogueID":900028,"GroupID":80013,"Order":1,"Speaker":"몬스터","Text":"으... 어쩔 수 없죠. 저도 면접 볼 체력을 아끼는 걸로 할게요. 감사합니다...","Notes":"기존 좀비 원문"},{"DialogueID":900029,"GroupID":80014,"Order":1,"Speaker":"몬스터","Text":"감사합니다…! 실수로 물어도 이해해주세요… 물고 늘어지는 건 제 장점이라...","Notes":"기존 좀비 원문"},{"DialogueID":900030,"GroupID":80015,"Order":1,"Speaker":"몬스터","Text":"감사합니다…! 실수로 물어도 이해해주세요… 물고 늘어지는 건 제 장점이라...","Notes":"기존 좀비 원문"},{"DialogueID":900031,"GroupID":80016,"Order":1,"Speaker":"몬스터","Text":"으어어...&lt;wait=0.35&gt; 안녕하십니까…!&lt;wait=0.25&gt; 하,&lt;wait=0.25&gt; 한번 맡은 일은 죽어서도 노, &lt;wait=0.25&gt;놓지 않는 지원자… &lt;wait=0.35&gt;으어어…&lt;wait=0.35&gt; 실제로 죽어봤습니다!","Notes":"기존 좀비 원문"},{"DialogueID":900032,"GroupID":80017,"Order":1,"Speaker":"몬스터","Text":"변명은 됐습니다…&lt;wait=0.35&gt; 저도 이빨 좀 쓰겠습니다!","Notes":"기존 좀비 원문"},{"DialogueID":900033,"GroupID":80018,"Order":1,"Speaker":"몬스터","Text":"제, &lt;wait=0.25&gt;제 강점은… &lt;wait=0.35&gt;끈질긴 후속 연락입니다…!","Notes":"기존 좀비 원문"},{"DialogueID":900034,"GroupID":80018,"Order":2,"Speaker":"몬스터","Text":"정시 출근...&lt;wait=0.35&gt; 아니,&lt;wait=0.25&gt; 정시 타격입니다...!","Notes":"기존 좀비 원문"},{"DialogueID":900035,"GroupID":80019,"Order":1,"Speaker":"몬스터","Text":"이건...&lt;wait=0.35&gt; 고객 피드백입니다...!","Notes":"기존 좀비 원문"},{"DialogueID":900036,"GroupID":80019,"Order":2,"Speaker":"몬스터","Text":"서류 30번 떨어진 한...&lt;wait=0.35&gt; 받아라!!","Notes":"기존 좀비 원문"},{"DialogueID":900037,"GroupID":80020,"Order":1,"Speaker":"몬스터","Text":"으어어…&lt;wait=0.35&gt; 머리만은 건드리지 말아주세요…!","Notes":"기존 좀비 원문"},{"DialogueID":900038,"GroupID":80021,"Order":1,"Speaker":"몬스터","Text":"커헉... &lt;wait=0.35&gt;스펙이 너무 높아...","Notes":"기존 좀비 원문"},{"DialogueID":900039,"GroupID":80022,"Order":1,"Speaker":"몬스터","Text":"제,&lt;wait=0.25&gt; 제 기세에,&lt;wait=0.25&gt; 압도되셨군요...!","Notes":"기존 좀비 원문"},{"DialogueID":900040,"GroupID":80023,"Order":1,"Speaker":"몬스터","Text":"버, &lt;wait=0.25&gt;벌써 지치셨,&lt;wait=0.25&gt; 습니까?&lt;wait=0.35&gt; 감점 들어갑니다.","Notes":"기존 좀비 원문"},{"DialogueID":900041,"GroupID":80024,"Order":1,"Speaker":"몬스터","Text":"으어어... &lt;wait=0.25&gt;지, &lt;wait=0.25&gt;지금 보니 이 머리도 괜찮네요...","Notes":"기존 좀비 원문"},{"DialogueID":900042,"GroupID":80025,"Order":1,"Speaker":"몬스터","Text":"약속대로...&lt;wait=0.35&gt; 돈은 돌려받겠습니다...","Notes":"기존 좀비 원문"},{"DialogueID":900043,"GroupID":80026,"Order":1,"Speaker":"몬스터","Text":"여, 역시 이 정도는 되어야... &lt;wait=0.35&gt;취업 성공하는 거군요...&lt;wait=0.35&gt; 리스펙합니다.","Notes":"기존 좀비 원문"},{"DialogueID":900044,"GroupID":80027,"Order":1,"Speaker":"몬스터","Text":"으어어어! &lt;wait=0.35&gt;이 기세로 합격까지,&lt;wait=0.25&gt; 갑니다!","Notes":"기존 좀비 원문"},{"DialogueID":900048,"GroupID":80029,"Order":1,"Speaker":"몬스터","Text":"으어… 머리도 잘됐고… 태어나서 처음으로 자신감이 생겼어요… 죽은 뒤에 생기긴 했지만…","Notes":"기존 좀비 원문"},{"DialogueID":900049,"GroupID":80029,"Order":2,"Speaker":"플레이어","Text":"그 자신감으로 내일은 말로 설득 가보자고요~!!","Notes":"기존 좀비 원문"},{"DialogueID":900050,"GroupID":80029,"Order":3,"Speaker":"몬스터","Text":"네... 그럼 안녕히...","Notes":"기존 좀비 원문"},{"DialogueID":900051,"GroupID":80030,"Order":1,"Speaker":"몬스터","Text":"으어어…머리가 헝클어졌네... 내일도 이러면 어떡하죠…","Notes":"기존 좀비 원문"},{"DialogueID":900052,"GroupID":80030,"Order":2,"Speaker":"플레이어","Text":"초~ 큐트한 키라키라★리본 머리핀 있는데 드릴까요?","Notes":"기존 좀비 원문"},{"DialogueID":900053,"GroupID":80030,"Order":3,"Speaker":"몬스터","Text":"아니요... 친근한 인상으로 승부해볼게요...","Notes":"기존 좀비 원문"},{"DialogueID":900054,"GroupID":80030,"Order":4,"Speaker":"몬스터","Text":"그럼 안녕히…","Notes":"기존 좀비 원문"},{"DialogueID":900055,"GroupID":80031,"Order":1,"Speaker":"몬스터","Text":"으어어… 어찌저찌 이겼으니… 내일 면접도 어떻게든 되겠죠…","Notes":"기존 좀비 원문"},{"DialogueID":900056,"GroupID":80031,"Order":2,"Speaker":"플레이어","Text":"에에~ 면접이랑 싸움은 별개쟝~","Notes":"기존 좀비 원문"},{"DialogueID":900057,"GroupID":80031,"Order":3,"Speaker":"몬스터","Text":"그건 그렇죠... 어쨌든 감사합니다...","Notes":"기존 좀비 원문"},{"DialogueID":900058,"GroupID":80031,"Order":4,"Speaker":"몬스터","Text":"그럼 안녕히…","Notes":"기존 좀비 원문"},{"DialogueID":900059,"GroupID":80032,"Order":1,"Speaker":"몬스터","Text":"으어어… 내일 이 머리 얘기가 나오면… 뭐라고 해야 할까요…","Notes":"기존 좀비 원문"},{"DialogueID":900060,"GroupID":80032,"Order":2,"Speaker":"플레이어","Text":"초- 신선한 유행의 선두주자― 인데스케도 면접관이 사람 보는 눈이 없는 거네~","Notes":"기존 좀비 원문"},{"DialogueID":900061,"GroupID":80032,"Order":3,"Speaker":"몬스터","Text":"새로운 시도를 두려워하지 않는다는 거죠... 어떻게든 해볼게요...","Notes":"기존 좀비 원문"},{"DialogueID":900062,"GroupID":80033,"Order":1,"Speaker":"몬스터","Text":"으어어… 내일 이 머리 얘기가 나오면… 뭐라고 해야 하지…","Notes":"기존 좀비 원문"},{"DialogueID":900063,"GroupID":80033,"Order":2,"Speaker":"플레이어","Text":"초- 신선한 유행의 선두주자― 인데스케도 면접관이 사람 보는 눈이 없는 거네~","Notes":"기존 좀비 원문"},{"DialogueID":900064,"GroupID":80033,"Order":3,"Speaker":"몬스터","Text":"........상당히 뻔뻔하시네요… 으어어….어떻게든 되겠죠…","Notes":"기존 좀비 원문"},{"DialogueID":900065,"GroupID":80033,"Order":4,"Speaker":"몬스터","Text":"이번에도 탈락하면... 대체 언제.....하아…","Notes":"기존 좀비 원문"},{"DialogueID":900066,"GroupID":80034,"Order":1,"Speaker":"몬스터","Text":"으어... 취직했다... 앞머리도 방구석 생활도 해방됨...... 몇달만에 사람 얼굴 제대로 보는 느낌ㅠㅠ #몬스터헤어살롱 덕분에 붙은 것 같아요 감사합니다. 모두 기 받아가세요! #취업성공 #취준생 #화이팅","Notes":"기존 좀비 원문"},{"DialogueID":900067,"GroupID":80035,"Order":1,"Speaker":"몬스터","Text":"역시나 면접 떨어졌다….. #취준생 #절규 #미용실저주함 돈도 잃고 머리도 잃음","Notes":"기존 좀비 원문"},{"DialogueID":900068,"GroupID":80036,"Order":1,"Speaker":"몬스터","Text":"&lt;wave=3 speed=5&gt;&lt;color=#FFD166&gt;&lt;size=24&gt;으하하하!&lt;/size&gt;&lt;/color&gt; 오랜만이구먼, &lt;color=#FFDA8A&gt;제이!!&lt;/color&gt;&lt;/wave&gt;&lt;wait=0.25&gt; 미용실에 불이 켜졌길래... 드디어 돌아온 줄 알았지!","Notes":"취객의 가업·제이·몬스터 소울을 떠올리는 단서. 실제 해금·튜토리얼은 야차 이후 미용실에서 진행."},{"DialogueID":900070,"GroupID":80038,"Order":1,"Speaker":"몬스터","Text":"&lt;shake=2 speed=15 dur=0.45&gt;어이쿠!&lt;/shake&gt;&lt;wait=0.3&gt; 손맛 한번 여전하구먼.&lt;wave=2 speed=4&gt; 근데 제이, 자네... 원래 둘이었나?&lt;/wave&gt;","Notes":"색·동작 태그는 문자 효과 규칙 시트 참고."},{"DialogueID":900071,"GroupID":80039,"Order":1,"Speaker":"몬스터","Text":"어...&lt;wait=0.4&gt; &lt;color=#A9E4DA&gt;이제 한 명으로 보이네.&lt;/color&gt; 제이가... 아니군.&lt;wait=0.45&gt; 미용실에 불이 들어왔길래, 그 녀석인 줄 알았어.","Notes":"취객의 가업·제이·몬스터 소울을 떠올리는 단서. 실제 해금·튜토리얼은 야차 이후 미용실에서 진행."},{"DialogueID":900072,"GroupID":80040,"Order":1,"Speaker":"몬스터","Text":"허... 막일할 때도 굳어 있던 손이...&lt;wait=0.4&gt; 이 감각, &lt;color=#FFD166&gt;소울을 벼리던 때&lt;/color&gt;랑 닮았구먼.&lt;wait=0.3&gt; 제이가 봤으면 또 실실 웃었겠어!","Notes":"취객의 가업·제이·몬스터 소울을 떠올리는 단서. 실제 해금·튜토리얼은 야차 이후 미용실에서 진행."},{"DialogueID":900073,"GroupID":80041,"Order":1,"Speaker":"몬스터","Text":"&lt;shake=2 speed=16 dur=0.4&gt;크하!&lt;/shake&gt; ...&lt;wait=0.4&gt;&lt;color=#B7F4D0&gt;다 깼다, 다 깼어!&lt;/color&gt;\n옛 솜씨도 술에 몽땅 절여진 줄 알았더니! &lt;pulse=1.1 speed=7&gt;아직 쓸 만하구먼! 으하하하!&lt;/pulse&gt;","Notes":"취객의 가업·제이·몬스터 소울을 떠올리는 단서. 실제 해금·튜토리얼은 야차 이후 미용실에서 진행."},{"DialogueID":900074,"GroupID":80042,"Order":1,"Speaker":"몬스터","Text":"우리 집안은 &lt;color=#FFD166&gt;몬스터 소울을 장비와 기술로 벼렸지.&lt;/color&gt; 세상은 바뀌고, 찾는 이도 줄고...&lt;wait=0.4&gt; 제이까지 사라지고 나니 더 붙들 이유가 없더군.","Notes":"취객의 가업·제이·몬스터 소울을 떠올리는 단서. 실제 해금·튜토리얼은 야차 이후 미용실에서 진행."},{"DialogueID":900075,"GroupID":80042,"Order":2,"Speaker":"몬스터","Text":"그런데 그 미용실에 &lt;color=#B7F4D0&gt;다시 불이 켜졌어.&lt;/color&gt;&lt;wait=0.4&gt; 내 손도 아직 기억하고 있고. 돌아가세. 자네한테 보여줄 게 떠올랐거든! &lt;wave=2 speed=6&gt;&lt;color=#FFD166&gt;으하하하!&lt;/color&gt;&lt;/wave&gt;","Notes":"취객의 가업·제이·몬스터 소울을 떠올리는 단서. 실제 해금·튜토리얼은 야차 이후 미용실에서 진행."},{"DialogueID":900069,"GroupID":80037,"Order":1,"Speaker":"몬스터","Text":"헤.&lt;wait=0.35&gt; 오늘은... &lt;wait=0.25&gt;&lt;color=#8BE9FD&gt;가볍게&lt;/color&gt; 가자고,&lt;wait=0.25&gt; 친구. &lt;wait=0.35&gt; 내 &lt;color=#1900d6&gt;파란 공격&lt;/color&gt;은 알고 있겠지?","Notes":"색·동작 태그는 문자 효과 규칙 시트 참고."},{"DialogueID":900076,"GroupID":80043,"Order":1,"Speaker":"몬스터","Text":"뭐야? &lt;wait=0.35&gt;그럼 내가 &lt;wave=2&gt;가만히 서서 맞아줄 줄 알았어?&lt;/wave&gt;","Notes":"색·동작 태그는 문자 효과 규칙 시트 참고."},{"DialogueID":900077,"GroupID":80044,"Order":1,"Speaker":"몬스터","Text":"어라? &lt;wait=0.35&gt;&lt;wave=1.4&gt;여기서 맞으면 안 되지 않나?&lt;/wave&gt;","Notes":"색·동작 태그는 문자 효과 규칙 시트 참고."},{"DialogueID":900078,"GroupID":80045,"Order":1,"Speaker":"몬스터","Text":"너, &lt;wait=0.25&gt;그, &lt;wait=0.25&gt;&lt;pulse=1.15&gt;그거 휘두르는 거 진짜 좋아하는구나, &lt;wait=0.25&gt;응?&lt;/pulse&gt;","Notes":"색·동작 태그는 문자 효과 규칙 시트 참고."},{"DialogueID":900079,"GroupID":80046,"Order":1,"Speaker":"몬스터","Text":"&lt;shake=2&gt;으악!!&lt;/shake&gt;&lt;wait=0.5&gt; &lt;wave=1&gt;크흠, &lt;wait=0.25&gt;큼,&lt;wait=0.25&gt; 그러니까, &lt;/wave&gt;&lt;wait=0.35&gt;아무것도 아니었어, 헤.","Notes":"색·동작 태그는 문자 효과 규칙 시트 참고."},{"DialogueID":900080,"GroupID":80047,"Order":1,"Speaker":"몬스터","Text":"&lt;wave=1&gt;잠깐... &lt;wait=0.25&gt;친구야,&lt;/wave&gt;&lt;wait=0.25&gt; &lt;shake=1.4&gt;나 기억 안 나?&lt;/shake&gt;&lt;wait=0.5&gt; &lt;shake=1.4&gt;그냥 다 잊어버리자고,&lt;wait=0.25&gt; 알겠지?&lt;/shake&gt;","Notes":"색·동작 태그는 문자 효과 규칙 시트 참고."},{"DialogueID":900081,"GroupID":80048,"Order":1,"Speaker":"몬스터","Text":"그냥...&lt;wait=0.4&gt; &lt;shake=1.2&gt;닮지 않았다고만 하지 말아줘.&lt;/shake&gt;","Notes":"색·동작 태그는 문자 효과 규칙 시트 참고."},{"DialogueID":900082,"GroupID":80049,"Order":1,"Speaker":"몬스터","Text":"&lt;wave=2 speed=5&gt;&lt;color=#B7F4D0&gt;으어어...&lt;wait=0.35&gt;&lt;/color&gt;&lt;/wave&gt; 손 좀 빌려주세요.&lt;wait=0.35&gt; 아, &lt;wait=0.25&gt;&lt;shake=2 dur=0.4&gt;떼어주시진 말고...!&lt;/shake&gt;","Notes":"전투 중 대사. 등장·미용 과정 대사는 보류."},{"DialogueID":900083,"GroupID":80049,"Order":2,"Speaker":"몬스터","Text":"&lt;color=#FFD166&gt;끈기&lt;wait=0.25&gt;&lt;/color&gt;, 하나는 자신 있습니다...!&lt;wait=0.3&gt; &lt;wave=2 speed=5&gt;죽어서도 출근하잖아요...&lt;/wave&gt;","Notes":"전투 중 대사. 등장·미용 과정 대사는 보류."},{"DialogueID":900084,"GroupID":80050,"Order":1,"Speaker":"몬스터","Text":"잠깐...&lt;wait=0.25&gt; &lt;shake=2 speed=16 dur=0.5&gt;뼈 때리시면...!&lt;wait=0.25&gt;&lt;/shake&gt; &lt;color=#FFD166&gt;지, &lt;wait=0.25&gt;진짜 뼈 맞는다고요...!&lt;/color&gt;","Notes":"전투 중 대사. 등장·미용 과정 대사는 보류."},{"DialogueID":900085,"GroupID":80051,"Order":1,"Speaker":"몬스터","Text":"&lt;cps=15&gt;끝난 줄... 아셨죠?&lt;/cps&gt;&lt;wait=0.5&gt; &lt;color=#B7F4D0&gt;&lt;size=23&gt;좀비는 다시 부활한다구요!&lt;/size&gt;&lt;/color&gt;\n&lt;shake=3 speed=16 dur=0.8&gt;&lt;wave=3 speed=5&gt;으어어어..!&lt;/wave&gt;&lt;/shake&gt;","Notes":"전투 중 대사. 등장·미용 과정 대사는 보류."},{"DialogueID":900086,"GroupID":80051,"Order":2,"Speaker":"몬스터","Text":"&lt;color=#FFD166&gt;재도전&lt;/color&gt;에는 자신 있습니다.&lt;wait=0.35&gt; 취업도...&lt;wait=0.5&gt; 이렇게 쉽게 부활하면 좋을 텐데요.","Notes":"전투 중 대사. 등장·미용 과정 대사는 보류."},{"DialogueID":900087,"GroupID":80052,"Order":1,"Speaker":"몬스터","Text":"&lt;wave=2 speed=3&gt;으어어...&lt;/wave&gt;&lt;wait=0.4&gt; 오늘은 여기까지...\n&lt;color=#B7F4D0&gt;재도전도 휴식이 필요하다구요.&lt;/color&gt;","Notes":"전투 중 대사. 등장·미용 과정 대사는 보류."},{"DialogueID":900088,"GroupID":80053,"Order":1,"Speaker":"몬스터","Text":"&lt;color=#FFD166&gt;끈기 있는 지원자!&lt;/color&gt; 저, 맞죠?&lt;wait=0.3&gt; &lt;wave=2 speed=5&gt;으허허... 아직 쓸 만하네요!&lt;/wave&gt;","Notes":"전투 중 대사. 등장·미용 과정 대사는 보류."},{"DialogueID":900089,"GroupID":80054,"Order":1,"Speaker":"몬스터","Text":"면접에선,&lt;wait=0.25&gt; 으어,&lt;wait=0.25&gt; 첫인상이 중요하니까요...\n덜 긴, 긴장하려면,&lt;wait=0.25&gt; &lt;color=#9A5B22&gt;&lt;pulse=1.06&gt;단정한 인상&lt;/pulse&gt;&lt;/color&gt;이면 덜 긴장할 것 같아요...&lt;wait=0.35&gt; 으어어...","Notes":"미용 요구 · 선택지 연결"},{"DialogueID":900090,"GroupID":80055,"Order":1,"Speaker":"몬스터","Text":"으어어...&lt;wait=0.35&gt; 염색은 &lt;wave=1.2&gt;&lt;color=#71508F&gt;아무렇게나&lt;/color&gt;&lt;/wave&gt; 괜찮아요...\n저, &lt;wait=0.25&gt;저는,&lt;wait=0.25&gt; &lt;color=#266B4D&gt;지금 머리 색도&lt;/color&gt;,&lt;wait=0.25&gt; 좋아요...","Notes":"미용 요구 · 선택지 연결"},{"DialogueID":900091,"GroupID":80056,"Order":1,"Speaker":"몬스터","Text":"&lt;wave=1&gt;으어어… &lt;wait=0.35&gt;머리도 하고…&lt;wait=0.35&gt; 상쾌하게 몸도 풀고...&lt;wait=0.35&gt; 면접 준비 끝났어요...&lt;/wave&gt;","Notes":"통합 플레이"},{"DialogueID":900092,"GroupID":80057,"Order":1,"Speaker":"몬스터","Text":"&lt;wave=1&gt;으어어...&lt;wait=0.35&gt; 연습은 여기까지 하죠...&lt;wait=0.35&gt; 저도 내일 면접이 있어서요.&lt;/wave&gt;","Notes":"통합 플레이"},{"DialogueID":900093,"GroupID":80058,"Order":1,"Speaker":"몬스터","Text":"&lt;shake=2&gt;으하하하!&lt;/shake&gt; 오랜만이구먼, 제이!!","Notes":"통합 플레이"},{"DialogueID":900094,"GroupID":80058,"Order":2,"Speaker":"몬스터","Text":"가게에 불이 켜져 있길래 냅다 뛰어왔지! 이야, 얼굴이 좀... &lt;wave=3&gt;두 개로 보이는구먼!&lt;/wave&gt;","Notes":"통합 플레이"},{"DialogueID":900095,"GroupID":80059,"Order":1,"Speaker":"몬스터","Text":"...자네, 제이가 아니었구먼. 허허. 이제야 제대로 보이는군.","Notes":"통합 플레이"},{"DialogueID":900096,"GroupID":80059,"Order":2,"Speaker":"몬스터","Text":"제이가 사라진 뒤로 이 가게도, 내 손끝도 멈춘 줄 알았지. 일용직 일 끝내고 한잔하는 게 하루의 전부였어.","Notes":"통합 플레이"},{"DialogueID":900097,"GroupID":80059,"Order":3,"Speaker":"몬스터","Text":"우리 집안은 몬스터의 소울에 남은 힘을 &lt;color=#9FE8D1&gt;장비와 기술로 빚어내던&lt;/color&gt; 일을 했네. 아는 이만 찾던 오래된 가업이지.","Notes":"통합 플레이"},{"DialogueID":900098,"GroupID":80059,"Order":4,"Speaker":"몬스터","Text":"세상이 편리해지니 그 솜씨를 찾는 이도 줄었어. 다시 쓸 일이 없을 줄 알았는데... 자네를 보니, &lt;wave=2&gt;손이 근질근질하구먼!&lt;/wave&gt;","Notes":"통합 플레이"},{"DialogueID":900099,"GroupID":80059,"Order":5,"Speaker":"몬스터","Text":"좋아. 머물러도 된다면 손끝부터 다시 깨워 보지. &lt;color=#FFD166&gt;몬스터 소울을 다루는 법&lt;/color&gt;도 차근차근 알려 주겠네.","Notes":"통합 플레이"},{"DialogueID":900100,"GroupID":80060,"Order":1,"Speaker":"몬스터","Text":"허허, 오늘은 술 대신 물 한 잔이면 되겠어. 도구를 챙겨 올 테니, 가게 불은 꺼뜨리지 말게!","Notes":"통합 플레이"},{"DialogueID":900101,"GroupID":80061,"Order":1,"Speaker":"몬스터","Text":"...헤. &lt;wait=0.35&gt;여기 솜씨가 좋다는 소문을 들었거든.","Notes":"통합 플레이"},{"DialogueID":900102,"GroupID":80061,"Order":2,"Speaker":"몬스터","Text":"&lt;pulse=1.15&gt;\"뼈\"&lt;/pulse&gt; 있는 부탁 하나 해도 될까?&lt;wait=0.35&gt; &lt;color=#FFD166&gt;얼굴 테두리&lt;/color&gt;만 다듬어 줘. &lt;wait=0.35&gt;머리카락은... &lt;wait=0.35&gt;보다시피 휴가 중이야.","Notes":"통합 플레이"},{"DialogueID":900103,"GroupID":80062,"Order":1,"Speaker":"몬스터","Text":"헤. &lt;wait=0.35&gt;오늘은 &lt;color=#52609B&gt;인상 좀 다듬으러&lt;/color&gt; 왔어.&lt;wait=0.35&gt;\n&lt;color=#52609B&gt;각진 데만 가볍게.&lt;wait=0.35&gt;&lt;/color&gt; &lt;wave=1.3&gt;뼈대는 괜찮잖아?&lt;/wave&gt;","Notes":"미용 요구 · 선택지 연결"},{"DialogueID":900104,"GroupID":80063,"Order":1,"Speaker":"몬스터","Text":"이번엔 좀 &lt;color=#9A4935&gt;&lt;shake=0.6&gt;만만하지 않은 인상&lt;/shake&gt;&lt;/color&gt;이면 좋겠어.&lt;wait=0.35&gt;\n&lt;color=#9A4935&gt;장식&lt;/color&gt;으로 한 수 보여 줄래?","Notes":"미용 요구 · 선택지 연결"},{"DialogueID":900105,"GroupID":80064,"Order":1,"Speaker":"몬스터","Text":"헤. &lt;wait=0.35&gt;꽤 뼈대 있는 실력이네.&lt;wait=0.35&gt; 그럼... &lt;wait=0.35&gt;몸도 한번 풀어 볼까?","Notes":"통합 플레이"},{"DialogueID":900106,"GroupID":80065,"Order":1,"Speaker":"몬스터","Text":"나쁘지 않네.&lt;wait=0.35&gt; 이번엔 다른 솜씨도 보여 줄래?","Notes":"통합 플레이"},{"DialogueID":900107,"GroupID":80066,"Order":1,"Speaker":"몬스터","Text":"...친구, &lt;wait=0.35&gt;이건 좀 &lt;pulse=1.15&gt;\"뼈\"&lt;/pulse&gt;아픈데.&lt;wait=0.35&gt; 잠깐 밖에서 얘기할까?","Notes":"통합 플레이"},{"DialogueID":900109,"GroupID":80068,"Order":1,"Speaker":"몬스터","Text":"&lt;color=#71508F&gt;무슨 색이든,&lt;wait=0.25&gt; 무슨 무늬든&lt;/color&gt; 사,&lt;wait=0.25&gt; 상관 없어요...&lt;wait=0.35&gt;\n&lt;color=#266B4D&gt;염색 안 해도 괜찮아요...&lt;/color&gt;&lt;wait=0.35&gt; 지금 머리도 마음에 들어요, &lt;wait=0.25&gt;으어...","Notes":"미용 선택지 대사"},{"DialogueID":900110,"GroupID":80069,"Order":1,"Speaker":"몬스터","Text":"&lt;color=#9A5B22&gt;단정하고 점잖아 보일 장식&lt;/color&gt;으로...&lt;wait=0.35&gt;\n&lt;color=#9A5B22&gt;하나만&lt;/color&gt;...&lt;wait=0.35&gt; 골라 주시겠어요?&lt;wait=0.35&gt; 으어,&lt;wait=0.25&gt; &lt;wave=1.2&gt;너무 요란, &lt;wait=0.25&gt;하진 않게요...&lt;/wave&gt;","Notes":"미용 선택지 대사"},{"DialogueID":900111,"GroupID":80070,"Order":1,"Speaker":"몬스터","Text":"&lt;color=#52609B&gt;얼굴 바깥 테두리만&lt;/color&gt; 망치랑 정으로 톡톡 다듬어 줘.&lt;wait=0.35&gt;\n&lt;color=#9A4935&gt;눈코입은 그대로.&lt;wait=0.35&gt;&lt;/color&gt; &lt;wave=1.2&gt;속까지 시원해질 필요는 없거든.&lt;/wave&gt;","Notes":"미용 선택지 대사"},{"DialogueID":900112,"GroupID":80071,"Order":1,"Speaker":"몬스터","Text":"색은 &lt;color=#71508F&gt;네 감각에 맡길게.&lt;wait=0.35&gt;&lt;/color&gt;\n&lt;color=#52609B&gt;원래 뼈 색&lt;/color&gt;도 꽤 멋지거든.&lt;wait=0.35&gt; &lt;wave=1.2&gt;&lt;pulse=1.15&gt;\"뼈\"&lt;/pulse&gt;가 있는 색이지.&lt;/wave&gt;","Notes":"미용 선택지 대사"},{"DialogueID":900113,"GroupID":80072,"Order":1,"Speaker":"몬스터","Text":"&lt;color=#71508F&gt;더한 뼈와 바깥 테두리&lt;/color&gt;에 마음 가는 색을 칠해 봐.&lt;wait=0.35&gt;\n&lt;color=#52609B&gt;그대로 둬도 좋아.&lt;wait=0.35&gt;&lt;/color&gt; 취향엔 정답이 없으니까. &lt;wait=0.35&gt;헤.","Notes":"미용 선택지 대사"},{"DialogueID":900114,"GroupID":80073,"Order":1,"Speaker":"몬스터","Text":"&lt;color=#9A4935&gt;강해 보이는 장식 하나&lt;/color&gt;를 &lt;color=#52609B&gt;얼굴이나 머리 쪽&lt;/color&gt;에 부탁해.&lt;wait=0.35&gt;\n딱 봤을 때 &lt;shake=0.6&gt;쉽게 덤비지는 못하겠다&lt;/shake&gt; 싶은 걸로.","Notes":"미용 선택지 대사"},{"DialogueID":900140,"GroupID":80056,"Order":2,"Speaker":"플레이어","Text":"두들겨 맞아서 어깨 힘도 다 빠졌죠?","Notes":"통합 개발실"},{"DialogueID":900141,"GroupID":80056,"Order":3,"Speaker":"몬스터","Text":"&lt;wave=1&gt;그렇네요... &lt;wait=0.35&gt;감사합니다...&lt;/wave&gt;","Notes":"통합 개발실"},{"DialogueID":900142,"GroupID":80037,"Order":2,"Speaker":"몬스터","Text":"뭐?&lt;wait=0.5&gt; &lt;shake=1&gt;모른다고?&lt;/shake&gt;&lt;wait=0.5&gt;&lt;shake=2&gt; 어떻게 그럴 수가 있지?&lt;/shake&gt; &lt;wait=0.5&gt;와,&lt;wait=0.25&gt; &lt;wave=1.4&gt;샌즈의 &lt;color=#1900d6&gt;파란 공격&lt;/color&gt;은 말이야...&lt;/wave&gt;","Notes":"통합 개발실"},{"DialogueID":900143,"GroupID":80037,"Order":3,"Speaker":"몬스터","Text":"아니야, &lt;wait=0.25&gt;그냥 직접 보여줘야겠어,&lt;wait=0.25&gt; &lt;wait=0.35&gt;헤.","Notes":"통합 개발실"},{"DialogueID":900137,"GroupID":80089,"Order":2,"Speaker":"몬스터","Text":"헤.&lt;wait=0.35&gt; 난 &lt;color=#ec6565&gt;그릴비&lt;/color&gt;나 가야겠군.","Notes":"통합 개발실"},{"DialogueID":900138,"GroupID":80089,"Order":1,"Speaker":"몬스터","Text":"크, &lt;wait=0.25&gt;크흠... &lt;wait=0.35&gt;제법인데, &lt;wait=0.25&gt;꼬마야. &lt;wave=1.4&gt;&lt;pulse=1.15&gt;\"뼈\"&lt;/pulse&gt;가 시리는 전투였어.&lt;/wave&gt;","Notes":"통합 개발실"},{"DialogueID":900139,"GroupID":80001,"Order":2,"Speaker":"몬스터","Text":"&lt;wave=1&gt;주,&lt;wait=0.25&gt; 죽고 나서 면접은,&lt;wait=0.25&gt; 처음이에요...&lt;/wave&gt;","Notes":"통합 개발실"},{"DialogueID":900115,"GroupID":80074,"Order":1,"Speaker":"몬스터","Text":"점검은 &lt;color=#52609B&gt;손님의 부탁을 얼마나 정확히 이루어 주는지&lt;/color&gt; 보겠습니다. 제 부탁으로 시험하지요.","Notes":"중간 점검: 한 번도 승인되지 않은 반차를 외모 변화로 설득하는 과제. 로컬 검토 초안."},{"DialogueID":900116,"GroupID":80074,"Order":2,"Speaker":"몬스터","Text":"우선 이 뿔부터입니다. 보고서는 정리했는데, 제 머리 위는 아직이군요.\n눈을 찌르면 점검표도 읽을 수 없습니다.","Notes":"중간 점검: 한 번도 승인되지 않은 반차를 외모 변화로 설득하는 과제. 로컬 검토 초안."},{"DialogueID":900117,"GroupID":80074,"Order":3,"Speaker":"몬스터","Text":"&lt;color=#52609B&gt;눈 세 개는 무사하게, 뿔은 왔을 때보다 가볍게&lt;/color&gt; 부탁드립니다.\n모양은 맡기겠습니다. 정해진 답을 베끼는 시험은 아니니까요.","Notes":"중간 점검: 한 번도 승인되지 않은 반차를 외모 변화로 설득하는 과제. 로컬 검토 초안."},{"DialogueID":900118,"GroupID":80075,"Order":1,"Speaker":"몬스터","Text":"&lt;color=#52609B&gt;세 눈에 닿지 않게&lt;/color&gt; 뿔을 다듬어 주세요.\n모양은 자유입니다. 다만 전체 양은 처음보다 줄어야 합니다. 줄여 달랬는데 늘어나면 곤란하겠지요.","Notes":"중간 점검: 한 번도 승인되지 않은 반차를 외모 변화로 설득하는 과제. 로컬 검토 초안."},{"DialogueID":900120,"GroupID":80076,"Order":1,"Speaker":"몬스터","Text":"이제 본시험입니다. 저는 &lt;color=#52609B&gt;666년 동안 단 한 번도 반차를 승인받지 못했습니다.&lt;/color&gt; 무슨 수를 써도 “멀쩡해 보인다”시더군요.\n&lt;color=#52609B&gt;세 눈 아래 모두, 가장 어두운 색으로 다크서클&lt;/color&gt;을 만들어 주십시오. 쉬어야 한다는 말이 얼굴만 봐도 전해지도록요.","Notes":"중간 점검: 한 번도 승인되지 않은 반차를 외모 변화로 설득하는 과제. 로컬 검토 초안."},{"DialogueID":900121,"GroupID":80077,"Order":1,"Speaker":"몬스터","Text":"&lt;color=#52609B&gt;이마의 눈과 안경 쓴 두 눈, 세 눈 아래를 모두&lt;/color&gt; 짙게 해 주세요.\n눈 자체와 나머지 얼굴은 깔끔하게. 피곤한 인상을 만드는 솜씨를 보는 거지, 보고서를 못 읽게 하는 시험은 아닙니다.","Notes":"중간 점검: 한 번도 승인되지 않은 반차를 외모 변화로 설득하는 과제. 로컬 검토 초안."},{"DialogueID":900122,"GroupID":80078,"Order":1,"Speaker":"몬스터","Text":"마지막으로 &lt;color=#D94B4B&gt;코끝에 빨간 코 장식 하나&lt;/color&gt;를 붙여 주십시오.\n마왕님이 제 얼굴을 보고 먼저 “오늘은 쉬어라” 하신다면…… 그보다 확실한 실력 증명이 있겠습니까?","Notes":"중간 점검: 한 번도 승인되지 않은 반차를 외모 변화로 설득하는 과제. 로컬 검토 초안."},{"DialogueID":900123,"GroupID":80079,"Order":1,"Speaker":"몬스터","Text":"&lt;color=#D94B4B&gt;빨간 코는 코 주변에 하나&lt;/color&gt;면 됩니다.\n아파 보이되 우스꽝스럽지는 않게. 반차 신청서이지, 궁정 축제 참가 신청서가 아닙니다.","Notes":"중간 점검: 한 번도 승인되지 않은 반차를 외모 변화로 설득하는 과제. 로컬 검토 초안."},{"DialogueID":900124,"GroupID":80080,"Order":1,"Speaker":"몬스터","Text":"실례합니다. 마왕님의 직속 부하입니다. 예고드린 &lt;color=#FFD166&gt;중간 점검&lt;/color&gt;을 하러 왔습니다.\n5일차에 마왕님을 모시려면, 별 세 개에 어울리는 솜씨를 보여 주셔야겠지요.","Notes":"중간 점검: 한 번도 승인되지 않은 반차를 외모 변화로 설득하는 과제. 로컬 검토 초안."},{"DialogueID":900125,"GroupID":80080,"Order":2,"Speaker":"몬스터","Text":"제게는 한 번도 통과하지 못한 결재가 있습니다. &lt;color=#FFD166&gt;반차 신청.&lt;/color&gt;\n저조차 포기한 부탁을 미용으로 이루어 주실 수 있습니까? 오늘은 제가 직접 손님이 되어 확인하겠습니다. 커피는…… 들고 앉아도 되겠지요?","Notes":"중간 점검: 한 번도 승인되지 않은 반차를 외모 변화로 설득하는 과제. 로컬 검토 초안."},{"DialogueID":900126,"GroupID":80081,"Order":1,"Speaker":"몬스터","Text":"&lt;wave=1.2&gt;호오……&lt;/wave&gt; 뿔은 가볍고, 세 눈과 코는 쉬어야 한다는 말을 분명히 전하는군요.\n부탁을 알아듣고 인상을 바꾸는 솜씨, 잘 보았습니다.","Notes":"중간 점검: 한 번도 승인되지 않은 반차를 외모 변화로 설득하는 과제. 로컬 검토 초안."},{"DialogueID":900127,"GroupID":80081,"Order":2,"Speaker":"몬스터","Text":"이번에는 반차 신청서에 제 얼굴도 첨부해야겠습니다.\n중간 점검에는 좋은 평가를 남기지요. 이 솜씨로 별 세 개까지 올라오십시오.","Notes":"중간 점검: 한 번도 승인되지 않은 반차를 외모 변화로 설득하는 과제. 로컬 검토 초안."},{"DialogueID":900128,"GroupID":80082,"Order":1,"Speaker":"몬스터","Text":"음…… 의도는 전해집니다. 다만 “당장 쉬어라”보다는 “커피 한 잔 더 마셔라”에 가깝군요.","Notes":"중간 점검: 한 번도 승인되지 않은 반차를 외모 변화로 설득하는 과제. 로컬 검토 초안."},{"DialogueID":900129,"GroupID":80082,"Order":2,"Speaker":"몬스터","Text":"점검 기록에는 조금 더 다듬을 여지가 있다고 적겠습니다.\n5일차까지 손님들의 부탁을 듣고, 그 차이를 익혀 보십시오. 제 반차도 아직 포기하지 않겠습니다.","Notes":"중간 점검: 한 번도 승인되지 않은 반차를 외모 변화로 설득하는 과제. 로컬 검토 초안."},{"DialogueID":900130,"GroupID":80083,"Order":1,"Speaker":"몬스터","Text":"&lt;shake=0.8&gt;하아……&lt;/shake&gt; 반차를 설득할 얼굴을 부탁드렸는데, 설명해야 할 부분이 더 늘었군요.","Notes":"중간 점검: 한 번도 승인되지 않은 반차를 외모 변화로 설득하는 과제. 로컬 검토 초안."},{"DialogueID":900131,"GroupID":80083,"Order":2,"Speaker":"몬스터","Text":"중간 점검에는 보완이 필요하다고 남기겠습니다.\n손님이 어떤 모습이 되고 싶은지, 그 말을 놓치지 마십시오. 마왕님을 만날 때도 중요할 겁니다.","Notes":"중간 점검: 한 번도 승인되지 않은 반차를 외모 변화로 설득하는 과제. 로컬 검토 초안."},{"DialogueID":900132,"GroupID":80084,"Order":1,"Speaker":"몬스터","Text":"점검은 여기까지입니다. 보고서와 반차 신청서를 함께 올리러 가겠습니다.\n다음에 마왕님을 모시고 올 때는, &lt;color=#FFD166&gt;별 세 개&lt;/color&gt;가 걸려 있기를 기대하지요.","Notes":"중간 점검: 한 번도 승인되지 않은 반차를 외모 변화로 설득하는 과제. 로컬 검토 초안."},{"DialogueID":900133,"GroupID":80085,"Order":1,"Speaker":"몬스터","Text":"잠깐! 점검하는 눈입니다. 심사위원을 안 보이게 한다고 통과가 되는 건 아닙니다!","Notes":"마왕 부하 · 눈에 닿았을 때 · 첫 항의"},{"DialogueID":900134,"GroupID":80086,"Order":1,"Speaker":"몬스터","Text":"하아…… 눈은 세 개지만, 재시험 기회까지 세 번인 건 아닙니다.","Notes":"마왕 부하 · 다시 눈에 닿았을 때 · 두 번째 항의"},{"DialogueID":900135,"GroupID":80087,"Order":1,"Speaker":"몬스터","Text":"잠깐…… 뿔은 줄여 달라고 말씀드렸습니다. 점검표의 줄 수를 늘릴 생각은 아니시지요?","Notes":"마왕 부하 · 뿔을 줄인 뒤 다시 불어날 때"},{"DialogueID":900136,"GroupID":80088,"Order":1,"Speaker":"몬스터","Text":"왔을 때보다 뿔이 더 많군요. “요구 이상의 성과”라고 적기에는 방향이 반대입니다만.","Notes":"마왕 부하 · 처음보다 뿔이 더 많아졌을 때"}]},{"name":"대화 그룹","keys":["GroupID","Name","PlaybackMode","PauseCombat","AdvanceMode","CPS","HoldMs","GapMs","Notes","ActorEffect","FinishEffect"],"rows":[{"GroupID":80001,"Name":"좀비 등장 대화","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80002,"Name":"취준좀비 · 형태 만들기 · 처음 부탁","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"미용 대사 연결에서 선택하는 부탁","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80003,"Name":"취준좀비 · 형태 만들기 · 자세한 부탁","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"미용 대사 연결에서 선택하는 부탁","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80004,"Name":"미용 요청 · 두 번째 되묻기","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80005,"Name":"미용 대성공 · 결과 반응","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80006,"Name":"미용 보통 성공 · 결과 반응","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80007,"Name":"미용 실패 · 결과 반응","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80008,"Name":"미용 대성공 · 야차 제안","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80009,"Name":"미용 보통 성공 · 야차 제안","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80010,"Name":"미용 실패 · 필수 야차 통보","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80011,"Name":"미용 실패 · 배상 완료","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80012,"Name":"미용 대성공 · 야차 거절","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80013,"Name":"미용 보통 성공 · 야차 거절","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80014,"Name":"미용 대성공 · 야차 수락","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80015,"Name":"미용 보통 성공 · 야차 수락","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80016,"Name":"미용 성공 · 전투 시작","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":30,"HoldMs":1500,"GapMs":400,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80017,"Name":"미용 실패 · 전투 시작","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":30,"HoldMs":1500,"GapMs":400,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80018,"Name":"미용 성공 · 전투 중 공격","PlaybackMode":"무작위 한 줄","PauseCombat":false,"AdvanceMode":"자동","CPS":30,"HoldMs":1500,"GapMs":400,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80019,"Name":"미용 실패 · 전투 중 공격","PlaybackMode":"무작위 한 줄","PauseCombat":false,"AdvanceMode":"자동","CPS":30,"HoldMs":1500,"GapMs":400,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80020,"Name":"미용 성공 · 좀비 HP 낮음","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":30,"HoldMs":1500,"GapMs":400,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80021,"Name":"미용 실패 · 좀비 HP 낮음","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":30,"HoldMs":1500,"GapMs":400,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80022,"Name":"미용 성공 · 플레이어 HP 낮음","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":30,"HoldMs":1500,"GapMs":400,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80023,"Name":"미용 실패 · 플레이어 HP 낮음","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":30,"HoldMs":1500,"GapMs":400,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80024,"Name":"미용 실패 · 플레이어 야차 승리","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":30,"HoldMs":1500,"GapMs":400,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80025,"Name":"미용 실패 · 플레이어 야차 패배","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":30,"HoldMs":1500,"GapMs":400,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80026,"Name":"미용 성공 · 플레이어 연습 야차 승리","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":30,"HoldMs":1500,"GapMs":400,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80027,"Name":"미용 성공 · 플레이어 연습 야차 패배","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":30,"HoldMs":1500,"GapMs":400,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80028,"Name":"미용 대성공 · 플레이어 승리 후 퇴장","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80029,"Name":"미용 대성공 · 플레이어 패배 후 퇴장","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80030,"Name":"미용 보통 성공 · 플레이어 승리 후 퇴장","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80031,"Name":"미용 보통 성공 · 플레이어 패배 후 퇴장","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80032,"Name":"미용 실패 · 플레이어 승리 후 퇴장","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80033,"Name":"미용 실패 · 플레이어 패배 후 퇴장","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80034,"Name":"몬스타그램 · 미용 성공 (야차 무관)","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":0,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80035,"Name":"몬스타그램 · 미용 실패 (조건 확인 필요)","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":0,"HoldMs":1500,"GapMs":0,"Notes":"원본의 대사 연결 순서를 순번으로 옮김. 본문은 그대로 유지.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80036,"Name":"취객 · 제이로 착각","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":29,"HoldMs":1200,"GapMs":250,"Notes":"취객·샌즈 전투 연출 초안. 태그와 시간은 자유롭게 조정 가능.","ActorEffect":"비틀거림","FinishEffect":"없음"},{"GroupID":80037,"Name":"샌즈 · 가볍게 인사","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"자동","CPS":23,"HoldMs":900,"GapMs":250,"Notes":"취객·샌즈 전투 연출 초안. 태그와 시간은 자유롭게 조정 가능.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80038,"Name":"취객 · 1단계 아직 두 명으로 보여","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"자동","CPS":27,"HoldMs":1300,"GapMs":250,"Notes":"취객·샌즈 전투 연출 초안. 태그와 시간은 자유롭게 조정 가능.","ActorEffect":"비틀거림","FinishEffect":"없음"},{"GroupID":80039,"Name":"취객 · 2단계 시야가 돌아와","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"자동","CPS":27,"HoldMs":1300,"GapMs":250,"Notes":"취객·샌즈 전투 연출 초안. 태그와 시간은 자유롭게 조정 가능.","ActorEffect":"놀람","FinishEffect":"없음"},{"GroupID":80040,"Name":"취객 · 3단계 제이와 가업","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"자동","CPS":27,"HoldMs":1300,"GapMs":250,"Notes":"취객·샌즈 전투 연출 초안. 태그와 시간은 자유롭게 조정 가능.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80041,"Name":"취객 · 4단계 돌아온 손끝","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"자동","CPS":27,"HoldMs":1300,"GapMs":250,"Notes":"취객·샌즈 전투 연출 초안. 태그와 시간은 자유롭게 조정 가능.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80042,"Name":"취객 · 미용실에서 이어질 이야기","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"자동","CPS":27,"HoldMs":1500,"GapMs":250,"Notes":"전투에서는 해금·지급 연출 없이 귀환을 예고합니다. 소울 해금과 튜토리얼은 이후 미용실 대화에서 진행.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80043,"Name":"샌즈 · 첫 MISS 여유","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":23,"HoldMs":1500,"GapMs":250,"Notes":"첫 MISS와 함께 재생. 말하는 중에도 빈틈 게이지와 연타 진행.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80044,"Name":"샌즈 · 첫 명중 허세","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"자동","CPS":23,"HoldMs":1500,"GapMs":250,"Notes":"취객·샌즈 전투 연출 초안. 태그와 시간은 자유롭게 조정 가능.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80045,"Name":"샌즈 · 두 번째 MISS 농담","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":23,"HoldMs":1500,"GapMs":250,"Notes":"첫 MISS와 함께 재생. 말하는 중에도 빈틈 게이지와 연타 진행.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80046,"Name":"샌즈 · 두 번째 명중 동요","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"자동","CPS":23,"HoldMs":1500,"GapMs":250,"Notes":"취객·샌즈 전투 연출 초안. 태그와 시간은 자유롭게 조정 가능.","ActorEffect":"식은땀","FinishEffect":"없음"},{"GroupID":80047,"Name":"샌즈 · 마지막 빈틈 경계","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":30,"HoldMs":900,"GapMs":250,"Notes":"세 번째 페이즈 빈틈 시작, 공격과 함께 말한다.","ActorEffect":"식은땀","FinishEffect":"없음"},{"GroupID":80048,"Name":"샌즈 · 마지막 말","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"자동","CPS":23,"HoldMs":1500,"GapMs":250,"Notes":"취객·샌즈 전투 연출 초안. 태그와 시간은 자유롭게 조정 가능.","ActorEffect":"식은땀","FinishEffect":"소멸"},{"GroupID":80049,"Name":"좀비 · 끈질긴 공격","PlaybackMode":"무작위 한 줄","PauseCombat":false,"AdvanceMode":"자동","CPS":26,"HoldMs":1400,"GapMs":250,"Notes":"좀비 전투 전용. 기존 문자 효과 태그로 연출.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80050,"Name":"좀비 · 빈틈 농담","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":26,"HoldMs":1400,"GapMs":250,"Notes":"좀비 전투 전용. 기존 문자 효과 태그로 연출.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80051,"Name":"좀비 · 부활 완료 후 한마디","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":26,"HoldMs":1400,"GapMs":250,"Notes":"실제 부활 모션 완료 → 글자 시작 → 다음 대사 입력 후 전투 재개.","ActorEffect":"부활 후 대사","FinishEffect":"없음"},{"GroupID":80052,"Name":"좀비 · 재도전 휴업","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":26,"HoldMs":1400,"GapMs":250,"Notes":"좀비 전투 전용. 기존 문자 효과 태그로 연출.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80053,"Name":"좀비 · 끝까지 버티기","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":26,"HoldMs":1400,"GapMs":250,"Notes":"좀비 전투 전용. 기존 문자 효과 태그로 연출.","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80054,"Name":"취준좀비 · 장식 붙이기 · 처음 부탁","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"미용 대사 연결에서 선택하는 부탁","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80055,"Name":"취준좀비 · 색·무늬 꾸미기 · 처음 부탁","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"미용 대사 연결에서 선택하는 부탁","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80056,"Name":"좀비 · 미용실 복귀","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"통합 프로토타입 미용실 대사","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80057,"Name":"좀비 · 연습 종료","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"통합 프로토타입 미용실 대사","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80058,"Name":"취객 · 불 켜진 미용실","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"통합 프로토타입 미용실 대사","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80059,"Name":"취객 · 돌아온 가업","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"통합 프로토타입 미용실 대사","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80060,"Name":"취객 · 잠깐의 외출","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"통합 프로토타입 미용실 대사","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80061,"Name":"샌즈 · 방문","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"통합 프로토타입 미용실 대사","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80062,"Name":"샌즈 · 형태 만들기 · 처음 부탁","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"미용 대사 연결에서 선택하는 부탁","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80063,"Name":"샌즈 · 장식 붙이기 · 처음 부탁","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"미용 대사 연결에서 선택하는 부탁","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80064,"Name":"샌즈 · 미용 만족","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"통합 프로토타입 미용실 대사","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80065,"Name":"샌즈 · 미용 보통","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"통합 프로토타입 미용실 대사","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80066,"Name":"샌즈 · 미용 실패","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"통합 프로토타입 미용실 대사","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80068,"Name":"취준좀비 · 색·무늬 꾸미기 · 자세한 부탁","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"미용 대사 연결에서 선택하는 부탁","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80069,"Name":"취준좀비 · 장식 붙이기 · 자세한 부탁","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"미용 대사 연결에서 선택하는 부탁","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80070,"Name":"샌즈 · 형태 만들기 · 자세한 부탁","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"미용 대사 연결에서 선택하는 부탁","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80071,"Name":"샌즈 · 색·무늬 꾸미기 · 처음 부탁","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"미용 대사 연결에서 선택하는 부탁","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80072,"Name":"샌즈 · 색·무늬 꾸미기 · 자세한 부탁","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"미용 대사 연결에서 선택하는 부탁","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80073,"Name":"샌즈 · 장식 붙이기 · 자세한 부탁","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"미용 대사 연결에서 선택하는 부탁","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80089,"Name":"샌즈 · 야차 승리 후 미용실","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"통합 개발실","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80074,"Name":"마왕 부하 · 형태 다듬기 · 처음 부탁","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"미용 시험용 대사 초안","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80075,"Name":"마왕 부하 · 형태 다듬기 · 자세한 부탁","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"미용 시험용 대사 초안","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80076,"Name":"마왕 부하 · 색·무늬 · 처음 부탁","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"미용 시험용 대사 초안","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80077,"Name":"마왕 부하 · 색·무늬 · 자세한 부탁","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"미용 시험용 대사 초안","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80078,"Name":"마왕 부하 · 장식 · 처음 부탁","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"미용 시험용 대사 초안","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80079,"Name":"마왕 부하 · 장식 · 자세한 부탁","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"미용 시험용 대사 초안","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80080,"Name":"마왕 부하 · 손님 등장","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"로컬 본편 시연용 임시 대사","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80081,"Name":"마왕 부하 · 미용 만족","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"로컬 본편 시연용 임시 대사","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80082,"Name":"마왕 부하 · 미용 보통","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"로컬 본편 시연용 임시 대사","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80083,"Name":"마왕 부하 · 미용 불만족","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"로컬 본편 시연용 임시 대사","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80084,"Name":"마왕 부하 · 손님 퇴장","PlaybackMode":"순서대로","PauseCombat":true,"AdvanceMode":"입력","CPS":30,"HoldMs":1400,"GapMs":100,"Notes":"로컬 본편 시연용 임시 대사","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80085,"Name":"마왕 부하 · 눈에 닿았을 때 · 첫 항의","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":30,"HoldMs":5500,"GapMs":100,"Notes":"미용 중 반응 · 조건과 재생 시점은 미용 설정","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80086,"Name":"마왕 부하 · 다시 눈에 닿았을 때 · 두 번째 항의","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":30,"HoldMs":5500,"GapMs":100,"Notes":"미용 중 반응 · 조건과 재생 시점은 미용 설정","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80087,"Name":"마왕 부하 · 뿔을 줄인 뒤 다시 불어날 때","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":30,"HoldMs":5500,"GapMs":100,"Notes":"미용 중 반응 · 조건과 재생 시점은 미용 설정","ActorEffect":"없음","FinishEffect":"없음"},{"GroupID":80088,"Name":"마왕 부하 · 처음보다 뿔이 더 많아졌을 때","PlaybackMode":"순서대로","PauseCombat":false,"AdvanceMode":"자동","CPS":30,"HoldMs":5500,"GapMs":100,"Notes":"미용 중 반응 · 조건과 재생 시점은 미용 설정","ActorEffect":"없음","FinishEffect":"없음"}]},{"name":"전투 대사 연결","keys":["TriggerID","MonsterID","PhaseID","EventType","PatternID","BeautyCondition","GroupID","HPThresholdPct","CooldownMs","MaxPerBattle","Enabled","Notes","EventCount"],"rows":[{"TriggerID":100001,"MonsterID":10001,"PhaseID":null,"EventType":"전투 시작","PatternID":null,"BeautyCondition":"미용 성공","GroupID":80016,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":false,"Notes":"기존 미용 분기 대사 보관. 현재는 전투 전용 공통 연결을 사용하며 등장·미용 흐름은 보류.","EventCount":null},{"TriggerID":100002,"MonsterID":10001,"PhaseID":null,"EventType":"공격 시작","PatternID":null,"BeautyCondition":"미용 성공","GroupID":80018,"HPThresholdPct":null,"CooldownMs":8000,"MaxPerBattle":0,"Enabled":false,"Notes":"기존 미용 분기 대사 보관. 현재는 전투 전용 공통 연결을 사용하며 등장·미용 흐름은 보류.","EventCount":null},{"TriggerID":100003,"MonsterID":10001,"PhaseID":null,"EventType":"몬스터 HP 이하","PatternID":null,"BeautyCondition":"미용 성공","GroupID":80020,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":false,"Notes":"기존 미용 분기 대사 보관. 현재는 전투 전용 공통 연결을 사용하며 등장·미용 흐름은 보류.","EventCount":null},{"TriggerID":100004,"MonsterID":10001,"PhaseID":null,"EventType":"플레이어 HP 이하","PatternID":null,"BeautyCondition":"미용 성공","GroupID":80022,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":false,"Notes":"기존 미용 분기 대사 보관. 현재는 전투 전용 공통 연결을 사용하며 등장·미용 흐름은 보류.","EventCount":null},{"TriggerID":100005,"MonsterID":10001,"PhaseID":null,"EventType":"승리","PatternID":null,"BeautyCondition":"미용 성공","GroupID":80026,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":false,"Notes":"기존 미용 분기 대사 보관. 현재는 전투 전용 공통 연결을 사용하며 등장·미용 흐름은 보류.","EventCount":null},{"TriggerID":100006,"MonsterID":10001,"PhaseID":null,"EventType":"패배","PatternID":null,"BeautyCondition":"미용 성공","GroupID":80027,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":false,"Notes":"기존 미용 분기 대사 보관. 현재는 전투 전용 공통 연결을 사용하며 등장·미용 흐름은 보류.","EventCount":null},{"TriggerID":100007,"MonsterID":10001,"PhaseID":null,"EventType":"전투 시작","PatternID":null,"BeautyCondition":"미용 실패","GroupID":80017,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":false,"Notes":"기존 미용 분기 대사 보관. 현재는 전투 전용 공통 연결을 사용하며 등장·미용 흐름은 보류.","EventCount":null},{"TriggerID":100008,"MonsterID":10001,"PhaseID":null,"EventType":"공격 시작","PatternID":null,"BeautyCondition":"미용 실패","GroupID":80019,"HPThresholdPct":null,"CooldownMs":8000,"MaxPerBattle":0,"Enabled":false,"Notes":"기존 미용 분기 대사 보관. 현재는 전투 전용 공통 연결을 사용하며 등장·미용 흐름은 보류.","EventCount":null},{"TriggerID":100009,"MonsterID":10001,"PhaseID":null,"EventType":"몬스터 HP 이하","PatternID":null,"BeautyCondition":"미용 실패","GroupID":80021,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":false,"Notes":"기존 미용 분기 대사 보관. 현재는 전투 전용 공통 연결을 사용하며 등장·미용 흐름은 보류.","EventCount":null},{"TriggerID":100010,"MonsterID":10001,"PhaseID":null,"EventType":"플레이어 HP 이하","PatternID":null,"BeautyCondition":"미용 실패","GroupID":80023,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":false,"Notes":"기존 미용 분기 대사 보관. 현재는 전투 전용 공통 연결을 사용하며 등장·미용 흐름은 보류.","EventCount":null},{"TriggerID":100011,"MonsterID":10001,"PhaseID":null,"EventType":"승리","PatternID":null,"BeautyCondition":"미용 실패","GroupID":80024,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":false,"Notes":"기존 미용 분기 대사 보관. 현재는 전투 전용 공통 연결을 사용하며 등장·미용 흐름은 보류.","EventCount":null},{"TriggerID":100012,"MonsterID":10001,"PhaseID":null,"EventType":"패배","PatternID":null,"BeautyCondition":"미용 실패","GroupID":80025,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":false,"Notes":"기존 미용 분기 대사 보관. 현재는 전투 전용 공통 연결을 사용하며 등장·미용 흐름은 보류.","EventCount":null},{"TriggerID":100013,"MonsterID":10002,"PhaseID":1,"EventType":"전투 시작","PatternID":null,"BeautyCondition":"공통","GroupID":80036,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":true,"Notes":"사건 발생 시 한 번 재생.","EventCount":null},{"TriggerID":100014,"MonsterID":10003,"PhaseID":1,"EventType":"전투 시작","PatternID":null,"BeautyCondition":"공통","GroupID":80037,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":true,"Notes":"사건 발생 시 한 번 재생.","EventCount":null},{"TriggerID":100015,"MonsterID":10002,"PhaseID":1,"EventType":"빈틈공격 성공","PatternID":null,"BeautyCondition":"공통","GroupID":80038,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":true,"Notes":"해당 페이즈에서 명중한 빈틈이 끝난 뒤 한 번. 대사 후 다음 페이즈 또는 승리.","EventCount":null},{"TriggerID":100016,"MonsterID":10002,"PhaseID":2,"EventType":"빈틈공격 성공","PatternID":null,"BeautyCondition":"공통","GroupID":80039,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":true,"Notes":"해당 페이즈에서 명중한 빈틈이 끝난 뒤 한 번. 대사 후 다음 페이즈 또는 승리.","EventCount":null},{"TriggerID":100017,"MonsterID":10002,"PhaseID":3,"EventType":"빈틈공격 성공","PatternID":null,"BeautyCondition":"공통","GroupID":80040,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":true,"Notes":"해당 페이즈에서 명중한 빈틈이 끝난 뒤 한 번. 대사 후 다음 페이즈 또는 승리.","EventCount":null},{"TriggerID":100018,"MonsterID":10002,"PhaseID":4,"EventType":"빈틈공격 성공","PatternID":null,"BeautyCondition":"공통","GroupID":80041,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":true,"Notes":"해당 페이즈에서 명중한 빈틈이 끝난 뒤 한 번. 대사 후 다음 페이즈 또는 승리.","EventCount":null},{"TriggerID":100019,"MonsterID":10002,"PhaseID":4,"EventType":"승리","PatternID":null,"BeautyCondition":"공통","GroupID":80042,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":true,"Notes":"사건 발생 시 한 번 재생.","EventCount":null},{"TriggerID":100020,"MonsterID":10003,"PhaseID":1,"EventType":"빈틈공격 MISS","PatternID":null,"BeautyCondition":"공통","GroupID":80043,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":true,"Notes":"첫 MISS 순간 대사 시작. 같은 빈틈의 후속 MISS에는 재시작하지 않음. 전투 정지 없음.","EventCount":1},{"TriggerID":100021,"MonsterID":10003,"PhaseID":1,"EventType":"빈틈공격 성공","PatternID":null,"BeautyCondition":"공통","GroupID":80044,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":true,"Notes":"1번째 명중한 빈틈 종료 후 한 번 재생. 연타 개수는 세지 않음.","EventCount":1},{"TriggerID":100022,"MonsterID":10003,"PhaseID":2,"EventType":"빈틈공격 MISS","PatternID":null,"BeautyCondition":"공통","GroupID":80045,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":true,"Notes":"첫 MISS 순간 대사 시작. 같은 빈틈의 후속 MISS에는 재시작하지 않음. 전투 정지 없음.","EventCount":1},{"TriggerID":100023,"MonsterID":10003,"PhaseID":2,"EventType":"빈틈공격 성공","PatternID":null,"BeautyCondition":"공통","GroupID":80046,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":true,"Notes":"1번째 명중한 빈틈 종료 후 한 번 재생. 연타 개수는 세지 않음.","EventCount":1},{"TriggerID":100024,"MonsterID":10003,"PhaseID":3,"EventType":"빈틈공격 MISS","PatternID":null,"BeautyCondition":"공통","GroupID":80047,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":true,"Notes":"첫 MISS 순간 대사 시작. 같은 빈틈의 후속 MISS에는 재시작하지 않음. 전투 정지 없음.","EventCount":1},{"TriggerID":100025,"MonsterID":10003,"PhaseID":3,"EventType":"빈틈공격 성공","PatternID":null,"BeautyCondition":"공통","GroupID":80048,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":true,"Notes":"1번째 명중한 빈틈 종료 후 한 번 재생. 연타 개수는 세지 않음.","EventCount":1},{"TriggerID":100026,"MonsterID":10001,"PhaseID":null,"EventType":"공격 시작","PatternID":null,"BeautyCondition":"공통","GroupID":80049,"HPThresholdPct":null,"CooldownMs":9000,"MaxPerBattle":0,"Enabled":true,"Notes":"등장·미용과 분리한 전투 대사.","EventCount":null},{"TriggerID":100027,"MonsterID":10001,"PhaseID":null,"EventType":"빈틈 발생","PatternID":null,"BeautyCondition":"공통","GroupID":80050,"HPThresholdPct":null,"CooldownMs":12000,"MaxPerBattle":2,"Enabled":true,"Notes":"등장·미용과 분리한 전투 대사.","EventCount":null},{"TriggerID":100028,"MonsterID":10001,"PhaseID":null,"EventType":"승리","PatternID":null,"BeautyCondition":"공통","GroupID":80052,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":true,"Notes":"등장·미용과 분리한 전투 대사.","EventCount":null},{"TriggerID":100029,"MonsterID":10001,"PhaseID":null,"EventType":"패배","PatternID":null,"BeautyCondition":"공통","GroupID":80053,"HPThresholdPct":null,"CooldownMs":0,"MaxPerBattle":1,"Enabled":true,"Notes":"등장·미용과 분리한 전투 대사.","EventCount":null}]},{"name":"문자 효과 규칙","keys":["Tag","Example","Description"],"rows":[{"Tag":"color","Example":"&lt;color=#FFD166&gt;으하하하!&lt;/color&gt;","Description":"글자색을 바꿉니다. #RRGGBB 또는 white/red 등 기본 색 이름을 씁니다."},{"Tag":"shake","Example":"&lt;shake=2 speed=16 dur=0.5&gt;어이쿠!&lt;/shake&gt;","Description":"글자를 떨리게 합니다. 2는 흔들림 크기, speed는 속도, dur는 지속 초입니다. dur 생략/0이면 대사 동안 계속합니다."},{"Tag":"wave","Example":"&lt;wave=3 speed=5&gt;오랜만이구먼!&lt;/wave&gt;","Description":"글자가 물결처럼 위아래로 움직입니다. 3은 높이, speed는 움직이는 속도입니다."},{"Tag":"wait","Example":"잠깐,&lt;wait=0.4&gt; 우리... 친구잖아?","Description":"이 위치에서 타이핑을 0.4초 쉽니다. 전투 시간을 멈출지는 대화 그룹에서 정합니다."},{"Tag":"cps","Example":"&lt;cps=16&gt;눈치 빠른 애송이들이...&lt;/cps&gt;","Description":"이 구간만 초당 글자 수를 바꿉니다. 0은 즉시 표시입니다."},{"Tag":"speed","Example":"&lt;speed=0.7&gt;천천히&lt;/speed&gt;","Description":"기본 타이핑 속도에 곱합니다. 0.7은 더 느리고 2는 두 배입니다."},{"Tag":"size","Example":"&lt;size=24&gt;으하하하!&lt;/size&gt;","Description":"이 구간의 글자 크기입니다. 화면 픽셀 기준이며 기본 크기는 17입니다."},{"Tag":"pulse","Example":"&lt;pulse=1.1 speed=7&gt;으하하하!&lt;/pulse&gt;","Description":"글자가 1.1배까지 가볍게 커졌다 작아집니다."},{"Tag":"fade","Example":"&lt;fade=0.3&gt;서서히&lt;/fade&gt;","Description":"각 글자가 나타난 뒤 0.3초 동안 천천히 선명해집니다."},{"Tag":"rainbow","Example":"&lt;rainbow=0.6 speed=3&gt;반짝이는 색&lt;/rainbow&gt;","Description":"시간에 따라 글자색을 무지개색으로 바꿉니다. 값은 색의 강도 0~1입니다."},{"Tag":"중첩","Example":"&lt;color=#8BE9FD&gt;&lt;shake=2&gt;친구잖아..?&lt;/shake&gt;&lt;/color&gt;","Description":"효과는 겹쳐 쓸 수 있습니다. 연 태그는 반대 순서로 닫습니다."},{"Tag":"캐릭터 연출","Example":"대화 그룹 → ActorEffect / FinishEffect","Description":"ActorEffect: 비틀거림·놀람·식은땀·부활 후 대사. 부활 후 대사는 모션이 끝나야 글자가 시작됩니다. FinishEffect: 대사 이후 소멸 등 마무리 연출."},{"Tag":"말투 참고","Example":"https://undertale.com/alarmclock/sans/","Description":"샌즈 말투는 공식 대사에서 짧은 말끝·뜸 들임·건조한 농담을 참고. 전투 대사는 사용자 제시 문장과 새 창작 문장으로 구성."}]},{"name":"미용 대사 연결","keys":["MonsterID","Stage","RequestGroupID","DetailGroupID"],"rows":[{"MonsterID":10001,"Stage":"cut","RequestGroupID":80002,"DetailGroupID":80003},{"MonsterID":10001,"Stage":"draw","RequestGroupID":80055,"DetailGroupID":80068},{"MonsterID":10001,"Stage":"attach","RequestGroupID":80054,"DetailGroupID":80069},{"MonsterID":10003,"Stage":"cut","RequestGroupID":80062,"DetailGroupID":80070},{"MonsterID":10003,"Stage":"draw","RequestGroupID":80071,"DetailGroupID":80072},{"MonsterID":10003,"Stage":"attach","RequestGroupID":80063,"DetailGroupID":80073},{"MonsterID":10004,"Stage":"cut","RequestGroupID":80074,"DetailGroupID":80075},{"MonsterID":10004,"Stage":"draw","RequestGroupID":80076,"DetailGroupID":80077},{"MonsterID":10004,"Stage":"attach","RequestGroupID":80078,"DetailGroupID":80079}]}]},"drafts":[{"MonsterID":10100,"PhaseID":1},{"MonsterID":10100,"PhaseID":2},{"MonsterID":10100,"PhaseID":3}]}</version>
 </file>
</xml_diff>